<commit_message>
📊 Update Excel with new control columns
</commit_message>
<xml_diff>
--- a/data/reporte.xlsx
+++ b/data/reporte.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre\OneDrive\Escritorio\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre\OneDrive\Escritorio\Universidad\2026-1\Modelos de Procesos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2034F3A6-4B31-4781-9779-4D865782C97C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEB94EDD-3F34-45D3-A944-D6BB47B04270}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{EF01AC27-D1AA-450D-80FE-C50ADE1636E7}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EF01AC27-D1AA-450D-80FE-C50ADE1636E7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sección 1" sheetId="1" r:id="rId1"/>
@@ -1365,6 +1365,22 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1376,22 +1392,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1744,6 +1744,9 @@
   <we:bindings/>
   <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
   <we:extLst>
+    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{D87F86FE-615C-45B5-9D79-34F1136793EB}">
+      <we:containsCustomFunctions/>
+    </a:ext>
     <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{7C84B067-C214-45C3-A712-C9D94CD141B2}">
       <we:customFunctionIdList>
         <we:customFunctionIds>_xldudf_GPT</we:customFunctionIds>
@@ -1774,35 +1777,35 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FAFB6214-215B-45FB-8876-0D7E2F238F6A}">
   <dimension ref="A1:T58"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A1" s="23"/>
-      <c r="B1" s="23"/>
+    <row r="1" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A1" s="33"/>
+      <c r="B1" s="33"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
-      <c r="F1" s="24" t="s">
-        <v>0</v>
-      </c>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
-      <c r="I1" s="25"/>
-      <c r="J1" s="25"/>
-      <c r="K1" s="25"/>
-      <c r="L1" s="25"/>
-      <c r="M1" s="25"/>
-      <c r="N1" s="25"/>
-      <c r="O1" s="25"/>
-      <c r="P1" s="25"/>
-      <c r="Q1" s="25"/>
-      <c r="R1" s="25"/>
-      <c r="S1" s="26"/>
+      <c r="F1" s="34" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1" s="35"/>
+      <c r="H1" s="35"/>
+      <c r="I1" s="35"/>
+      <c r="J1" s="35"/>
+      <c r="K1" s="35"/>
+      <c r="L1" s="35"/>
+      <c r="M1" s="35"/>
+      <c r="N1" s="35"/>
+      <c r="O1" s="35"/>
+      <c r="P1" s="35"/>
+      <c r="Q1" s="35"/>
+      <c r="R1" s="35"/>
+      <c r="S1" s="36"/>
       <c r="T1" s="2"/>
     </row>
-    <row r="2" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="27"/>
-      <c r="B2" s="27"/>
+    <row r="2" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="37"/>
+      <c r="B2" s="37"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -1852,7 +1855,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A3" s="6">
         <v>1</v>
       </c>
@@ -1892,9 +1895,15 @@
       <c r="M3" s="9">
         <v>1</v>
       </c>
-      <c r="N3" s="9"/>
-      <c r="O3" s="9"/>
-      <c r="P3" s="9"/>
+      <c r="N3" s="9">
+        <v>3</v>
+      </c>
+      <c r="O3" s="9">
+        <v>4</v>
+      </c>
+      <c r="P3" s="9">
+        <v>3</v>
+      </c>
       <c r="Q3" s="9"/>
       <c r="R3" s="9"/>
       <c r="S3" s="9"/>
@@ -1902,7 +1911,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A4" s="11">
         <v>2</v>
       </c>
@@ -1942,9 +1951,15 @@
       <c r="M4" s="1">
         <v>3</v>
       </c>
-      <c r="N4" s="1"/>
-      <c r="O4" s="1"/>
-      <c r="P4" s="1"/>
+      <c r="N4" s="1">
+        <v>0</v>
+      </c>
+      <c r="O4" s="1">
+        <v>0</v>
+      </c>
+      <c r="P4" s="1">
+        <v>1</v>
+      </c>
       <c r="Q4" s="1"/>
       <c r="R4" s="1"/>
       <c r="S4" s="1"/>
@@ -1952,7 +1967,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A5" s="11">
         <v>3</v>
       </c>
@@ -1992,9 +2007,15 @@
       <c r="M5" s="1">
         <v>0</v>
       </c>
-      <c r="N5" s="1"/>
-      <c r="O5" s="1"/>
-      <c r="P5" s="1"/>
+      <c r="N5" s="1">
+        <v>1</v>
+      </c>
+      <c r="O5" s="1">
+        <v>0</v>
+      </c>
+      <c r="P5" s="1">
+        <v>1</v>
+      </c>
       <c r="Q5" s="1"/>
       <c r="R5" s="1"/>
       <c r="S5" s="1"/>
@@ -2002,7 +2023,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A6" s="11">
         <v>4</v>
       </c>
@@ -2042,9 +2063,15 @@
       <c r="M6" s="1">
         <v>4</v>
       </c>
-      <c r="N6" s="1"/>
-      <c r="O6" s="1"/>
-      <c r="P6" s="1"/>
+      <c r="N6" s="1">
+        <v>1</v>
+      </c>
+      <c r="O6" s="1">
+        <v>3</v>
+      </c>
+      <c r="P6" s="1">
+        <v>1</v>
+      </c>
       <c r="Q6" s="1"/>
       <c r="R6" s="1"/>
       <c r="S6" s="1"/>
@@ -2052,7 +2079,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A7" s="11">
         <v>5</v>
       </c>
@@ -2092,9 +2119,15 @@
       <c r="M7" s="1">
         <v>1</v>
       </c>
-      <c r="N7" s="1"/>
-      <c r="O7" s="1"/>
-      <c r="P7" s="1"/>
+      <c r="N7" s="1">
+        <v>2</v>
+      </c>
+      <c r="O7" s="1">
+        <v>3</v>
+      </c>
+      <c r="P7" s="1">
+        <v>2</v>
+      </c>
       <c r="Q7" s="1"/>
       <c r="R7" s="1"/>
       <c r="S7" s="1"/>
@@ -2102,7 +2135,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A8" s="11">
         <v>6</v>
       </c>
@@ -2142,9 +2175,15 @@
       <c r="M8" s="1">
         <v>4</v>
       </c>
-      <c r="N8" s="1"/>
-      <c r="O8" s="1"/>
-      <c r="P8" s="1"/>
+      <c r="N8" s="1">
+        <v>5</v>
+      </c>
+      <c r="O8" s="1">
+        <v>5</v>
+      </c>
+      <c r="P8" s="1">
+        <v>4</v>
+      </c>
       <c r="Q8" s="1"/>
       <c r="R8" s="1"/>
       <c r="S8" s="1"/>
@@ -2152,7 +2191,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A9" s="11">
         <v>7</v>
       </c>
@@ -2192,9 +2231,15 @@
       <c r="M9" s="1">
         <v>2</v>
       </c>
-      <c r="N9" s="1"/>
-      <c r="O9" s="1"/>
-      <c r="P9" s="1"/>
+      <c r="N9" s="1">
+        <v>0</v>
+      </c>
+      <c r="O9" s="1">
+        <v>4</v>
+      </c>
+      <c r="P9" s="1">
+        <v>2</v>
+      </c>
       <c r="Q9" s="1"/>
       <c r="R9" s="1"/>
       <c r="S9" s="1"/>
@@ -2202,7 +2247,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A10" s="11">
         <v>8</v>
       </c>
@@ -2242,9 +2287,15 @@
       <c r="M10" s="1">
         <v>0</v>
       </c>
-      <c r="N10" s="1"/>
-      <c r="O10" s="1"/>
-      <c r="P10" s="1"/>
+      <c r="N10" s="1">
+        <v>2</v>
+      </c>
+      <c r="O10" s="1">
+        <v>0</v>
+      </c>
+      <c r="P10" s="1">
+        <v>2</v>
+      </c>
       <c r="Q10" s="1"/>
       <c r="R10" s="1"/>
       <c r="S10" s="1"/>
@@ -2252,7 +2303,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A11" s="11">
         <v>9</v>
       </c>
@@ -2292,9 +2343,15 @@
       <c r="M11" s="1">
         <v>5</v>
       </c>
-      <c r="N11" s="1"/>
-      <c r="O11" s="1"/>
-      <c r="P11" s="1"/>
+      <c r="N11" s="1">
+        <v>3</v>
+      </c>
+      <c r="O11" s="1">
+        <v>5</v>
+      </c>
+      <c r="P11" s="1">
+        <v>3</v>
+      </c>
       <c r="Q11" s="1"/>
       <c r="R11" s="1"/>
       <c r="S11" s="1"/>
@@ -2302,7 +2359,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A12" s="11">
         <v>10</v>
       </c>
@@ -2342,9 +2399,15 @@
       <c r="M12" s="1">
         <v>3</v>
       </c>
-      <c r="N12" s="1"/>
-      <c r="O12" s="1"/>
-      <c r="P12" s="1"/>
+      <c r="N12" s="1">
+        <v>2</v>
+      </c>
+      <c r="O12" s="1">
+        <v>5</v>
+      </c>
+      <c r="P12" s="1">
+        <v>3</v>
+      </c>
       <c r="Q12" s="1"/>
       <c r="R12" s="1"/>
       <c r="S12" s="1"/>
@@ -2352,7 +2415,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A13" s="11">
         <v>11</v>
       </c>
@@ -2392,9 +2455,15 @@
       <c r="M13" s="1">
         <v>0</v>
       </c>
-      <c r="N13" s="1"/>
-      <c r="O13" s="1"/>
-      <c r="P13" s="1"/>
+      <c r="N13" s="1">
+        <v>0</v>
+      </c>
+      <c r="O13" s="1">
+        <v>3</v>
+      </c>
+      <c r="P13" s="1">
+        <v>3</v>
+      </c>
       <c r="Q13" s="1"/>
       <c r="R13" s="1"/>
       <c r="S13" s="1"/>
@@ -2402,7 +2471,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A14" s="11">
         <v>12</v>
       </c>
@@ -2442,9 +2511,15 @@
       <c r="M14" s="1">
         <v>1</v>
       </c>
-      <c r="N14" s="1"/>
-      <c r="O14" s="1"/>
-      <c r="P14" s="1"/>
+      <c r="N14" s="1">
+        <v>2</v>
+      </c>
+      <c r="O14" s="1">
+        <v>0</v>
+      </c>
+      <c r="P14" s="1">
+        <v>3</v>
+      </c>
       <c r="Q14" s="1"/>
       <c r="R14" s="1"/>
       <c r="S14" s="1"/>
@@ -2452,7 +2527,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A15" s="11">
         <v>13</v>
       </c>
@@ -2492,9 +2567,15 @@
       <c r="M15" s="1">
         <v>4</v>
       </c>
-      <c r="N15" s="1"/>
-      <c r="O15" s="1"/>
-      <c r="P15" s="1"/>
+      <c r="N15" s="1">
+        <v>2</v>
+      </c>
+      <c r="O15" s="1">
+        <v>4</v>
+      </c>
+      <c r="P15" s="1">
+        <v>0</v>
+      </c>
       <c r="Q15" s="1"/>
       <c r="R15" s="1"/>
       <c r="S15" s="1"/>
@@ -2502,7 +2583,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A16" s="11">
         <v>14</v>
       </c>
@@ -2542,9 +2623,15 @@
       <c r="M16" s="1">
         <v>2</v>
       </c>
-      <c r="N16" s="1"/>
-      <c r="O16" s="1"/>
-      <c r="P16" s="1"/>
+      <c r="N16" s="1">
+        <v>4</v>
+      </c>
+      <c r="O16" s="1">
+        <v>0</v>
+      </c>
+      <c r="P16" s="1">
+        <v>2</v>
+      </c>
       <c r="Q16" s="1"/>
       <c r="R16" s="1"/>
       <c r="S16" s="1"/>
@@ -2552,7 +2639,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A17" s="11">
         <v>15</v>
       </c>
@@ -2592,9 +2679,15 @@
       <c r="M17" s="1">
         <v>0</v>
       </c>
-      <c r="N17" s="1"/>
-      <c r="O17" s="1"/>
-      <c r="P17" s="1"/>
+      <c r="N17" s="1">
+        <v>1</v>
+      </c>
+      <c r="O17" s="1">
+        <v>3</v>
+      </c>
+      <c r="P17" s="1">
+        <v>1</v>
+      </c>
       <c r="Q17" s="1"/>
       <c r="R17" s="1"/>
       <c r="S17" s="1"/>
@@ -2602,7 +2695,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A18" s="11">
         <v>16</v>
       </c>
@@ -2642,9 +2735,15 @@
       <c r="M18" s="1">
         <v>2</v>
       </c>
-      <c r="N18" s="1"/>
-      <c r="O18" s="1"/>
-      <c r="P18" s="1"/>
+      <c r="N18" s="1">
+        <v>2</v>
+      </c>
+      <c r="O18" s="1">
+        <v>4</v>
+      </c>
+      <c r="P18" s="1">
+        <v>4</v>
+      </c>
       <c r="Q18" s="1"/>
       <c r="R18" s="1"/>
       <c r="S18" s="1"/>
@@ -2652,7 +2751,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A19" s="11">
         <v>17</v>
       </c>
@@ -2692,9 +2791,15 @@
       <c r="M19" s="1">
         <v>2</v>
       </c>
-      <c r="N19" s="1"/>
-      <c r="O19" s="1"/>
-      <c r="P19" s="1"/>
+      <c r="N19" s="1">
+        <v>1</v>
+      </c>
+      <c r="O19" s="1">
+        <v>0</v>
+      </c>
+      <c r="P19" s="1">
+        <v>4</v>
+      </c>
       <c r="Q19" s="1"/>
       <c r="R19" s="1"/>
       <c r="S19" s="1"/>
@@ -2702,7 +2807,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A20" s="11">
         <v>18</v>
       </c>
@@ -2742,9 +2847,15 @@
       <c r="M20" s="1">
         <v>2</v>
       </c>
-      <c r="N20" s="1"/>
-      <c r="O20" s="1"/>
-      <c r="P20" s="1"/>
+      <c r="N20" s="1">
+        <v>2</v>
+      </c>
+      <c r="O20" s="1">
+        <v>4</v>
+      </c>
+      <c r="P20" s="1">
+        <v>3</v>
+      </c>
       <c r="Q20" s="1"/>
       <c r="R20" s="1"/>
       <c r="S20" s="1"/>
@@ -2752,7 +2863,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A21" s="11">
         <v>19</v>
       </c>
@@ -2792,9 +2903,15 @@
       <c r="M21" s="1">
         <v>1</v>
       </c>
-      <c r="N21" s="1"/>
-      <c r="O21" s="1"/>
-      <c r="P21" s="1"/>
+      <c r="N21" s="1">
+        <v>3</v>
+      </c>
+      <c r="O21" s="1">
+        <v>0</v>
+      </c>
+      <c r="P21" s="1">
+        <v>2</v>
+      </c>
       <c r="Q21" s="1"/>
       <c r="R21" s="1"/>
       <c r="S21" s="1"/>
@@ -2802,7 +2919,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A22" s="11">
         <v>20</v>
       </c>
@@ -2842,9 +2959,15 @@
       <c r="M22" s="1">
         <v>3</v>
       </c>
-      <c r="N22" s="1"/>
-      <c r="O22" s="1"/>
-      <c r="P22" s="1"/>
+      <c r="N22" s="1">
+        <v>4</v>
+      </c>
+      <c r="O22" s="1">
+        <v>0</v>
+      </c>
+      <c r="P22" s="1">
+        <v>4</v>
+      </c>
       <c r="Q22" s="1"/>
       <c r="R22" s="1"/>
       <c r="S22" s="1"/>
@@ -2852,7 +2975,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A23" s="11">
         <v>21</v>
       </c>
@@ -2892,9 +3015,15 @@
       <c r="M23" s="1">
         <v>3</v>
       </c>
-      <c r="N23" s="1"/>
-      <c r="O23" s="1"/>
-      <c r="P23" s="1"/>
+      <c r="N23" s="1">
+        <v>0</v>
+      </c>
+      <c r="O23" s="1">
+        <v>0</v>
+      </c>
+      <c r="P23" s="1">
+        <v>0</v>
+      </c>
       <c r="Q23" s="1"/>
       <c r="R23" s="1"/>
       <c r="S23" s="1"/>
@@ -2902,7 +3031,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A24" s="11">
         <v>22</v>
       </c>
@@ -2942,9 +3071,15 @@
       <c r="M24" s="1">
         <v>3</v>
       </c>
-      <c r="N24" s="1"/>
-      <c r="O24" s="1"/>
-      <c r="P24" s="1"/>
+      <c r="N24" s="1">
+        <v>1</v>
+      </c>
+      <c r="O24" s="1">
+        <v>0</v>
+      </c>
+      <c r="P24" s="1">
+        <v>0</v>
+      </c>
       <c r="Q24" s="1"/>
       <c r="R24" s="1"/>
       <c r="S24" s="1"/>
@@ -2952,7 +3087,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A25" s="11">
         <v>23</v>
       </c>
@@ -2992,9 +3127,15 @@
       <c r="M25" s="1">
         <v>0</v>
       </c>
-      <c r="N25" s="1"/>
-      <c r="O25" s="1"/>
-      <c r="P25" s="1"/>
+      <c r="N25" s="1">
+        <v>3</v>
+      </c>
+      <c r="O25" s="1">
+        <v>3</v>
+      </c>
+      <c r="P25" s="1">
+        <v>0</v>
+      </c>
       <c r="Q25" s="1"/>
       <c r="R25" s="1"/>
       <c r="S25" s="1"/>
@@ -3002,7 +3143,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A26" s="11">
         <v>24</v>
       </c>
@@ -3042,9 +3183,15 @@
       <c r="M26" s="1">
         <v>1</v>
       </c>
-      <c r="N26" s="1"/>
-      <c r="O26" s="1"/>
-      <c r="P26" s="1"/>
+      <c r="N26" s="1">
+        <v>1</v>
+      </c>
+      <c r="O26" s="1">
+        <v>0</v>
+      </c>
+      <c r="P26" s="1">
+        <v>2</v>
+      </c>
       <c r="Q26" s="1"/>
       <c r="R26" s="1"/>
       <c r="S26" s="1"/>
@@ -3052,7 +3199,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A27" s="11">
         <v>25</v>
       </c>
@@ -3092,9 +3239,15 @@
       <c r="M27" s="1">
         <v>1</v>
       </c>
-      <c r="N27" s="1"/>
-      <c r="O27" s="1"/>
-      <c r="P27" s="1"/>
+      <c r="N27" s="1">
+        <v>3</v>
+      </c>
+      <c r="O27" s="1">
+        <v>0</v>
+      </c>
+      <c r="P27" s="1">
+        <v>3</v>
+      </c>
       <c r="Q27" s="1"/>
       <c r="R27" s="1"/>
       <c r="S27" s="1"/>
@@ -3102,7 +3255,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A28" s="11">
         <v>26</v>
       </c>
@@ -3142,9 +3295,15 @@
       <c r="M28" s="1">
         <v>1</v>
       </c>
-      <c r="N28" s="1"/>
-      <c r="O28" s="1"/>
-      <c r="P28" s="1"/>
+      <c r="N28" s="1">
+        <v>1</v>
+      </c>
+      <c r="O28" s="1">
+        <v>0</v>
+      </c>
+      <c r="P28" s="1">
+        <v>1</v>
+      </c>
       <c r="Q28" s="1"/>
       <c r="R28" s="1"/>
       <c r="S28" s="1"/>
@@ -3152,7 +3311,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A29" s="11">
         <v>27</v>
       </c>
@@ -3192,9 +3351,15 @@
       <c r="M29" s="1">
         <v>2</v>
       </c>
-      <c r="N29" s="1"/>
-      <c r="O29" s="1"/>
-      <c r="P29" s="1"/>
+      <c r="N29" s="1">
+        <v>4</v>
+      </c>
+      <c r="O29" s="1">
+        <v>4</v>
+      </c>
+      <c r="P29" s="1">
+        <v>5</v>
+      </c>
       <c r="Q29" s="1"/>
       <c r="R29" s="1"/>
       <c r="S29" s="1"/>
@@ -3202,7 +3367,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A30" s="11">
         <v>28</v>
       </c>
@@ -3242,9 +3407,15 @@
       <c r="M30" s="1">
         <v>0</v>
       </c>
-      <c r="N30" s="1"/>
-      <c r="O30" s="1"/>
-      <c r="P30" s="1"/>
+      <c r="N30" s="1">
+        <v>0</v>
+      </c>
+      <c r="O30" s="1">
+        <v>0</v>
+      </c>
+      <c r="P30" s="1">
+        <v>0</v>
+      </c>
       <c r="Q30" s="1"/>
       <c r="R30" s="1"/>
       <c r="S30" s="1"/>
@@ -3252,7 +3423,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A31" s="11">
         <v>29</v>
       </c>
@@ -3292,9 +3463,15 @@
       <c r="M31" s="1">
         <v>1</v>
       </c>
-      <c r="N31" s="1"/>
-      <c r="O31" s="1"/>
-      <c r="P31" s="1"/>
+      <c r="N31" s="1">
+        <v>0</v>
+      </c>
+      <c r="O31" s="1">
+        <v>4</v>
+      </c>
+      <c r="P31" s="1">
+        <v>2</v>
+      </c>
       <c r="Q31" s="1"/>
       <c r="R31" s="1"/>
       <c r="S31" s="1"/>
@@ -3302,7 +3479,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A32" s="11">
         <v>30</v>
       </c>
@@ -3342,9 +3519,15 @@
       <c r="M32" s="1">
         <v>0</v>
       </c>
-      <c r="N32" s="1"/>
-      <c r="O32" s="1"/>
-      <c r="P32" s="1"/>
+      <c r="N32" s="1">
+        <v>0</v>
+      </c>
+      <c r="O32" s="1">
+        <v>3</v>
+      </c>
+      <c r="P32" s="1">
+        <v>3</v>
+      </c>
       <c r="Q32" s="1"/>
       <c r="R32" s="1"/>
       <c r="S32" s="1"/>
@@ -3352,7 +3535,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="33" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A33" s="11">
         <v>31</v>
       </c>
@@ -3392,9 +3575,15 @@
       <c r="M33" s="1">
         <v>0</v>
       </c>
-      <c r="N33" s="1"/>
-      <c r="O33" s="1"/>
-      <c r="P33" s="1"/>
+      <c r="N33" s="1">
+        <v>4</v>
+      </c>
+      <c r="O33" s="1">
+        <v>4</v>
+      </c>
+      <c r="P33" s="1">
+        <v>4</v>
+      </c>
       <c r="Q33" s="1"/>
       <c r="R33" s="1"/>
       <c r="S33" s="1"/>
@@ -3402,7 +3591,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="34" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A34" s="11">
         <v>32</v>
       </c>
@@ -3442,9 +3631,15 @@
       <c r="M34" s="1">
         <v>1</v>
       </c>
-      <c r="N34" s="1"/>
-      <c r="O34" s="1"/>
-      <c r="P34" s="1"/>
+      <c r="N34" s="1">
+        <v>4</v>
+      </c>
+      <c r="O34" s="1">
+        <v>3</v>
+      </c>
+      <c r="P34" s="1">
+        <v>5</v>
+      </c>
       <c r="Q34" s="1"/>
       <c r="R34" s="1"/>
       <c r="S34" s="1"/>
@@ -3452,7 +3647,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="35" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A35" s="11">
         <v>33</v>
       </c>
@@ -3492,9 +3687,15 @@
       <c r="M35" s="1">
         <v>3</v>
       </c>
-      <c r="N35" s="1"/>
-      <c r="O35" s="1"/>
-      <c r="P35" s="1"/>
+      <c r="N35" s="1">
+        <v>3</v>
+      </c>
+      <c r="O35" s="1">
+        <v>4</v>
+      </c>
+      <c r="P35" s="1">
+        <v>4</v>
+      </c>
       <c r="Q35" s="1"/>
       <c r="R35" s="1"/>
       <c r="S35" s="1"/>
@@ -3502,7 +3703,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="36" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A36" s="11">
         <v>34</v>
       </c>
@@ -3542,9 +3743,15 @@
       <c r="M36" s="1">
         <v>1</v>
       </c>
-      <c r="N36" s="1"/>
-      <c r="O36" s="1"/>
-      <c r="P36" s="1"/>
+      <c r="N36" s="1">
+        <v>0</v>
+      </c>
+      <c r="O36" s="1">
+        <v>0</v>
+      </c>
+      <c r="P36" s="1">
+        <v>3</v>
+      </c>
       <c r="Q36" s="1"/>
       <c r="R36" s="1"/>
       <c r="S36" s="1"/>
@@ -3552,7 +3759,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="37" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A37" s="11">
         <v>35</v>
       </c>
@@ -3592,9 +3799,15 @@
       <c r="M37" s="1">
         <v>1</v>
       </c>
-      <c r="N37" s="1"/>
-      <c r="O37" s="1"/>
-      <c r="P37" s="1"/>
+      <c r="N37" s="1">
+        <v>2</v>
+      </c>
+      <c r="O37" s="1">
+        <v>0</v>
+      </c>
+      <c r="P37" s="1">
+        <v>2</v>
+      </c>
       <c r="Q37" s="1"/>
       <c r="R37" s="1"/>
       <c r="S37" s="1"/>
@@ -3602,7 +3815,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="38" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A38" s="11">
         <v>36</v>
       </c>
@@ -3642,9 +3855,15 @@
       <c r="M38" s="1">
         <v>1</v>
       </c>
-      <c r="N38" s="1"/>
-      <c r="O38" s="1"/>
-      <c r="P38" s="1"/>
+      <c r="N38" s="1">
+        <v>0</v>
+      </c>
+      <c r="O38" s="1">
+        <v>0</v>
+      </c>
+      <c r="P38" s="1">
+        <v>0</v>
+      </c>
       <c r="Q38" s="1"/>
       <c r="R38" s="1"/>
       <c r="S38" s="1"/>
@@ -3652,7 +3871,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="39" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A39" s="11">
         <v>37</v>
       </c>
@@ -3692,9 +3911,15 @@
       <c r="M39" s="1">
         <v>5</v>
       </c>
-      <c r="N39" s="1"/>
-      <c r="O39" s="1"/>
-      <c r="P39" s="1"/>
+      <c r="N39" s="1">
+        <v>1</v>
+      </c>
+      <c r="O39" s="1">
+        <v>5</v>
+      </c>
+      <c r="P39" s="1">
+        <v>4</v>
+      </c>
       <c r="Q39" s="1"/>
       <c r="R39" s="1"/>
       <c r="S39" s="1"/>
@@ -3702,7 +3927,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="40" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A40" s="11">
         <v>38</v>
       </c>
@@ -3742,9 +3967,15 @@
       <c r="M40" s="1">
         <v>2</v>
       </c>
-      <c r="N40" s="1"/>
-      <c r="O40" s="1"/>
-      <c r="P40" s="1"/>
+      <c r="N40" s="1">
+        <v>2</v>
+      </c>
+      <c r="O40" s="1">
+        <v>0</v>
+      </c>
+      <c r="P40" s="1">
+        <v>2</v>
+      </c>
       <c r="Q40" s="1"/>
       <c r="R40" s="1"/>
       <c r="S40" s="1"/>
@@ -3752,7 +3983,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="41" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A41" s="11">
         <v>39</v>
       </c>
@@ -3792,9 +4023,15 @@
       <c r="M41" s="1">
         <v>0</v>
       </c>
-      <c r="N41" s="1"/>
-      <c r="O41" s="1"/>
-      <c r="P41" s="1"/>
+      <c r="N41" s="1">
+        <v>0</v>
+      </c>
+      <c r="O41" s="1">
+        <v>0</v>
+      </c>
+      <c r="P41" s="1">
+        <v>1</v>
+      </c>
       <c r="Q41" s="1"/>
       <c r="R41" s="1"/>
       <c r="S41" s="1"/>
@@ -3802,7 +4039,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A42" s="11">
         <v>40</v>
       </c>
@@ -3842,9 +4079,15 @@
       <c r="M42" s="1">
         <v>0</v>
       </c>
-      <c r="N42" s="1"/>
-      <c r="O42" s="1"/>
-      <c r="P42" s="1"/>
+      <c r="N42" s="1">
+        <v>2</v>
+      </c>
+      <c r="O42" s="1">
+        <v>3</v>
+      </c>
+      <c r="P42" s="1">
+        <v>3</v>
+      </c>
       <c r="Q42" s="1"/>
       <c r="R42" s="1"/>
       <c r="S42" s="1"/>
@@ -3852,7 +4095,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="43" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A43" s="11">
         <v>41</v>
       </c>
@@ -3892,9 +4135,15 @@
       <c r="M43" s="1">
         <v>3</v>
       </c>
-      <c r="N43" s="1"/>
-      <c r="O43" s="1"/>
-      <c r="P43" s="1"/>
+      <c r="N43" s="1">
+        <v>5</v>
+      </c>
+      <c r="O43" s="1">
+        <v>5</v>
+      </c>
+      <c r="P43" s="1">
+        <v>4</v>
+      </c>
       <c r="Q43" s="1"/>
       <c r="R43" s="1"/>
       <c r="S43" s="1"/>
@@ -3902,7 +4151,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="44" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A44" s="11">
         <v>42</v>
       </c>
@@ -3942,9 +4191,15 @@
       <c r="M44" s="1">
         <v>1</v>
       </c>
-      <c r="N44" s="1"/>
-      <c r="O44" s="1"/>
-      <c r="P44" s="1"/>
+      <c r="N44" s="1">
+        <v>1</v>
+      </c>
+      <c r="O44" s="1">
+        <v>0</v>
+      </c>
+      <c r="P44" s="1">
+        <v>3</v>
+      </c>
       <c r="Q44" s="1"/>
       <c r="R44" s="1"/>
       <c r="S44" s="1"/>
@@ -3952,7 +4207,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="45" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A45" s="11">
         <v>43</v>
       </c>
@@ -3992,9 +4247,15 @@
       <c r="M45" s="1">
         <v>1</v>
       </c>
-      <c r="N45" s="1"/>
-      <c r="O45" s="1"/>
-      <c r="P45" s="1"/>
+      <c r="N45" s="1">
+        <v>2</v>
+      </c>
+      <c r="O45" s="1">
+        <v>4</v>
+      </c>
+      <c r="P45" s="1">
+        <v>2</v>
+      </c>
       <c r="Q45" s="1"/>
       <c r="R45" s="1"/>
       <c r="S45" s="1"/>
@@ -4002,7 +4263,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="46" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A46" s="11">
         <v>44</v>
       </c>
@@ -4042,9 +4303,15 @@
       <c r="M46" s="1">
         <v>3</v>
       </c>
-      <c r="N46" s="1"/>
-      <c r="O46" s="1"/>
-      <c r="P46" s="1"/>
+      <c r="N46" s="1">
+        <v>3</v>
+      </c>
+      <c r="O46" s="1">
+        <v>4</v>
+      </c>
+      <c r="P46" s="1">
+        <v>1</v>
+      </c>
       <c r="Q46" s="1"/>
       <c r="R46" s="1"/>
       <c r="S46" s="1"/>
@@ -4052,7 +4319,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="47" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A47" s="11">
         <v>45</v>
       </c>
@@ -4092,9 +4359,15 @@
       <c r="M47" s="1">
         <v>4</v>
       </c>
-      <c r="N47" s="1"/>
-      <c r="O47" s="1"/>
-      <c r="P47" s="1"/>
+      <c r="N47" s="1">
+        <v>5</v>
+      </c>
+      <c r="O47" s="1">
+        <v>4</v>
+      </c>
+      <c r="P47" s="1">
+        <v>5</v>
+      </c>
       <c r="Q47" s="1"/>
       <c r="R47" s="1"/>
       <c r="S47" s="1"/>
@@ -4102,7 +4375,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="48" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A48" s="11">
         <v>46</v>
       </c>
@@ -4142,9 +4415,15 @@
       <c r="M48" s="1">
         <v>3</v>
       </c>
-      <c r="N48" s="1"/>
-      <c r="O48" s="1"/>
-      <c r="P48" s="1"/>
+      <c r="N48" s="1">
+        <v>3</v>
+      </c>
+      <c r="O48" s="1">
+        <v>4</v>
+      </c>
+      <c r="P48" s="1">
+        <v>2</v>
+      </c>
       <c r="Q48" s="1"/>
       <c r="R48" s="1"/>
       <c r="S48" s="1"/>
@@ -4152,7 +4431,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="49" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A49" s="11">
         <v>47</v>
       </c>
@@ -4192,9 +4471,15 @@
       <c r="M49" s="1">
         <v>1</v>
       </c>
-      <c r="N49" s="1"/>
-      <c r="O49" s="1"/>
-      <c r="P49" s="1"/>
+      <c r="N49" s="1">
+        <v>2</v>
+      </c>
+      <c r="O49" s="1">
+        <v>4</v>
+      </c>
+      <c r="P49" s="1">
+        <v>1</v>
+      </c>
       <c r="Q49" s="1"/>
       <c r="R49" s="1"/>
       <c r="S49" s="1"/>
@@ -4202,7 +4487,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="50" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A50" s="11">
         <v>48</v>
       </c>
@@ -4242,9 +4527,15 @@
       <c r="M50" s="1">
         <v>2</v>
       </c>
-      <c r="N50" s="1"/>
-      <c r="O50" s="1"/>
-      <c r="P50" s="1"/>
+      <c r="N50" s="1">
+        <v>4</v>
+      </c>
+      <c r="O50" s="1">
+        <v>1</v>
+      </c>
+      <c r="P50" s="1">
+        <v>2</v>
+      </c>
       <c r="Q50" s="1"/>
       <c r="R50" s="1"/>
       <c r="S50" s="1"/>
@@ -4252,7 +4543,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="51" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A51" s="11">
         <v>49</v>
       </c>
@@ -4292,9 +4583,15 @@
       <c r="M51" s="1">
         <v>2</v>
       </c>
-      <c r="N51" s="1"/>
-      <c r="O51" s="1"/>
-      <c r="P51" s="1"/>
+      <c r="N51" s="1">
+        <v>3</v>
+      </c>
+      <c r="O51" s="1">
+        <v>3</v>
+      </c>
+      <c r="P51" s="1">
+        <v>1</v>
+      </c>
       <c r="Q51" s="1"/>
       <c r="R51" s="1"/>
       <c r="S51" s="1"/>
@@ -4302,7 +4599,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="52" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A52" s="11">
         <v>50</v>
       </c>
@@ -4342,9 +4639,15 @@
       <c r="M52" s="1">
         <v>2</v>
       </c>
-      <c r="N52" s="1"/>
-      <c r="O52" s="1"/>
-      <c r="P52" s="1"/>
+      <c r="N52" s="1">
+        <v>2</v>
+      </c>
+      <c r="O52" s="1">
+        <v>0</v>
+      </c>
+      <c r="P52" s="1">
+        <v>1</v>
+      </c>
       <c r="Q52" s="1"/>
       <c r="R52" s="1"/>
       <c r="S52" s="1"/>
@@ -4352,7 +4655,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="53" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A53" s="11">
         <v>51</v>
       </c>
@@ -4392,9 +4695,15 @@
       <c r="M53" s="1">
         <v>3</v>
       </c>
-      <c r="N53" s="1"/>
-      <c r="O53" s="1"/>
-      <c r="P53" s="1"/>
+      <c r="N53" s="1">
+        <v>1</v>
+      </c>
+      <c r="O53" s="1">
+        <v>3</v>
+      </c>
+      <c r="P53" s="1">
+        <v>3</v>
+      </c>
       <c r="Q53" s="1"/>
       <c r="R53" s="1"/>
       <c r="S53" s="1"/>
@@ -4402,7 +4711,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="54" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A54" s="11">
         <v>52</v>
       </c>
@@ -4442,9 +4751,15 @@
       <c r="M54" s="1">
         <v>2</v>
       </c>
-      <c r="N54" s="1"/>
-      <c r="O54" s="1"/>
-      <c r="P54" s="1"/>
+      <c r="N54" s="1">
+        <v>4</v>
+      </c>
+      <c r="O54" s="1">
+        <v>4</v>
+      </c>
+      <c r="P54" s="1">
+        <v>4</v>
+      </c>
       <c r="Q54" s="1"/>
       <c r="R54" s="1"/>
       <c r="S54" s="1"/>
@@ -4452,7 +4767,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="55" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A55" s="11">
         <v>53</v>
       </c>
@@ -4492,9 +4807,15 @@
       <c r="M55" s="1">
         <v>4</v>
       </c>
-      <c r="N55" s="1"/>
-      <c r="O55" s="1"/>
-      <c r="P55" s="1"/>
+      <c r="N55" s="1">
+        <v>4</v>
+      </c>
+      <c r="O55" s="1">
+        <v>4</v>
+      </c>
+      <c r="P55" s="1">
+        <v>4</v>
+      </c>
       <c r="Q55" s="1"/>
       <c r="R55" s="1"/>
       <c r="S55" s="1"/>
@@ -4502,7 +4823,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="56" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A56" s="11">
         <v>54</v>
       </c>
@@ -4542,9 +4863,15 @@
       <c r="M56" s="1">
         <v>1</v>
       </c>
-      <c r="N56" s="1"/>
-      <c r="O56" s="1"/>
-      <c r="P56" s="1"/>
+      <c r="N56" s="1">
+        <v>3</v>
+      </c>
+      <c r="O56" s="1">
+        <v>4</v>
+      </c>
+      <c r="P56" s="1">
+        <v>2</v>
+      </c>
       <c r="Q56" s="1"/>
       <c r="R56" s="1"/>
       <c r="S56" s="1"/>
@@ -4552,7 +4879,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="57" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A57" s="19">
         <v>55</v>
       </c>
@@ -4592,9 +4919,15 @@
       <c r="M57" s="22">
         <v>2</v>
       </c>
-      <c r="N57" s="22"/>
-      <c r="O57" s="22"/>
-      <c r="P57" s="22"/>
+      <c r="N57" s="22">
+        <v>3</v>
+      </c>
+      <c r="O57" s="22">
+        <v>4</v>
+      </c>
+      <c r="P57" s="22">
+        <v>5</v>
+      </c>
       <c r="Q57" s="22"/>
       <c r="R57" s="22"/>
       <c r="S57" s="22"/>
@@ -4602,7 +4935,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="58" spans="1:20" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="58" spans="1:20" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:B1"/>
@@ -4616,95 +4949,95 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7CD6AE0E-6B38-4517-9EE7-74576DF1F95D}">
   <dimension ref="A1:T51"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A1" s="23"/>
-      <c r="B1" s="23"/>
+    <row r="1" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A1" s="33"/>
+      <c r="B1" s="33"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
-      <c r="F1" s="24" t="s">
-        <v>0</v>
-      </c>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
-      <c r="I1" s="25"/>
-      <c r="J1" s="25"/>
-      <c r="K1" s="25"/>
-      <c r="L1" s="25"/>
-      <c r="M1" s="25"/>
-      <c r="N1" s="25"/>
-      <c r="O1" s="25"/>
-      <c r="P1" s="25"/>
-      <c r="Q1" s="25"/>
-      <c r="R1" s="25"/>
-      <c r="S1" s="26"/>
+      <c r="F1" s="34" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1" s="35"/>
+      <c r="H1" s="35"/>
+      <c r="I1" s="35"/>
+      <c r="J1" s="35"/>
+      <c r="K1" s="35"/>
+      <c r="L1" s="35"/>
+      <c r="M1" s="35"/>
+      <c r="N1" s="35"/>
+      <c r="O1" s="35"/>
+      <c r="P1" s="35"/>
+      <c r="Q1" s="35"/>
+      <c r="R1" s="35"/>
+      <c r="S1" s="36"/>
       <c r="T1" s="2"/>
     </row>
-    <row r="2" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="23"/>
-      <c r="B2" s="23"/>
+    <row r="2" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="33"/>
+      <c r="B2" s="33"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
-      <c r="F2" s="36" t="s">
+      <c r="F2" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="G2" s="37" t="s">
-        <v>2</v>
-      </c>
-      <c r="H2" s="37" t="s">
-        <v>3</v>
-      </c>
-      <c r="I2" s="37" t="s">
-        <v>4</v>
-      </c>
-      <c r="J2" s="37" t="s">
-        <v>5</v>
-      </c>
-      <c r="K2" s="37" t="s">
+      <c r="G2" s="32" t="s">
+        <v>2</v>
+      </c>
+      <c r="H2" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="I2" s="32" t="s">
+        <v>4</v>
+      </c>
+      <c r="J2" s="32" t="s">
+        <v>5</v>
+      </c>
+      <c r="K2" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="L2" s="37" t="s">
+      <c r="L2" s="32" t="s">
         <v>7</v>
       </c>
-      <c r="M2" s="37" t="s">
+      <c r="M2" s="32" t="s">
         <v>8</v>
       </c>
-      <c r="N2" s="37" t="s">
+      <c r="N2" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="O2" s="37" t="s">
+      <c r="O2" s="32" t="s">
         <v>10</v>
       </c>
-      <c r="P2" s="37" t="s">
+      <c r="P2" s="32" t="s">
         <v>11</v>
       </c>
-      <c r="Q2" s="37" t="s">
+      <c r="Q2" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="R2" s="37" t="s">
+      <c r="R2" s="32" t="s">
         <v>13</v>
       </c>
-      <c r="S2" s="37" t="s">
+      <c r="S2" s="32" t="s">
         <v>14</v>
       </c>
       <c r="T2" s="5" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A3" s="11">
         <v>1</v>
       </c>
-      <c r="B3" s="28" t="s">
+      <c r="B3" s="24" t="s">
         <v>172</v>
       </c>
-      <c r="C3" s="28" t="s">
+      <c r="C3" s="24" t="s">
         <v>173</v>
       </c>
-      <c r="D3" s="28" t="s">
+      <c r="D3" s="24" t="s">
         <v>174</v>
       </c>
       <c r="E3" s="8">
@@ -4734,9 +5067,15 @@
       <c r="M3" s="1">
         <v>2</v>
       </c>
-      <c r="N3" s="1"/>
-      <c r="O3" s="1"/>
-      <c r="P3" s="1"/>
+      <c r="N3" s="1">
+        <v>1</v>
+      </c>
+      <c r="O3" s="1">
+        <v>2</v>
+      </c>
+      <c r="P3" s="1">
+        <v>3</v>
+      </c>
       <c r="Q3" s="1"/>
       <c r="R3" s="1"/>
       <c r="S3" s="1"/>
@@ -4744,17 +5083,17 @@
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A4" s="11">
         <v>2</v>
       </c>
-      <c r="B4" s="29" t="s">
+      <c r="B4" s="25" t="s">
         <v>175</v>
       </c>
-      <c r="C4" s="29" t="s">
+      <c r="C4" s="25" t="s">
         <v>176</v>
       </c>
-      <c r="D4" s="29" t="s">
+      <c r="D4" s="25" t="s">
         <v>177</v>
       </c>
       <c r="E4" s="13">
@@ -4784,9 +5123,15 @@
       <c r="M4" s="1">
         <v>2</v>
       </c>
-      <c r="N4" s="1"/>
-      <c r="O4" s="1"/>
-      <c r="P4" s="1"/>
+      <c r="N4" s="1">
+        <v>2</v>
+      </c>
+      <c r="O4" s="1">
+        <v>3</v>
+      </c>
+      <c r="P4" s="1">
+        <v>1</v>
+      </c>
       <c r="Q4" s="1"/>
       <c r="R4" s="1"/>
       <c r="S4" s="1"/>
@@ -4794,17 +5139,17 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A5" s="11">
         <v>3</v>
       </c>
-      <c r="B5" s="29" t="s">
+      <c r="B5" s="25" t="s">
         <v>178</v>
       </c>
-      <c r="C5" s="29" t="s">
+      <c r="C5" s="25" t="s">
         <v>179</v>
       </c>
-      <c r="D5" s="29" t="s">
+      <c r="D5" s="25" t="s">
         <v>180</v>
       </c>
       <c r="E5" s="13">
@@ -4834,9 +5179,15 @@
       <c r="M5" s="1">
         <v>0</v>
       </c>
-      <c r="N5" s="1"/>
-      <c r="O5" s="1"/>
-      <c r="P5" s="1"/>
+      <c r="N5" s="1">
+        <v>0</v>
+      </c>
+      <c r="O5" s="1">
+        <v>0</v>
+      </c>
+      <c r="P5" s="1">
+        <v>0</v>
+      </c>
       <c r="Q5" s="1"/>
       <c r="R5" s="1"/>
       <c r="S5" s="1"/>
@@ -4844,17 +5195,17 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A6" s="11">
         <v>4</v>
       </c>
-      <c r="B6" s="29" t="s">
+      <c r="B6" s="25" t="s">
         <v>181</v>
       </c>
-      <c r="C6" s="29" t="s">
+      <c r="C6" s="25" t="s">
         <v>182</v>
       </c>
-      <c r="D6" s="29" t="s">
+      <c r="D6" s="25" t="s">
         <v>183</v>
       </c>
       <c r="E6" s="13">
@@ -4884,9 +5235,15 @@
       <c r="M6" s="1">
         <v>1</v>
       </c>
-      <c r="N6" s="1"/>
-      <c r="O6" s="1"/>
-      <c r="P6" s="1"/>
+      <c r="N6" s="1">
+        <v>1</v>
+      </c>
+      <c r="O6" s="1">
+        <v>0</v>
+      </c>
+      <c r="P6" s="1">
+        <v>1</v>
+      </c>
       <c r="Q6" s="1"/>
       <c r="R6" s="1"/>
       <c r="S6" s="1"/>
@@ -4894,17 +5251,17 @@
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A7" s="11">
         <v>5</v>
       </c>
-      <c r="B7" s="29" t="s">
+      <c r="B7" s="25" t="s">
         <v>184</v>
       </c>
-      <c r="C7" s="29" t="s">
+      <c r="C7" s="25" t="s">
         <v>57</v>
       </c>
-      <c r="D7" s="29" t="s">
+      <c r="D7" s="25" t="s">
         <v>185</v>
       </c>
       <c r="E7" s="13">
@@ -4934,9 +5291,15 @@
       <c r="M7" s="1">
         <v>2</v>
       </c>
-      <c r="N7" s="1"/>
-      <c r="O7" s="1"/>
-      <c r="P7" s="1"/>
+      <c r="N7" s="1">
+        <v>2</v>
+      </c>
+      <c r="O7" s="1">
+        <v>4</v>
+      </c>
+      <c r="P7" s="1">
+        <v>3</v>
+      </c>
       <c r="Q7" s="1"/>
       <c r="R7" s="1"/>
       <c r="S7" s="1"/>
@@ -4944,17 +5307,17 @@
         <v>33</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A8" s="11">
         <v>6</v>
       </c>
-      <c r="B8" s="29" t="s">
+      <c r="B8" s="25" t="s">
         <v>186</v>
       </c>
-      <c r="C8" s="29" t="s">
+      <c r="C8" s="25" t="s">
         <v>187</v>
       </c>
-      <c r="D8" s="30" t="s">
+      <c r="D8" s="26" t="s">
         <v>111</v>
       </c>
       <c r="E8" s="13">
@@ -4984,9 +5347,15 @@
       <c r="M8" s="1">
         <v>0</v>
       </c>
-      <c r="N8" s="1"/>
-      <c r="O8" s="1"/>
-      <c r="P8" s="1"/>
+      <c r="N8" s="1">
+        <v>0</v>
+      </c>
+      <c r="O8" s="1">
+        <v>4</v>
+      </c>
+      <c r="P8" s="1">
+        <v>2</v>
+      </c>
       <c r="Q8" s="1"/>
       <c r="R8" s="1"/>
       <c r="S8" s="1"/>
@@ -4994,17 +5363,17 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A9" s="11">
         <v>7</v>
       </c>
-      <c r="B9" s="29" t="s">
+      <c r="B9" s="25" t="s">
         <v>188</v>
       </c>
-      <c r="C9" s="29" t="s">
+      <c r="C9" s="25" t="s">
         <v>189</v>
       </c>
-      <c r="D9" s="29" t="s">
+      <c r="D9" s="25" t="s">
         <v>190</v>
       </c>
       <c r="E9" s="13">
@@ -5034,9 +5403,15 @@
       <c r="M9" s="1">
         <v>3</v>
       </c>
-      <c r="N9" s="1"/>
-      <c r="O9" s="1"/>
-      <c r="P9" s="1"/>
+      <c r="N9" s="1">
+        <v>3</v>
+      </c>
+      <c r="O9" s="1">
+        <v>5</v>
+      </c>
+      <c r="P9" s="1">
+        <v>2</v>
+      </c>
       <c r="Q9" s="1"/>
       <c r="R9" s="1"/>
       <c r="S9" s="1"/>
@@ -5044,17 +5419,17 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A10" s="11">
         <v>8</v>
       </c>
-      <c r="B10" s="29" t="s">
+      <c r="B10" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="C10" s="29" t="s">
+      <c r="C10" s="25" t="s">
         <v>192</v>
       </c>
-      <c r="D10" s="29" t="s">
+      <c r="D10" s="25" t="s">
         <v>139</v>
       </c>
       <c r="E10" s="13">
@@ -5084,9 +5459,15 @@
       <c r="M10" s="1">
         <v>3</v>
       </c>
-      <c r="N10" s="1"/>
-      <c r="O10" s="1"/>
-      <c r="P10" s="1"/>
+      <c r="N10" s="1">
+        <v>3</v>
+      </c>
+      <c r="O10" s="1">
+        <v>3</v>
+      </c>
+      <c r="P10" s="1">
+        <v>3</v>
+      </c>
       <c r="Q10" s="1"/>
       <c r="R10" s="1"/>
       <c r="S10" s="1"/>
@@ -5094,17 +5475,17 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A11" s="11">
         <v>9</v>
       </c>
-      <c r="B11" s="29" t="s">
+      <c r="B11" s="25" t="s">
         <v>193</v>
       </c>
-      <c r="C11" s="29" t="s">
+      <c r="C11" s="25" t="s">
         <v>194</v>
       </c>
-      <c r="D11" s="29" t="s">
+      <c r="D11" s="25" t="s">
         <v>195</v>
       </c>
       <c r="E11" s="13">
@@ -5134,9 +5515,15 @@
       <c r="M11" s="1">
         <v>3</v>
       </c>
-      <c r="N11" s="1"/>
-      <c r="O11" s="1"/>
-      <c r="P11" s="1"/>
+      <c r="N11" s="1">
+        <v>0</v>
+      </c>
+      <c r="O11" s="1">
+        <v>0</v>
+      </c>
+      <c r="P11" s="1">
+        <v>1</v>
+      </c>
       <c r="Q11" s="1"/>
       <c r="R11" s="1"/>
       <c r="S11" s="1"/>
@@ -5144,17 +5531,17 @@
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A12" s="11">
         <v>10</v>
       </c>
-      <c r="B12" s="29" t="s">
+      <c r="B12" s="25" t="s">
         <v>196</v>
       </c>
-      <c r="C12" s="29" t="s">
+      <c r="C12" s="25" t="s">
         <v>178</v>
       </c>
-      <c r="D12" s="30" t="s">
+      <c r="D12" s="26" t="s">
         <v>197</v>
       </c>
       <c r="E12" s="13">
@@ -5184,9 +5571,15 @@
       <c r="M12" s="1">
         <v>2</v>
       </c>
-      <c r="N12" s="1"/>
-      <c r="O12" s="1"/>
-      <c r="P12" s="1"/>
+      <c r="N12" s="1">
+        <v>1</v>
+      </c>
+      <c r="O12" s="1">
+        <v>4</v>
+      </c>
+      <c r="P12" s="1">
+        <v>3</v>
+      </c>
       <c r="Q12" s="1"/>
       <c r="R12" s="1"/>
       <c r="S12" s="1"/>
@@ -5194,17 +5587,17 @@
         <v>32</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A13" s="11">
         <v>11</v>
       </c>
-      <c r="B13" s="29" t="s">
+      <c r="B13" s="25" t="s">
         <v>198</v>
       </c>
-      <c r="C13" s="29" t="s">
+      <c r="C13" s="25" t="s">
         <v>199</v>
       </c>
-      <c r="D13" s="29" t="s">
+      <c r="D13" s="25" t="s">
         <v>177</v>
       </c>
       <c r="E13" s="13">
@@ -5234,9 +5627,15 @@
       <c r="M13" s="1">
         <v>3</v>
       </c>
-      <c r="N13" s="1"/>
-      <c r="O13" s="1"/>
-      <c r="P13" s="1"/>
+      <c r="N13" s="1">
+        <v>5</v>
+      </c>
+      <c r="O13" s="1">
+        <v>4</v>
+      </c>
+      <c r="P13" s="1">
+        <v>4</v>
+      </c>
       <c r="Q13" s="1"/>
       <c r="R13" s="1"/>
       <c r="S13" s="1"/>
@@ -5244,17 +5643,17 @@
         <v>35</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A14" s="11">
         <v>12</v>
       </c>
-      <c r="B14" s="29" t="s">
+      <c r="B14" s="25" t="s">
         <v>200</v>
       </c>
-      <c r="C14" s="29" t="s">
+      <c r="C14" s="25" t="s">
         <v>201</v>
       </c>
-      <c r="D14" s="29" t="s">
+      <c r="D14" s="25" t="s">
         <v>202</v>
       </c>
       <c r="E14" s="13" t="s">
@@ -5284,9 +5683,15 @@
       <c r="M14" s="1">
         <v>2</v>
       </c>
-      <c r="N14" s="1"/>
-      <c r="O14" s="1"/>
-      <c r="P14" s="1"/>
+      <c r="N14" s="1">
+        <v>3</v>
+      </c>
+      <c r="O14" s="1">
+        <v>0</v>
+      </c>
+      <c r="P14" s="1">
+        <v>2</v>
+      </c>
       <c r="Q14" s="1"/>
       <c r="R14" s="1"/>
       <c r="S14" s="1"/>
@@ -5294,17 +5699,17 @@
         <v>21</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A15" s="11">
         <v>13</v>
       </c>
-      <c r="B15" s="29" t="s">
+      <c r="B15" s="25" t="s">
         <v>204</v>
       </c>
-      <c r="C15" s="29" t="s">
+      <c r="C15" s="25" t="s">
         <v>205</v>
       </c>
-      <c r="D15" s="29" t="s">
+      <c r="D15" s="25" t="s">
         <v>206</v>
       </c>
       <c r="E15" s="13">
@@ -5334,9 +5739,15 @@
       <c r="M15" s="1">
         <v>1</v>
       </c>
-      <c r="N15" s="1"/>
-      <c r="O15" s="1"/>
-      <c r="P15" s="1"/>
+      <c r="N15" s="1">
+        <v>2</v>
+      </c>
+      <c r="O15" s="1">
+        <v>3</v>
+      </c>
+      <c r="P15" s="1">
+        <v>3</v>
+      </c>
       <c r="Q15" s="1"/>
       <c r="R15" s="1"/>
       <c r="S15" s="1"/>
@@ -5344,17 +5755,17 @@
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A16" s="11">
         <v>14</v>
       </c>
-      <c r="B16" s="29" t="s">
+      <c r="B16" s="25" t="s">
         <v>207</v>
       </c>
-      <c r="C16" s="29" t="s">
+      <c r="C16" s="25" t="s">
         <v>147</v>
       </c>
-      <c r="D16" s="29" t="s">
+      <c r="D16" s="25" t="s">
         <v>155</v>
       </c>
       <c r="E16" s="13">
@@ -5384,9 +5795,15 @@
       <c r="M16" s="1">
         <v>3</v>
       </c>
-      <c r="N16" s="1"/>
-      <c r="O16" s="1"/>
-      <c r="P16" s="1"/>
+      <c r="N16" s="1">
+        <v>1</v>
+      </c>
+      <c r="O16" s="1">
+        <v>4</v>
+      </c>
+      <c r="P16" s="1">
+        <v>2</v>
+      </c>
       <c r="Q16" s="1"/>
       <c r="R16" s="1"/>
       <c r="S16" s="1"/>
@@ -5394,17 +5811,17 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A17" s="11">
         <v>15</v>
       </c>
-      <c r="B17" s="29" t="s">
+      <c r="B17" s="25" t="s">
         <v>208</v>
       </c>
-      <c r="C17" s="29" t="s">
+      <c r="C17" s="25" t="s">
         <v>209</v>
       </c>
-      <c r="D17" s="29" t="s">
+      <c r="D17" s="25" t="s">
         <v>210</v>
       </c>
       <c r="E17" s="13">
@@ -5434,9 +5851,15 @@
       <c r="M17" s="1">
         <v>1</v>
       </c>
-      <c r="N17" s="1"/>
-      <c r="O17" s="1"/>
-      <c r="P17" s="1"/>
+      <c r="N17" s="1">
+        <v>2</v>
+      </c>
+      <c r="O17" s="1">
+        <v>0</v>
+      </c>
+      <c r="P17" s="1">
+        <v>1</v>
+      </c>
       <c r="Q17" s="1"/>
       <c r="R17" s="1"/>
       <c r="S17" s="1"/>
@@ -5444,17 +5867,17 @@
         <v>27</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A18" s="11">
         <v>16</v>
       </c>
-      <c r="B18" s="29" t="s">
+      <c r="B18" s="25" t="s">
         <v>211</v>
       </c>
-      <c r="C18" s="29" t="s">
+      <c r="C18" s="25" t="s">
         <v>212</v>
       </c>
-      <c r="D18" s="29" t="s">
+      <c r="D18" s="25" t="s">
         <v>213</v>
       </c>
       <c r="E18" s="13">
@@ -5484,9 +5907,15 @@
       <c r="M18" s="1">
         <v>0</v>
       </c>
-      <c r="N18" s="1"/>
-      <c r="O18" s="1"/>
-      <c r="P18" s="1"/>
+      <c r="N18" s="1">
+        <v>2</v>
+      </c>
+      <c r="O18" s="1">
+        <v>3</v>
+      </c>
+      <c r="P18" s="1">
+        <v>1</v>
+      </c>
       <c r="Q18" s="1"/>
       <c r="R18" s="1"/>
       <c r="S18" s="1"/>
@@ -5494,17 +5923,17 @@
         <v>30</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A19" s="11">
         <v>17</v>
       </c>
-      <c r="B19" s="29" t="s">
+      <c r="B19" s="25" t="s">
         <v>214</v>
       </c>
-      <c r="C19" s="29" t="s">
+      <c r="C19" s="25" t="s">
         <v>215</v>
       </c>
-      <c r="D19" s="29" t="s">
+      <c r="D19" s="25" t="s">
         <v>216</v>
       </c>
       <c r="E19" s="13">
@@ -5534,9 +5963,15 @@
       <c r="M19" s="1">
         <v>3</v>
       </c>
-      <c r="N19" s="1"/>
-      <c r="O19" s="1"/>
-      <c r="P19" s="1"/>
+      <c r="N19" s="1">
+        <v>0</v>
+      </c>
+      <c r="O19" s="1">
+        <v>0</v>
+      </c>
+      <c r="P19" s="1">
+        <v>0</v>
+      </c>
       <c r="Q19" s="1"/>
       <c r="R19" s="1"/>
       <c r="S19" s="1"/>
@@ -5544,17 +5979,17 @@
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A20" s="11">
         <v>18</v>
       </c>
-      <c r="B20" s="29" t="s">
+      <c r="B20" s="25" t="s">
         <v>217</v>
       </c>
-      <c r="C20" s="29" t="s">
+      <c r="C20" s="25" t="s">
         <v>218</v>
       </c>
-      <c r="D20" s="29" t="s">
+      <c r="D20" s="25" t="s">
         <v>219</v>
       </c>
       <c r="E20" s="13">
@@ -5584,9 +6019,15 @@
       <c r="M20" s="1">
         <v>2</v>
       </c>
-      <c r="N20" s="1"/>
-      <c r="O20" s="1"/>
-      <c r="P20" s="1"/>
+      <c r="N20" s="1">
+        <v>3</v>
+      </c>
+      <c r="O20" s="1">
+        <v>3</v>
+      </c>
+      <c r="P20" s="1">
+        <v>2</v>
+      </c>
       <c r="Q20" s="1"/>
       <c r="R20" s="1"/>
       <c r="S20" s="1"/>
@@ -5594,17 +6035,17 @@
         <v>28</v>
       </c>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A21" s="11">
         <v>19</v>
       </c>
-      <c r="B21" s="29" t="s">
+      <c r="B21" s="25" t="s">
         <v>220</v>
       </c>
-      <c r="C21" s="29" t="s">
+      <c r="C21" s="25" t="s">
         <v>221</v>
       </c>
-      <c r="D21" s="29" t="s">
+      <c r="D21" s="25" t="s">
         <v>222</v>
       </c>
       <c r="E21" s="13">
@@ -5634,9 +6075,15 @@
       <c r="M21" s="1">
         <v>1</v>
       </c>
-      <c r="N21" s="1"/>
-      <c r="O21" s="1"/>
-      <c r="P21" s="1"/>
+      <c r="N21" s="1">
+        <v>0</v>
+      </c>
+      <c r="O21" s="1">
+        <v>5</v>
+      </c>
+      <c r="P21" s="1">
+        <v>4</v>
+      </c>
       <c r="Q21" s="1"/>
       <c r="R21" s="1"/>
       <c r="S21" s="1"/>
@@ -5644,17 +6091,17 @@
         <v>26</v>
       </c>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A22" s="11">
         <v>20</v>
       </c>
-      <c r="B22" s="29" t="s">
+      <c r="B22" s="25" t="s">
         <v>223</v>
       </c>
-      <c r="C22" s="29" t="s">
+      <c r="C22" s="25" t="s">
         <v>224</v>
       </c>
-      <c r="D22" s="29" t="s">
+      <c r="D22" s="25" t="s">
         <v>144</v>
       </c>
       <c r="E22" s="13">
@@ -5684,9 +6131,15 @@
       <c r="M22" s="1">
         <v>4</v>
       </c>
-      <c r="N22" s="1"/>
-      <c r="O22" s="1"/>
-      <c r="P22" s="1"/>
+      <c r="N22" s="1">
+        <v>4</v>
+      </c>
+      <c r="O22" s="1">
+        <v>4</v>
+      </c>
+      <c r="P22" s="1">
+        <v>3</v>
+      </c>
       <c r="Q22" s="1"/>
       <c r="R22" s="1"/>
       <c r="S22" s="1"/>
@@ -5694,17 +6147,17 @@
         <v>30</v>
       </c>
     </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A23" s="11">
         <v>21</v>
       </c>
-      <c r="B23" s="29" t="s">
+      <c r="B23" s="25" t="s">
         <v>225</v>
       </c>
-      <c r="C23" s="29" t="s">
+      <c r="C23" s="25" t="s">
         <v>226</v>
       </c>
-      <c r="D23" s="29" t="s">
+      <c r="D23" s="25" t="s">
         <v>59</v>
       </c>
       <c r="E23" s="13">
@@ -5734,9 +6187,15 @@
       <c r="M23" s="1">
         <v>1</v>
       </c>
-      <c r="N23" s="1"/>
-      <c r="O23" s="1"/>
-      <c r="P23" s="1"/>
+      <c r="N23" s="1">
+        <v>1</v>
+      </c>
+      <c r="O23" s="1">
+        <v>2</v>
+      </c>
+      <c r="P23" s="1">
+        <v>0</v>
+      </c>
       <c r="Q23" s="1"/>
       <c r="R23" s="1"/>
       <c r="S23" s="1"/>
@@ -5744,17 +6203,17 @@
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A24" s="11">
         <v>22</v>
       </c>
-      <c r="B24" s="29" t="s">
+      <c r="B24" s="25" t="s">
         <v>227</v>
       </c>
-      <c r="C24" s="29" t="s">
+      <c r="C24" s="25" t="s">
         <v>228</v>
       </c>
-      <c r="D24" s="29" t="s">
+      <c r="D24" s="25" t="s">
         <v>229</v>
       </c>
       <c r="E24" s="13">
@@ -5784,9 +6243,15 @@
       <c r="M24" s="1">
         <v>2</v>
       </c>
-      <c r="N24" s="1"/>
-      <c r="O24" s="1"/>
-      <c r="P24" s="1"/>
+      <c r="N24" s="1">
+        <v>3</v>
+      </c>
+      <c r="O24" s="1">
+        <v>4</v>
+      </c>
+      <c r="P24" s="1">
+        <v>2</v>
+      </c>
       <c r="Q24" s="1"/>
       <c r="R24" s="1"/>
       <c r="S24" s="1"/>
@@ -5794,17 +6259,17 @@
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A25" s="11">
         <v>23</v>
       </c>
-      <c r="B25" s="29" t="s">
+      <c r="B25" s="25" t="s">
         <v>230</v>
       </c>
-      <c r="C25" s="29" t="s">
+      <c r="C25" s="25" t="s">
         <v>230</v>
       </c>
-      <c r="D25" s="29" t="s">
+      <c r="D25" s="25" t="s">
         <v>231</v>
       </c>
       <c r="E25" s="13">
@@ -5834,9 +6299,15 @@
       <c r="M25" s="1">
         <v>0</v>
       </c>
-      <c r="N25" s="1"/>
-      <c r="O25" s="1"/>
-      <c r="P25" s="1"/>
+      <c r="N25" s="1">
+        <v>0</v>
+      </c>
+      <c r="O25" s="1">
+        <v>0</v>
+      </c>
+      <c r="P25" s="1">
+        <v>0</v>
+      </c>
       <c r="Q25" s="1"/>
       <c r="R25" s="1"/>
       <c r="S25" s="1"/>
@@ -5844,17 +6315,17 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A26" s="11">
         <v>24</v>
       </c>
-      <c r="B26" s="29" t="s">
+      <c r="B26" s="25" t="s">
         <v>230</v>
       </c>
-      <c r="C26" s="29" t="s">
+      <c r="C26" s="25" t="s">
         <v>232</v>
       </c>
-      <c r="D26" s="29" t="s">
+      <c r="D26" s="25" t="s">
         <v>233</v>
       </c>
       <c r="E26" s="13">
@@ -5884,9 +6355,15 @@
       <c r="M26" s="1">
         <v>2</v>
       </c>
-      <c r="N26" s="1"/>
-      <c r="O26" s="1"/>
-      <c r="P26" s="1"/>
+      <c r="N26" s="1">
+        <v>0</v>
+      </c>
+      <c r="O26" s="1">
+        <v>0</v>
+      </c>
+      <c r="P26" s="1">
+        <v>0</v>
+      </c>
       <c r="Q26" s="1"/>
       <c r="R26" s="1"/>
       <c r="S26" s="1"/>
@@ -5894,17 +6371,17 @@
         <v>32</v>
       </c>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A27" s="11">
         <v>25</v>
       </c>
-      <c r="B27" s="29" t="s">
+      <c r="B27" s="25" t="s">
         <v>234</v>
       </c>
-      <c r="C27" s="29" t="s">
+      <c r="C27" s="25" t="s">
         <v>235</v>
       </c>
-      <c r="D27" s="29" t="s">
+      <c r="D27" s="25" t="s">
         <v>236</v>
       </c>
       <c r="E27" s="13">
@@ -5934,9 +6411,15 @@
       <c r="M27" s="1">
         <v>2</v>
       </c>
-      <c r="N27" s="1"/>
-      <c r="O27" s="1"/>
-      <c r="P27" s="1"/>
+      <c r="N27" s="1">
+        <v>2</v>
+      </c>
+      <c r="O27" s="1">
+        <v>3</v>
+      </c>
+      <c r="P27" s="1">
+        <v>3</v>
+      </c>
       <c r="Q27" s="1"/>
       <c r="R27" s="1"/>
       <c r="S27" s="1"/>
@@ -5944,17 +6427,17 @@
         <v>34</v>
       </c>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A28" s="11">
         <v>26</v>
       </c>
-      <c r="B28" s="29" t="s">
+      <c r="B28" s="25" t="s">
         <v>237</v>
       </c>
-      <c r="C28" s="29" t="s">
+      <c r="C28" s="25" t="s">
         <v>238</v>
       </c>
-      <c r="D28" s="29" t="s">
+      <c r="D28" s="25" t="s">
         <v>239</v>
       </c>
       <c r="E28" s="13">
@@ -5984,9 +6467,15 @@
       <c r="M28" s="1">
         <v>3</v>
       </c>
-      <c r="N28" s="1"/>
-      <c r="O28" s="1"/>
-      <c r="P28" s="1"/>
+      <c r="N28" s="1">
+        <v>2</v>
+      </c>
+      <c r="O28" s="1">
+        <v>5</v>
+      </c>
+      <c r="P28" s="1">
+        <v>3</v>
+      </c>
       <c r="Q28" s="1"/>
       <c r="R28" s="1"/>
       <c r="S28" s="1"/>
@@ -5994,17 +6483,17 @@
         <v>34</v>
       </c>
     </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A29" s="11">
         <v>27</v>
       </c>
-      <c r="B29" s="29" t="s">
+      <c r="B29" s="25" t="s">
         <v>240</v>
       </c>
-      <c r="C29" s="29" t="s">
+      <c r="C29" s="25" t="s">
         <v>241</v>
       </c>
-      <c r="D29" s="29" t="s">
+      <c r="D29" s="25" t="s">
         <v>242</v>
       </c>
       <c r="E29" s="13" t="s">
@@ -6034,9 +6523,15 @@
       <c r="M29" s="1">
         <v>0</v>
       </c>
-      <c r="N29" s="1"/>
-      <c r="O29" s="1"/>
-      <c r="P29" s="1"/>
+      <c r="N29" s="1">
+        <v>0</v>
+      </c>
+      <c r="O29" s="1">
+        <v>0</v>
+      </c>
+      <c r="P29" s="1">
+        <v>0</v>
+      </c>
       <c r="Q29" s="1"/>
       <c r="R29" s="1"/>
       <c r="S29" s="1"/>
@@ -6044,17 +6539,17 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A30" s="11">
         <v>28</v>
       </c>
-      <c r="B30" s="29" t="s">
+      <c r="B30" s="25" t="s">
         <v>244</v>
       </c>
-      <c r="C30" s="29" t="s">
+      <c r="C30" s="25" t="s">
         <v>245</v>
       </c>
-      <c r="D30" s="29" t="s">
+      <c r="D30" s="25" t="s">
         <v>246</v>
       </c>
       <c r="E30" s="13">
@@ -6084,9 +6579,15 @@
       <c r="M30" s="1">
         <v>0</v>
       </c>
-      <c r="N30" s="1"/>
-      <c r="O30" s="1"/>
-      <c r="P30" s="1"/>
+      <c r="N30" s="1">
+        <v>3</v>
+      </c>
+      <c r="O30" s="1">
+        <v>4</v>
+      </c>
+      <c r="P30" s="1">
+        <v>0</v>
+      </c>
       <c r="Q30" s="1"/>
       <c r="R30" s="1"/>
       <c r="S30" s="1"/>
@@ -6094,17 +6595,17 @@
         <v>22</v>
       </c>
     </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A31" s="11">
         <v>29</v>
       </c>
-      <c r="B31" s="29" t="s">
+      <c r="B31" s="25" t="s">
         <v>247</v>
       </c>
-      <c r="C31" s="29" t="s">
+      <c r="C31" s="25" t="s">
         <v>248</v>
       </c>
-      <c r="D31" s="29" t="s">
+      <c r="D31" s="25" t="s">
         <v>139</v>
       </c>
       <c r="E31" s="13">
@@ -6134,9 +6635,15 @@
       <c r="M31" s="1">
         <v>1</v>
       </c>
-      <c r="N31" s="1"/>
-      <c r="O31" s="1"/>
-      <c r="P31" s="1"/>
+      <c r="N31" s="1">
+        <v>3</v>
+      </c>
+      <c r="O31" s="1">
+        <v>5</v>
+      </c>
+      <c r="P31" s="1">
+        <v>4</v>
+      </c>
       <c r="Q31" s="1"/>
       <c r="R31" s="1"/>
       <c r="S31" s="1"/>
@@ -6144,17 +6651,17 @@
         <v>25</v>
       </c>
     </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A32" s="11">
         <v>30</v>
       </c>
-      <c r="B32" s="29" t="s">
+      <c r="B32" s="25" t="s">
         <v>249</v>
       </c>
-      <c r="C32" s="29" t="s">
+      <c r="C32" s="25" t="s">
         <v>250</v>
       </c>
-      <c r="D32" s="29" t="s">
+      <c r="D32" s="25" t="s">
         <v>251</v>
       </c>
       <c r="E32" s="13">
@@ -6184,9 +6691,15 @@
       <c r="M32" s="1">
         <v>2</v>
       </c>
-      <c r="N32" s="1"/>
-      <c r="O32" s="1"/>
-      <c r="P32" s="1"/>
+      <c r="N32" s="1">
+        <v>1</v>
+      </c>
+      <c r="O32" s="1">
+        <v>1</v>
+      </c>
+      <c r="P32" s="1">
+        <v>3</v>
+      </c>
       <c r="Q32" s="1"/>
       <c r="R32" s="1"/>
       <c r="S32" s="1"/>
@@ -6194,17 +6707,17 @@
         <v>34</v>
       </c>
     </row>
-    <row r="33" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A33" s="11">
         <v>31</v>
       </c>
-      <c r="B33" s="29" t="s">
+      <c r="B33" s="25" t="s">
         <v>252</v>
       </c>
-      <c r="C33" s="29" t="s">
+      <c r="C33" s="25" t="s">
         <v>253</v>
       </c>
-      <c r="D33" s="29" t="s">
+      <c r="D33" s="25" t="s">
         <v>254</v>
       </c>
       <c r="E33" s="13">
@@ -6234,9 +6747,15 @@
       <c r="M33" s="1">
         <v>0</v>
       </c>
-      <c r="N33" s="1"/>
-      <c r="O33" s="1"/>
-      <c r="P33" s="1"/>
+      <c r="N33" s="1">
+        <v>1</v>
+      </c>
+      <c r="O33" s="1">
+        <v>0</v>
+      </c>
+      <c r="P33" s="1">
+        <v>2</v>
+      </c>
       <c r="Q33" s="1"/>
       <c r="R33" s="1"/>
       <c r="S33" s="1"/>
@@ -6244,17 +6763,17 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A34" s="11">
         <v>32</v>
       </c>
-      <c r="B34" s="29" t="s">
+      <c r="B34" s="25" t="s">
         <v>252</v>
       </c>
-      <c r="C34" s="29" t="s">
+      <c r="C34" s="25" t="s">
         <v>60</v>
       </c>
-      <c r="D34" s="29" t="s">
+      <c r="D34" s="25" t="s">
         <v>197</v>
       </c>
       <c r="E34" s="13">
@@ -6284,9 +6803,15 @@
       <c r="M34" s="1">
         <v>0</v>
       </c>
-      <c r="N34" s="1"/>
-      <c r="O34" s="1"/>
-      <c r="P34" s="1"/>
+      <c r="N34" s="1">
+        <v>0</v>
+      </c>
+      <c r="O34" s="1">
+        <v>0</v>
+      </c>
+      <c r="P34" s="1">
+        <v>0</v>
+      </c>
       <c r="Q34" s="1"/>
       <c r="R34" s="1"/>
       <c r="S34" s="1"/>
@@ -6294,17 +6819,17 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A35" s="11">
         <v>33</v>
       </c>
-      <c r="B35" s="29" t="s">
+      <c r="B35" s="25" t="s">
         <v>255</v>
       </c>
-      <c r="C35" s="29" t="s">
+      <c r="C35" s="25" t="s">
         <v>256</v>
       </c>
-      <c r="D35" s="29" t="s">
+      <c r="D35" s="25" t="s">
         <v>257</v>
       </c>
       <c r="E35" s="13">
@@ -6334,9 +6859,15 @@
       <c r="M35" s="1">
         <v>3</v>
       </c>
-      <c r="N35" s="1"/>
-      <c r="O35" s="1"/>
-      <c r="P35" s="1"/>
+      <c r="N35" s="1">
+        <v>3</v>
+      </c>
+      <c r="O35" s="1">
+        <v>3</v>
+      </c>
+      <c r="P35" s="1">
+        <v>3</v>
+      </c>
       <c r="Q35" s="1"/>
       <c r="R35" s="1"/>
       <c r="S35" s="1"/>
@@ -6344,17 +6875,17 @@
         <v>32</v>
       </c>
     </row>
-    <row r="36" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A36" s="11">
         <v>34</v>
       </c>
-      <c r="B36" s="29" t="s">
+      <c r="B36" s="25" t="s">
         <v>258</v>
       </c>
-      <c r="C36" s="29" t="s">
+      <c r="C36" s="25" t="s">
         <v>259</v>
       </c>
-      <c r="D36" s="29" t="s">
+      <c r="D36" s="25" t="s">
         <v>260</v>
       </c>
       <c r="E36" s="13">
@@ -6384,9 +6915,15 @@
       <c r="M36" s="1">
         <v>1</v>
       </c>
-      <c r="N36" s="1"/>
-      <c r="O36" s="1"/>
-      <c r="P36" s="1"/>
+      <c r="N36" s="1">
+        <v>4</v>
+      </c>
+      <c r="O36" s="1">
+        <v>4</v>
+      </c>
+      <c r="P36" s="1">
+        <v>2</v>
+      </c>
       <c r="Q36" s="1"/>
       <c r="R36" s="1"/>
       <c r="S36" s="1"/>
@@ -6394,17 +6931,17 @@
         <v>24</v>
       </c>
     </row>
-    <row r="37" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A37" s="11">
         <v>35</v>
       </c>
-      <c r="B37" s="29" t="s">
+      <c r="B37" s="25" t="s">
         <v>261</v>
       </c>
-      <c r="C37" s="29" t="s">
+      <c r="C37" s="25" t="s">
         <v>212</v>
       </c>
-      <c r="D37" s="29" t="s">
+      <c r="D37" s="25" t="s">
         <v>262</v>
       </c>
       <c r="E37" s="13">
@@ -6434,9 +6971,15 @@
       <c r="M37" s="1">
         <v>3</v>
       </c>
-      <c r="N37" s="1"/>
-      <c r="O37" s="1"/>
-      <c r="P37" s="1"/>
+      <c r="N37" s="1">
+        <v>2</v>
+      </c>
+      <c r="O37" s="1">
+        <v>4</v>
+      </c>
+      <c r="P37" s="1">
+        <v>0</v>
+      </c>
       <c r="Q37" s="1"/>
       <c r="R37" s="1"/>
       <c r="S37" s="1"/>
@@ -6444,17 +6987,17 @@
         <v>34</v>
       </c>
     </row>
-    <row r="38" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A38" s="11">
         <v>36</v>
       </c>
-      <c r="B38" s="29" t="s">
+      <c r="B38" s="25" t="s">
         <v>218</v>
       </c>
-      <c r="C38" s="29" t="s">
+      <c r="C38" s="25" t="s">
         <v>263</v>
       </c>
-      <c r="D38" s="29" t="s">
+      <c r="D38" s="25" t="s">
         <v>264</v>
       </c>
       <c r="E38" s="13">
@@ -6484,9 +7027,15 @@
       <c r="M38" s="1">
         <v>3</v>
       </c>
-      <c r="N38" s="1"/>
-      <c r="O38" s="1"/>
-      <c r="P38" s="1"/>
+      <c r="N38" s="1">
+        <v>4</v>
+      </c>
+      <c r="O38" s="1">
+        <v>2</v>
+      </c>
+      <c r="P38" s="1">
+        <v>3</v>
+      </c>
       <c r="Q38" s="1"/>
       <c r="R38" s="1"/>
       <c r="S38" s="1"/>
@@ -6494,17 +7043,17 @@
         <v>30</v>
       </c>
     </row>
-    <row r="39" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A39" s="11">
         <v>37</v>
       </c>
-      <c r="B39" s="29" t="s">
+      <c r="B39" s="25" t="s">
         <v>265</v>
       </c>
-      <c r="C39" s="29" t="s">
+      <c r="C39" s="25" t="s">
         <v>266</v>
       </c>
-      <c r="D39" s="29" t="s">
+      <c r="D39" s="25" t="s">
         <v>267</v>
       </c>
       <c r="E39" s="13">
@@ -6534,9 +7083,15 @@
       <c r="M39" s="1">
         <v>1</v>
       </c>
-      <c r="N39" s="1"/>
-      <c r="O39" s="1"/>
-      <c r="P39" s="1"/>
+      <c r="N39" s="1">
+        <v>2</v>
+      </c>
+      <c r="O39" s="1">
+        <v>4</v>
+      </c>
+      <c r="P39" s="1">
+        <v>1</v>
+      </c>
       <c r="Q39" s="1"/>
       <c r="R39" s="1"/>
       <c r="S39" s="1"/>
@@ -6544,17 +7099,17 @@
         <v>26</v>
       </c>
     </row>
-    <row r="40" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A40" s="11">
         <v>38</v>
       </c>
-      <c r="B40" s="29" t="s">
+      <c r="B40" s="25" t="s">
         <v>268</v>
       </c>
-      <c r="C40" s="29" t="s">
+      <c r="C40" s="25" t="s">
         <v>72</v>
       </c>
-      <c r="D40" s="29" t="s">
+      <c r="D40" s="25" t="s">
         <v>269</v>
       </c>
       <c r="E40" s="13">
@@ -6584,9 +7139,15 @@
       <c r="M40" s="1">
         <v>1</v>
       </c>
-      <c r="N40" s="1"/>
-      <c r="O40" s="1"/>
-      <c r="P40" s="1"/>
+      <c r="N40" s="1">
+        <v>0</v>
+      </c>
+      <c r="O40" s="1">
+        <v>0</v>
+      </c>
+      <c r="P40" s="1">
+        <v>0</v>
+      </c>
       <c r="Q40" s="1"/>
       <c r="R40" s="1"/>
       <c r="S40" s="1"/>
@@ -6594,17 +7155,17 @@
         <v>13</v>
       </c>
     </row>
-    <row r="41" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A41" s="11">
         <v>39</v>
       </c>
-      <c r="B41" s="29" t="s">
+      <c r="B41" s="25" t="s">
         <v>270</v>
       </c>
-      <c r="C41" s="29" t="s">
+      <c r="C41" s="25" t="s">
         <v>271</v>
       </c>
-      <c r="D41" s="29" t="s">
+      <c r="D41" s="25" t="s">
         <v>272</v>
       </c>
       <c r="E41" s="13">
@@ -6634,9 +7195,15 @@
       <c r="M41" s="1">
         <v>0</v>
       </c>
-      <c r="N41" s="1"/>
-      <c r="O41" s="1"/>
-      <c r="P41" s="1"/>
+      <c r="N41" s="1">
+        <v>0</v>
+      </c>
+      <c r="O41" s="1">
+        <v>0</v>
+      </c>
+      <c r="P41" s="1">
+        <v>0</v>
+      </c>
       <c r="Q41" s="1"/>
       <c r="R41" s="1"/>
       <c r="S41" s="1"/>
@@ -6644,17 +7211,17 @@
         <v>11</v>
       </c>
     </row>
-    <row r="42" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A42" s="11">
         <v>40</v>
       </c>
-      <c r="B42" s="29" t="s">
+      <c r="B42" s="25" t="s">
         <v>273</v>
       </c>
-      <c r="C42" s="29" t="s">
+      <c r="C42" s="25" t="s">
         <v>274</v>
       </c>
-      <c r="D42" s="29" t="s">
+      <c r="D42" s="25" t="s">
         <v>275</v>
       </c>
       <c r="E42" s="13">
@@ -6684,9 +7251,15 @@
       <c r="M42" s="1">
         <v>1</v>
       </c>
-      <c r="N42" s="1"/>
-      <c r="O42" s="1"/>
-      <c r="P42" s="1"/>
+      <c r="N42" s="1">
+        <v>1</v>
+      </c>
+      <c r="O42" s="1">
+        <v>3</v>
+      </c>
+      <c r="P42" s="1">
+        <v>2</v>
+      </c>
       <c r="Q42" s="1"/>
       <c r="R42" s="1"/>
       <c r="S42" s="1"/>
@@ -6694,17 +7267,17 @@
         <v>27</v>
       </c>
     </row>
-    <row r="43" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A43" s="11">
         <v>41</v>
       </c>
-      <c r="B43" s="29" t="s">
+      <c r="B43" s="25" t="s">
         <v>276</v>
       </c>
-      <c r="C43" s="29" t="s">
+      <c r="C43" s="25" t="s">
         <v>82</v>
       </c>
-      <c r="D43" s="29" t="s">
+      <c r="D43" s="25" t="s">
         <v>277</v>
       </c>
       <c r="E43" s="13">
@@ -6734,9 +7307,15 @@
       <c r="M43" s="1">
         <v>3</v>
       </c>
-      <c r="N43" s="1"/>
-      <c r="O43" s="1"/>
-      <c r="P43" s="1"/>
+      <c r="N43" s="1">
+        <v>5</v>
+      </c>
+      <c r="O43" s="1">
+        <v>4</v>
+      </c>
+      <c r="P43" s="1">
+        <v>3</v>
+      </c>
       <c r="Q43" s="1"/>
       <c r="R43" s="1"/>
       <c r="S43" s="1"/>
@@ -6744,17 +7323,17 @@
         <v>30</v>
       </c>
     </row>
-    <row r="44" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A44" s="11">
         <v>42</v>
       </c>
-      <c r="B44" s="29" t="s">
+      <c r="B44" s="25" t="s">
         <v>194</v>
       </c>
-      <c r="C44" s="29" t="s">
+      <c r="C44" s="25" t="s">
         <v>278</v>
       </c>
-      <c r="D44" s="29" t="s">
+      <c r="D44" s="25" t="s">
         <v>279</v>
       </c>
       <c r="E44" s="13">
@@ -6784,9 +7363,15 @@
       <c r="M44" s="1">
         <v>0</v>
       </c>
-      <c r="N44" s="1"/>
-      <c r="O44" s="1"/>
-      <c r="P44" s="1"/>
+      <c r="N44" s="1">
+        <v>0</v>
+      </c>
+      <c r="O44" s="1">
+        <v>0</v>
+      </c>
+      <c r="P44" s="1">
+        <v>0</v>
+      </c>
       <c r="Q44" s="1"/>
       <c r="R44" s="1"/>
       <c r="S44" s="1"/>
@@ -6794,17 +7379,17 @@
         <v>3</v>
       </c>
     </row>
-    <row r="45" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A45" s="11">
         <v>43</v>
       </c>
-      <c r="B45" s="29" t="s">
+      <c r="B45" s="25" t="s">
         <v>194</v>
       </c>
-      <c r="C45" s="29" t="s">
+      <c r="C45" s="25" t="s">
         <v>147</v>
       </c>
-      <c r="D45" s="29" t="s">
+      <c r="D45" s="25" t="s">
         <v>280</v>
       </c>
       <c r="E45" s="13">
@@ -6834,9 +7419,15 @@
       <c r="M45" s="1">
         <v>1</v>
       </c>
-      <c r="N45" s="1"/>
-      <c r="O45" s="1"/>
-      <c r="P45" s="1"/>
+      <c r="N45" s="1">
+        <v>1</v>
+      </c>
+      <c r="O45" s="1">
+        <v>2</v>
+      </c>
+      <c r="P45" s="1">
+        <v>1</v>
+      </c>
       <c r="Q45" s="1"/>
       <c r="R45" s="1"/>
       <c r="S45" s="1"/>
@@ -6844,17 +7435,17 @@
         <v>28</v>
       </c>
     </row>
-    <row r="46" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A46" s="11">
         <v>44</v>
       </c>
-      <c r="B46" s="29" t="s">
+      <c r="B46" s="25" t="s">
         <v>281</v>
       </c>
-      <c r="C46" s="29" t="s">
+      <c r="C46" s="25" t="s">
         <v>282</v>
       </c>
-      <c r="D46" s="29" t="s">
+      <c r="D46" s="25" t="s">
         <v>283</v>
       </c>
       <c r="E46" s="13">
@@ -6884,9 +7475,15 @@
       <c r="M46" s="1">
         <v>1</v>
       </c>
-      <c r="N46" s="1"/>
-      <c r="O46" s="1"/>
-      <c r="P46" s="1"/>
+      <c r="N46" s="1">
+        <v>5</v>
+      </c>
+      <c r="O46" s="1">
+        <v>0</v>
+      </c>
+      <c r="P46" s="1">
+        <v>2</v>
+      </c>
       <c r="Q46" s="1"/>
       <c r="R46" s="1"/>
       <c r="S46" s="1"/>
@@ -6894,17 +7491,17 @@
         <v>29</v>
       </c>
     </row>
-    <row r="47" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A47" s="11">
         <v>45</v>
       </c>
-      <c r="B47" s="29" t="s">
+      <c r="B47" s="25" t="s">
         <v>250</v>
       </c>
-      <c r="C47" s="29" t="s">
+      <c r="C47" s="25" t="s">
         <v>142</v>
       </c>
-      <c r="D47" s="29" t="s">
+      <c r="D47" s="25" t="s">
         <v>284</v>
       </c>
       <c r="E47" s="13">
@@ -6934,9 +7531,15 @@
       <c r="M47" s="1">
         <v>1</v>
       </c>
-      <c r="N47" s="1"/>
-      <c r="O47" s="1"/>
-      <c r="P47" s="1"/>
+      <c r="N47" s="1">
+        <v>4</v>
+      </c>
+      <c r="O47" s="1">
+        <v>3</v>
+      </c>
+      <c r="P47" s="1">
+        <v>2</v>
+      </c>
       <c r="Q47" s="1"/>
       <c r="R47" s="1"/>
       <c r="S47" s="1"/>
@@ -6944,17 +7547,17 @@
         <v>29</v>
       </c>
     </row>
-    <row r="48" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A48" s="11">
         <v>46</v>
       </c>
-      <c r="B48" s="29" t="s">
+      <c r="B48" s="25" t="s">
         <v>285</v>
       </c>
-      <c r="C48" s="29" t="s">
+      <c r="C48" s="25" t="s">
         <v>286</v>
       </c>
-      <c r="D48" s="29" t="s">
+      <c r="D48" s="25" t="s">
         <v>287</v>
       </c>
       <c r="E48" s="13">
@@ -6984,9 +7587,15 @@
       <c r="M48" s="1">
         <v>0</v>
       </c>
-      <c r="N48" s="1"/>
-      <c r="O48" s="1"/>
-      <c r="P48" s="1"/>
+      <c r="N48" s="1">
+        <v>1</v>
+      </c>
+      <c r="O48" s="1">
+        <v>4</v>
+      </c>
+      <c r="P48" s="1">
+        <v>4</v>
+      </c>
       <c r="Q48" s="1"/>
       <c r="R48" s="1"/>
       <c r="S48" s="1"/>
@@ -6994,17 +7603,17 @@
         <v>29</v>
       </c>
     </row>
-    <row r="49" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A49" s="11">
         <v>47</v>
       </c>
-      <c r="B49" s="29" t="s">
+      <c r="B49" s="25" t="s">
         <v>288</v>
       </c>
-      <c r="C49" s="29" t="s">
+      <c r="C49" s="25" t="s">
         <v>289</v>
       </c>
-      <c r="D49" s="29" t="s">
+      <c r="D49" s="25" t="s">
         <v>290</v>
       </c>
       <c r="E49" s="13">
@@ -7034,9 +7643,15 @@
       <c r="M49" s="1">
         <v>2</v>
       </c>
-      <c r="N49" s="1"/>
-      <c r="O49" s="1"/>
-      <c r="P49" s="1"/>
+      <c r="N49" s="1">
+        <v>3</v>
+      </c>
+      <c r="O49" s="1">
+        <v>0</v>
+      </c>
+      <c r="P49" s="1">
+        <v>3</v>
+      </c>
       <c r="Q49" s="1"/>
       <c r="R49" s="1"/>
       <c r="S49" s="1"/>
@@ -7044,17 +7659,17 @@
         <v>2</v>
       </c>
     </row>
-    <row r="50" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A50" s="11">
         <v>48</v>
       </c>
-      <c r="B50" s="29" t="s">
+      <c r="B50" s="25" t="s">
         <v>291</v>
       </c>
-      <c r="C50" s="29" t="s">
+      <c r="C50" s="25" t="s">
         <v>292</v>
       </c>
-      <c r="D50" s="29" t="s">
+      <c r="D50" s="25" t="s">
         <v>59</v>
       </c>
       <c r="E50" s="13">
@@ -7084,9 +7699,15 @@
       <c r="M50" s="1">
         <v>2</v>
       </c>
-      <c r="N50" s="1"/>
-      <c r="O50" s="1"/>
-      <c r="P50" s="1"/>
+      <c r="N50" s="1">
+        <v>3</v>
+      </c>
+      <c r="O50" s="1">
+        <v>5</v>
+      </c>
+      <c r="P50" s="1">
+        <v>3</v>
+      </c>
       <c r="Q50" s="1"/>
       <c r="R50" s="1"/>
       <c r="S50" s="1"/>
@@ -7094,52 +7715,58 @@
         <v>28</v>
       </c>
     </row>
-    <row r="51" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="31">
+    <row r="51" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A51" s="27">
         <v>49</v>
       </c>
-      <c r="B51" s="32" t="s">
+      <c r="B51" s="28" t="s">
         <v>293</v>
       </c>
-      <c r="C51" s="32" t="s">
+      <c r="C51" s="28" t="s">
         <v>294</v>
       </c>
-      <c r="D51" s="33" t="s">
+      <c r="D51" s="29" t="s">
         <v>295</v>
       </c>
-      <c r="E51" s="34">
+      <c r="E51" s="30">
         <v>23645903</v>
       </c>
-      <c r="F51" s="35">
-        <v>5</v>
-      </c>
-      <c r="G51" s="35">
-        <v>5</v>
-      </c>
-      <c r="H51" s="35">
-        <v>5</v>
-      </c>
-      <c r="I51" s="35">
-        <v>4</v>
-      </c>
-      <c r="J51" s="35">
-        <v>4</v>
-      </c>
-      <c r="K51" s="35">
-        <v>3</v>
-      </c>
-      <c r="L51" s="35">
-        <v>5</v>
-      </c>
-      <c r="M51" s="35">
-        <v>3</v>
-      </c>
-      <c r="N51" s="35"/>
-      <c r="O51" s="35"/>
-      <c r="P51" s="35"/>
-      <c r="Q51" s="35"/>
-      <c r="R51" s="35"/>
-      <c r="S51" s="35"/>
+      <c r="F51" s="23">
+        <v>5</v>
+      </c>
+      <c r="G51" s="23">
+        <v>5</v>
+      </c>
+      <c r="H51" s="23">
+        <v>5</v>
+      </c>
+      <c r="I51" s="23">
+        <v>4</v>
+      </c>
+      <c r="J51" s="23">
+        <v>4</v>
+      </c>
+      <c r="K51" s="23">
+        <v>3</v>
+      </c>
+      <c r="L51" s="23">
+        <v>5</v>
+      </c>
+      <c r="M51" s="23">
+        <v>3</v>
+      </c>
+      <c r="N51" s="23">
+        <v>2</v>
+      </c>
+      <c r="O51" s="23">
+        <v>3</v>
+      </c>
+      <c r="P51" s="23">
+        <v>3</v>
+      </c>
+      <c r="Q51" s="23"/>
+      <c r="R51" s="23"/>
+      <c r="S51" s="23"/>
       <c r="T51" s="10">
         <v>34</v>
       </c>
@@ -7157,7 +7784,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E8177AD-01C8-476C-943E-ED9E51CF18DE}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Update Excel + Add horizontal scroll to charts for many controls
</commit_message>
<xml_diff>
--- a/data/reporte.xlsx
+++ b/data/reporte.xlsx
@@ -8,14 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre\OneDrive\Escritorio\Universidad\2026-1\Modelos de Procesos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEB94EDD-3F34-45D3-A944-D6BB47B04270}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C6601AA-7D2D-4B12-9D5B-A3DBCA659876}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EF01AC27-D1AA-450D-80FE-C50ADE1636E7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sección 1" sheetId="1" r:id="rId1"/>
     <sheet name="Sección 2" sheetId="2" r:id="rId2"/>
-    <sheet name="Reporte" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -932,7 +931,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -966,6 +965,14 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -1323,7 +1330,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1392,6 +1399,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1904,11 +1912,14 @@
       <c r="P3" s="9">
         <v>3</v>
       </c>
-      <c r="Q3" s="9"/>
+      <c r="Q3" s="9">
+        <v>5</v>
+      </c>
       <c r="R3" s="9"/>
       <c r="S3" s="9"/>
       <c r="T3" s="10">
-        <v>22</v>
+        <f>($F3+$G3+$H3+$I3+$J3+$K3+$L3+$M3+$N3+$O3+$P3+$Q3)</f>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.3">
@@ -1960,11 +1971,14 @@
       <c r="P4" s="1">
         <v>1</v>
       </c>
-      <c r="Q4" s="1"/>
+      <c r="Q4" s="1">
+        <v>5</v>
+      </c>
       <c r="R4" s="1"/>
       <c r="S4" s="1"/>
       <c r="T4" s="10">
-        <v>20</v>
+        <f t="shared" ref="T4:T57" si="0">($F4+$G4+$H4+$I4+$J4+$K4+$L4+$M4+$N4+$O4+$P4+$Q4)</f>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.3">
@@ -2016,11 +2030,14 @@
       <c r="P5" s="1">
         <v>1</v>
       </c>
-      <c r="Q5" s="1"/>
+      <c r="Q5" s="1">
+        <v>4</v>
+      </c>
       <c r="R5" s="1"/>
       <c r="S5" s="1"/>
       <c r="T5" s="10">
-        <v>19</v>
+        <f t="shared" si="0"/>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.3">
@@ -2072,11 +2089,14 @@
       <c r="P6" s="1">
         <v>1</v>
       </c>
-      <c r="Q6" s="1"/>
+      <c r="Q6" s="1">
+        <v>5</v>
+      </c>
       <c r="R6" s="1"/>
       <c r="S6" s="1"/>
       <c r="T6" s="10">
-        <v>28</v>
+        <f t="shared" si="0"/>
+        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.3">
@@ -2128,11 +2148,14 @@
       <c r="P7" s="1">
         <v>2</v>
       </c>
-      <c r="Q7" s="1"/>
+      <c r="Q7" s="1">
+        <v>0</v>
+      </c>
       <c r="R7" s="1"/>
       <c r="S7" s="1"/>
       <c r="T7" s="10">
-        <v>27</v>
+        <f t="shared" si="0"/>
+        <v>34</v>
       </c>
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.3">
@@ -2184,11 +2207,14 @@
       <c r="P8" s="1">
         <v>4</v>
       </c>
-      <c r="Q8" s="1"/>
+      <c r="Q8" s="1">
+        <v>5</v>
+      </c>
       <c r="R8" s="1"/>
       <c r="S8" s="1"/>
       <c r="T8" s="10">
-        <v>36</v>
+        <f t="shared" si="0"/>
+        <v>55</v>
       </c>
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.3">
@@ -2240,11 +2266,14 @@
       <c r="P9" s="1">
         <v>2</v>
       </c>
-      <c r="Q9" s="1"/>
+      <c r="Q9" s="1">
+        <v>0</v>
+      </c>
       <c r="R9" s="1"/>
       <c r="S9" s="1"/>
       <c r="T9" s="10">
-        <v>26</v>
+        <f t="shared" si="0"/>
+        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.3">
@@ -2296,11 +2325,14 @@
       <c r="P10" s="1">
         <v>2</v>
       </c>
-      <c r="Q10" s="1"/>
+      <c r="Q10" s="1">
+        <v>5</v>
+      </c>
       <c r="R10" s="1"/>
       <c r="S10" s="1"/>
       <c r="T10" s="10">
-        <v>17</v>
+        <f t="shared" si="0"/>
+        <v>26</v>
       </c>
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.3">
@@ -2352,11 +2384,14 @@
       <c r="P11" s="1">
         <v>3</v>
       </c>
-      <c r="Q11" s="1"/>
+      <c r="Q11" s="1">
+        <v>4</v>
+      </c>
       <c r="R11" s="1"/>
       <c r="S11" s="1"/>
       <c r="T11" s="10">
-        <v>33</v>
+        <f t="shared" si="0"/>
+        <v>48</v>
       </c>
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.3">
@@ -2408,11 +2443,14 @@
       <c r="P12" s="1">
         <v>3</v>
       </c>
-      <c r="Q12" s="1"/>
+      <c r="Q12" s="1">
+        <v>5</v>
+      </c>
       <c r="R12" s="1"/>
       <c r="S12" s="1"/>
       <c r="T12" s="10">
-        <v>29</v>
+        <f t="shared" si="0"/>
+        <v>44</v>
       </c>
     </row>
     <row r="13" spans="1:20" x14ac:dyDescent="0.3">
@@ -2464,11 +2502,14 @@
       <c r="P13" s="1">
         <v>3</v>
       </c>
-      <c r="Q13" s="1"/>
+      <c r="Q13" s="1">
+        <v>0</v>
+      </c>
       <c r="R13" s="1"/>
       <c r="S13" s="1"/>
       <c r="T13" s="10">
-        <v>17</v>
+        <f>($F13+$G13+$H13+$I13+$J13+$K13+$L13+$M13+$N13+$O13+$P13+$Q13)</f>
+        <v>23</v>
       </c>
     </row>
     <row r="14" spans="1:20" x14ac:dyDescent="0.3">
@@ -2520,11 +2561,14 @@
       <c r="P14" s="1">
         <v>3</v>
       </c>
-      <c r="Q14" s="1"/>
+      <c r="Q14" s="1">
+        <v>5</v>
+      </c>
       <c r="R14" s="1"/>
       <c r="S14" s="1"/>
       <c r="T14" s="10">
-        <v>19</v>
+        <f t="shared" si="0"/>
+        <v>29</v>
       </c>
     </row>
     <row r="15" spans="1:20" x14ac:dyDescent="0.3">
@@ -2576,11 +2620,14 @@
       <c r="P15" s="1">
         <v>0</v>
       </c>
-      <c r="Q15" s="1"/>
+      <c r="Q15" s="1">
+        <v>5</v>
+      </c>
       <c r="R15" s="1"/>
       <c r="S15" s="1"/>
       <c r="T15" s="10">
-        <v>26</v>
+        <f t="shared" si="0"/>
+        <v>37</v>
       </c>
     </row>
     <row r="16" spans="1:20" x14ac:dyDescent="0.3">
@@ -2632,11 +2679,14 @@
       <c r="P16" s="1">
         <v>2</v>
       </c>
-      <c r="Q16" s="1"/>
+      <c r="Q16" s="1">
+        <v>5</v>
+      </c>
       <c r="R16" s="1"/>
       <c r="S16" s="1"/>
       <c r="T16" s="10">
-        <v>23</v>
+        <f t="shared" si="0"/>
+        <v>34</v>
       </c>
     </row>
     <row r="17" spans="1:20" x14ac:dyDescent="0.3">
@@ -2688,11 +2738,14 @@
       <c r="P17" s="1">
         <v>1</v>
       </c>
-      <c r="Q17" s="1"/>
+      <c r="Q17" s="1">
+        <v>5</v>
+      </c>
       <c r="R17" s="1"/>
       <c r="S17" s="1"/>
       <c r="T17" s="10">
-        <v>22</v>
+        <f t="shared" si="0"/>
+        <v>32</v>
       </c>
     </row>
     <row r="18" spans="1:20" x14ac:dyDescent="0.3">
@@ -2744,11 +2797,14 @@
       <c r="P18" s="1">
         <v>4</v>
       </c>
-      <c r="Q18" s="1"/>
+      <c r="Q18" s="1">
+        <v>5</v>
+      </c>
       <c r="R18" s="1"/>
       <c r="S18" s="1"/>
       <c r="T18" s="10">
-        <v>29</v>
+        <f t="shared" si="0"/>
+        <v>44</v>
       </c>
     </row>
     <row r="19" spans="1:20" x14ac:dyDescent="0.3">
@@ -2800,11 +2856,14 @@
       <c r="P19" s="1">
         <v>4</v>
       </c>
-      <c r="Q19" s="1"/>
+      <c r="Q19" s="1">
+        <v>5</v>
+      </c>
       <c r="R19" s="1"/>
       <c r="S19" s="1"/>
       <c r="T19" s="10">
-        <v>19</v>
+        <f t="shared" si="0"/>
+        <v>29</v>
       </c>
     </row>
     <row r="20" spans="1:20" x14ac:dyDescent="0.3">
@@ -2856,11 +2915,14 @@
       <c r="P20" s="1">
         <v>3</v>
       </c>
-      <c r="Q20" s="1"/>
+      <c r="Q20" s="1">
+        <v>5</v>
+      </c>
       <c r="R20" s="1"/>
       <c r="S20" s="1"/>
       <c r="T20" s="10">
-        <v>27</v>
+        <f t="shared" si="0"/>
+        <v>41</v>
       </c>
     </row>
     <row r="21" spans="1:20" x14ac:dyDescent="0.3">
@@ -2912,11 +2974,14 @@
       <c r="P21" s="1">
         <v>2</v>
       </c>
-      <c r="Q21" s="1"/>
+      <c r="Q21" s="1">
+        <v>3</v>
+      </c>
       <c r="R21" s="1"/>
       <c r="S21" s="1"/>
       <c r="T21" s="10">
-        <v>26</v>
+        <f t="shared" si="0"/>
+        <v>34</v>
       </c>
     </row>
     <row r="22" spans="1:20" x14ac:dyDescent="0.3">
@@ -2968,11 +3033,14 @@
       <c r="P22" s="1">
         <v>4</v>
       </c>
-      <c r="Q22" s="1"/>
+      <c r="Q22" s="1">
+        <v>4</v>
+      </c>
       <c r="R22" s="1"/>
       <c r="S22" s="1"/>
       <c r="T22" s="10">
-        <v>34</v>
+        <f t="shared" si="0"/>
+        <v>46</v>
       </c>
     </row>
     <row r="23" spans="1:20" x14ac:dyDescent="0.3">
@@ -3024,11 +3092,14 @@
       <c r="P23" s="1">
         <v>0</v>
       </c>
-      <c r="Q23" s="1"/>
+      <c r="Q23" s="1">
+        <v>5</v>
+      </c>
       <c r="R23" s="1"/>
       <c r="S23" s="1"/>
       <c r="T23" s="10">
-        <v>33</v>
+        <f t="shared" si="0"/>
+        <v>38</v>
       </c>
     </row>
     <row r="24" spans="1:20" x14ac:dyDescent="0.3">
@@ -3080,11 +3151,14 @@
       <c r="P24" s="1">
         <v>0</v>
       </c>
-      <c r="Q24" s="1"/>
+      <c r="Q24" s="1">
+        <v>0</v>
+      </c>
       <c r="R24" s="1"/>
       <c r="S24" s="1"/>
       <c r="T24" s="10">
-        <v>18</v>
+        <f t="shared" si="0"/>
+        <v>19</v>
       </c>
     </row>
     <row r="25" spans="1:20" x14ac:dyDescent="0.3">
@@ -3136,11 +3210,14 @@
       <c r="P25" s="1">
         <v>0</v>
       </c>
-      <c r="Q25" s="1"/>
+      <c r="Q25" s="1">
+        <v>5</v>
+      </c>
       <c r="R25" s="1"/>
       <c r="S25" s="1"/>
       <c r="T25" s="10">
-        <v>15</v>
+        <f t="shared" si="0"/>
+        <v>26</v>
       </c>
     </row>
     <row r="26" spans="1:20" x14ac:dyDescent="0.3">
@@ -3192,11 +3269,14 @@
       <c r="P26" s="1">
         <v>2</v>
       </c>
-      <c r="Q26" s="1"/>
+      <c r="Q26" s="1">
+        <v>5</v>
+      </c>
       <c r="R26" s="1"/>
       <c r="S26" s="1"/>
       <c r="T26" s="10">
-        <v>12</v>
+        <f t="shared" si="0"/>
+        <v>20</v>
       </c>
     </row>
     <row r="27" spans="1:20" x14ac:dyDescent="0.3">
@@ -3248,11 +3328,14 @@
       <c r="P27" s="1">
         <v>3</v>
       </c>
-      <c r="Q27" s="1"/>
+      <c r="Q27" s="1">
+        <v>5</v>
+      </c>
       <c r="R27" s="1"/>
       <c r="S27" s="1"/>
       <c r="T27" s="10">
-        <v>27</v>
+        <f t="shared" si="0"/>
+        <v>38</v>
       </c>
     </row>
     <row r="28" spans="1:20" x14ac:dyDescent="0.3">
@@ -3304,11 +3387,14 @@
       <c r="P28" s="1">
         <v>1</v>
       </c>
-      <c r="Q28" s="1"/>
+      <c r="Q28" s="1">
+        <v>5</v>
+      </c>
       <c r="R28" s="1"/>
       <c r="S28" s="1"/>
       <c r="T28" s="10">
-        <v>29</v>
+        <f t="shared" si="0"/>
+        <v>36</v>
       </c>
     </row>
     <row r="29" spans="1:20" x14ac:dyDescent="0.3">
@@ -3360,11 +3446,14 @@
       <c r="P29" s="1">
         <v>5</v>
       </c>
-      <c r="Q29" s="1"/>
+      <c r="Q29" s="1">
+        <v>5</v>
+      </c>
       <c r="R29" s="1"/>
       <c r="S29" s="1"/>
       <c r="T29" s="10">
-        <v>30</v>
+        <f t="shared" si="0"/>
+        <v>48</v>
       </c>
     </row>
     <row r="30" spans="1:20" x14ac:dyDescent="0.3">
@@ -3416,10 +3505,13 @@
       <c r="P30" s="1">
         <v>0</v>
       </c>
-      <c r="Q30" s="1"/>
+      <c r="Q30" s="1">
+        <v>0</v>
+      </c>
       <c r="R30" s="1"/>
       <c r="S30" s="1"/>
       <c r="T30" s="10">
+        <f t="shared" si="0"/>
         <v>14</v>
       </c>
     </row>
@@ -3472,11 +3564,14 @@
       <c r="P31" s="1">
         <v>2</v>
       </c>
-      <c r="Q31" s="1"/>
+      <c r="Q31" s="1">
+        <v>5</v>
+      </c>
       <c r="R31" s="1"/>
       <c r="S31" s="1"/>
       <c r="T31" s="10">
-        <v>27</v>
+        <f t="shared" si="0"/>
+        <v>38</v>
       </c>
     </row>
     <row r="32" spans="1:20" x14ac:dyDescent="0.3">
@@ -3528,11 +3623,14 @@
       <c r="P32" s="1">
         <v>3</v>
       </c>
-      <c r="Q32" s="1"/>
+      <c r="Q32" s="1">
+        <v>0</v>
+      </c>
       <c r="R32" s="1"/>
       <c r="S32" s="1"/>
       <c r="T32" s="10">
-        <v>28</v>
+        <f t="shared" si="0"/>
+        <v>34</v>
       </c>
     </row>
     <row r="33" spans="1:20" x14ac:dyDescent="0.3">
@@ -3584,11 +3682,14 @@
       <c r="P33" s="1">
         <v>4</v>
       </c>
-      <c r="Q33" s="1"/>
+      <c r="Q33" s="1">
+        <v>5</v>
+      </c>
       <c r="R33" s="1"/>
       <c r="S33" s="1"/>
       <c r="T33" s="10">
-        <v>33</v>
+        <f t="shared" si="0"/>
+        <v>50</v>
       </c>
     </row>
     <row r="34" spans="1:20" x14ac:dyDescent="0.3">
@@ -3640,11 +3741,14 @@
       <c r="P34" s="1">
         <v>5</v>
       </c>
-      <c r="Q34" s="1"/>
+      <c r="Q34" s="1">
+        <v>5</v>
+      </c>
       <c r="R34" s="1"/>
       <c r="S34" s="1"/>
       <c r="T34" s="10">
-        <v>28</v>
+        <f t="shared" si="0"/>
+        <v>45</v>
       </c>
     </row>
     <row r="35" spans="1:20" x14ac:dyDescent="0.3">
@@ -3696,11 +3800,14 @@
       <c r="P35" s="1">
         <v>4</v>
       </c>
-      <c r="Q35" s="1"/>
+      <c r="Q35" s="1">
+        <v>5</v>
+      </c>
       <c r="R35" s="1"/>
       <c r="S35" s="1"/>
       <c r="T35" s="10">
-        <v>23</v>
+        <f t="shared" si="0"/>
+        <v>39</v>
       </c>
     </row>
     <row r="36" spans="1:20" x14ac:dyDescent="0.3">
@@ -3752,11 +3859,14 @@
       <c r="P36" s="1">
         <v>3</v>
       </c>
-      <c r="Q36" s="1"/>
+      <c r="Q36" s="1">
+        <v>5</v>
+      </c>
       <c r="R36" s="1"/>
       <c r="S36" s="1"/>
       <c r="T36" s="10">
-        <v>28</v>
+        <f t="shared" si="0"/>
+        <v>36</v>
       </c>
     </row>
     <row r="37" spans="1:20" x14ac:dyDescent="0.3">
@@ -3808,11 +3918,14 @@
       <c r="P37" s="1">
         <v>2</v>
       </c>
-      <c r="Q37" s="1"/>
+      <c r="Q37" s="1">
+        <v>5</v>
+      </c>
       <c r="R37" s="1"/>
       <c r="S37" s="1"/>
       <c r="T37" s="10">
-        <v>23</v>
+        <f t="shared" si="0"/>
+        <v>32</v>
       </c>
     </row>
     <row r="38" spans="1:20" x14ac:dyDescent="0.3">
@@ -3864,10 +3977,13 @@
       <c r="P38" s="1">
         <v>0</v>
       </c>
-      <c r="Q38" s="1"/>
+      <c r="Q38" s="1">
+        <v>0</v>
+      </c>
       <c r="R38" s="1"/>
       <c r="S38" s="1"/>
       <c r="T38" s="10">
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
     </row>
@@ -3920,11 +4036,14 @@
       <c r="P39" s="1">
         <v>4</v>
       </c>
-      <c r="Q39" s="1"/>
+      <c r="Q39" s="1">
+        <v>5</v>
+      </c>
       <c r="R39" s="1"/>
       <c r="S39" s="1"/>
       <c r="T39" s="10">
-        <v>35</v>
+        <f t="shared" si="0"/>
+        <v>50</v>
       </c>
     </row>
     <row r="40" spans="1:20" x14ac:dyDescent="0.3">
@@ -3976,11 +4095,14 @@
       <c r="P40" s="1">
         <v>2</v>
       </c>
-      <c r="Q40" s="1"/>
+      <c r="Q40" s="1">
+        <v>0</v>
+      </c>
       <c r="R40" s="1"/>
       <c r="S40" s="1"/>
       <c r="T40" s="10">
-        <v>19</v>
+        <f t="shared" si="0"/>
+        <v>23</v>
       </c>
     </row>
     <row r="41" spans="1:20" x14ac:dyDescent="0.3">
@@ -4032,11 +4154,14 @@
       <c r="P41" s="1">
         <v>1</v>
       </c>
-      <c r="Q41" s="1"/>
+      <c r="Q41" s="1">
+        <v>3</v>
+      </c>
       <c r="R41" s="1"/>
       <c r="S41" s="1"/>
       <c r="T41" s="10">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>4</v>
       </c>
     </row>
     <row r="42" spans="1:20" x14ac:dyDescent="0.3">
@@ -4088,11 +4213,14 @@
       <c r="P42" s="1">
         <v>3</v>
       </c>
-      <c r="Q42" s="1"/>
+      <c r="Q42" s="1">
+        <v>5</v>
+      </c>
       <c r="R42" s="1"/>
       <c r="S42" s="1"/>
       <c r="T42" s="10">
-        <v>4</v>
+        <f t="shared" si="0"/>
+        <v>17</v>
       </c>
     </row>
     <row r="43" spans="1:20" x14ac:dyDescent="0.3">
@@ -4144,11 +4272,14 @@
       <c r="P43" s="1">
         <v>4</v>
       </c>
-      <c r="Q43" s="1"/>
+      <c r="Q43" s="1">
+        <v>5</v>
+      </c>
       <c r="R43" s="1"/>
       <c r="S43" s="1"/>
       <c r="T43" s="10">
-        <v>20</v>
+        <f t="shared" si="0"/>
+        <v>39</v>
       </c>
     </row>
     <row r="44" spans="1:20" x14ac:dyDescent="0.3">
@@ -4200,11 +4331,14 @@
       <c r="P44" s="1">
         <v>3</v>
       </c>
-      <c r="Q44" s="1"/>
+      <c r="Q44" s="1">
+        <v>5</v>
+      </c>
       <c r="R44" s="1"/>
       <c r="S44" s="1"/>
       <c r="T44" s="10">
-        <v>18</v>
+        <f t="shared" si="0"/>
+        <v>27</v>
       </c>
     </row>
     <row r="45" spans="1:20" x14ac:dyDescent="0.3">
@@ -4256,11 +4390,14 @@
       <c r="P45" s="1">
         <v>2</v>
       </c>
-      <c r="Q45" s="1"/>
+      <c r="Q45" s="1">
+        <v>5</v>
+      </c>
       <c r="R45" s="1"/>
       <c r="S45" s="1"/>
       <c r="T45" s="10">
-        <v>20</v>
+        <f t="shared" si="0"/>
+        <v>33</v>
       </c>
     </row>
     <row r="46" spans="1:20" x14ac:dyDescent="0.3">
@@ -4312,11 +4449,14 @@
       <c r="P46" s="1">
         <v>1</v>
       </c>
-      <c r="Q46" s="1"/>
+      <c r="Q46" s="1">
+        <v>5</v>
+      </c>
       <c r="R46" s="1"/>
       <c r="S46" s="1"/>
       <c r="T46" s="10">
-        <v>29</v>
+        <f t="shared" si="0"/>
+        <v>42</v>
       </c>
     </row>
     <row r="47" spans="1:20" x14ac:dyDescent="0.3">
@@ -4368,11 +4508,14 @@
       <c r="P47" s="1">
         <v>5</v>
       </c>
-      <c r="Q47" s="1"/>
+      <c r="Q47" s="1">
+        <v>5</v>
+      </c>
       <c r="R47" s="1"/>
       <c r="S47" s="1"/>
       <c r="T47" s="10">
-        <v>24</v>
+        <f t="shared" si="0"/>
+        <v>43</v>
       </c>
     </row>
     <row r="48" spans="1:20" x14ac:dyDescent="0.3">
@@ -4424,11 +4567,14 @@
       <c r="P48" s="1">
         <v>2</v>
       </c>
-      <c r="Q48" s="1"/>
+      <c r="Q48" s="1">
+        <v>5</v>
+      </c>
       <c r="R48" s="1"/>
       <c r="S48" s="1"/>
       <c r="T48" s="10">
-        <v>35</v>
+        <f t="shared" si="0"/>
+        <v>49</v>
       </c>
     </row>
     <row r="49" spans="1:20" x14ac:dyDescent="0.3">
@@ -4480,11 +4626,14 @@
       <c r="P49" s="1">
         <v>1</v>
       </c>
-      <c r="Q49" s="1"/>
+      <c r="Q49" s="1">
+        <v>5</v>
+      </c>
       <c r="R49" s="1"/>
       <c r="S49" s="1"/>
       <c r="T49" s="10">
-        <v>29</v>
+        <f t="shared" si="0"/>
+        <v>41</v>
       </c>
     </row>
     <row r="50" spans="1:20" x14ac:dyDescent="0.3">
@@ -4536,11 +4685,14 @@
       <c r="P50" s="1">
         <v>2</v>
       </c>
-      <c r="Q50" s="1"/>
+      <c r="Q50" s="1">
+        <v>5</v>
+      </c>
       <c r="R50" s="1"/>
       <c r="S50" s="1"/>
       <c r="T50" s="10">
-        <v>34</v>
+        <f t="shared" si="0"/>
+        <v>46</v>
       </c>
     </row>
     <row r="51" spans="1:20" x14ac:dyDescent="0.3">
@@ -4592,11 +4744,14 @@
       <c r="P51" s="1">
         <v>1</v>
       </c>
-      <c r="Q51" s="1"/>
+      <c r="Q51" s="1">
+        <v>3</v>
+      </c>
       <c r="R51" s="1"/>
       <c r="S51" s="1"/>
       <c r="T51" s="10">
-        <v>16</v>
+        <f t="shared" si="0"/>
+        <v>26</v>
       </c>
     </row>
     <row r="52" spans="1:20" x14ac:dyDescent="0.3">
@@ -4648,11 +4803,14 @@
       <c r="P52" s="1">
         <v>1</v>
       </c>
-      <c r="Q52" s="1"/>
+      <c r="Q52" s="1">
+        <v>5</v>
+      </c>
       <c r="R52" s="1"/>
       <c r="S52" s="1"/>
       <c r="T52" s="10">
-        <v>26</v>
+        <f t="shared" si="0"/>
+        <v>34</v>
       </c>
     </row>
     <row r="53" spans="1:20" x14ac:dyDescent="0.3">
@@ -4704,11 +4862,14 @@
       <c r="P53" s="1">
         <v>3</v>
       </c>
-      <c r="Q53" s="1"/>
+      <c r="Q53" s="1">
+        <v>5</v>
+      </c>
       <c r="R53" s="1"/>
       <c r="S53" s="1"/>
       <c r="T53" s="10">
-        <v>35</v>
+        <f t="shared" si="0"/>
+        <v>47</v>
       </c>
     </row>
     <row r="54" spans="1:20" x14ac:dyDescent="0.3">
@@ -4760,11 +4921,14 @@
       <c r="P54" s="1">
         <v>4</v>
       </c>
-      <c r="Q54" s="1"/>
+      <c r="Q54" s="1">
+        <v>5</v>
+      </c>
       <c r="R54" s="1"/>
       <c r="S54" s="1"/>
       <c r="T54" s="10">
-        <v>34</v>
+        <f t="shared" si="0"/>
+        <v>51</v>
       </c>
     </row>
     <row r="55" spans="1:20" x14ac:dyDescent="0.3">
@@ -4816,11 +4980,14 @@
       <c r="P55" s="1">
         <v>4</v>
       </c>
-      <c r="Q55" s="1"/>
+      <c r="Q55" s="1">
+        <v>4</v>
+      </c>
       <c r="R55" s="1"/>
       <c r="S55" s="1"/>
       <c r="T55" s="10">
-        <v>37</v>
+        <f t="shared" si="0"/>
+        <v>53</v>
       </c>
     </row>
     <row r="56" spans="1:20" x14ac:dyDescent="0.3">
@@ -4872,11 +5039,14 @@
       <c r="P56" s="1">
         <v>2</v>
       </c>
-      <c r="Q56" s="1"/>
+      <c r="Q56" s="1">
+        <v>5</v>
+      </c>
       <c r="R56" s="1"/>
       <c r="S56" s="1"/>
       <c r="T56" s="10">
-        <v>34</v>
+        <f t="shared" si="0"/>
+        <v>48</v>
       </c>
     </row>
     <row r="57" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -4928,11 +5098,14 @@
       <c r="P57" s="22">
         <v>5</v>
       </c>
-      <c r="Q57" s="22"/>
+      <c r="Q57" s="22">
+        <v>5</v>
+      </c>
       <c r="R57" s="22"/>
       <c r="S57" s="22"/>
       <c r="T57" s="10">
-        <v>32</v>
+        <f t="shared" si="0"/>
+        <v>49</v>
       </c>
     </row>
     <row r="58" spans="1:20" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
@@ -4948,7 +5121,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7CD6AE0E-6B38-4517-9EE7-74576DF1F95D}">
-  <dimension ref="A1:T51"/>
+  <dimension ref="A1:T64"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.3">
@@ -5076,11 +5249,14 @@
       <c r="P3" s="1">
         <v>3</v>
       </c>
-      <c r="Q3" s="1"/>
+      <c r="Q3" s="1">
+        <v>0</v>
+      </c>
       <c r="R3" s="1"/>
       <c r="S3" s="1"/>
       <c r="T3" s="10">
-        <v>29</v>
+        <f>($F3+$G3+$H3+$I3+$J3+$K3+$L3+$M3+$N3+$O3+$P3+$Q3)</f>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.3">
@@ -5132,11 +5308,14 @@
       <c r="P4" s="1">
         <v>1</v>
       </c>
-      <c r="Q4" s="1"/>
+      <c r="Q4" s="1">
+        <v>5</v>
+      </c>
       <c r="R4" s="1"/>
       <c r="S4" s="1"/>
       <c r="T4" s="10">
-        <v>18</v>
+        <f t="shared" ref="T4:T51" si="0">($F4+$G4+$H4+$I4+$J4+$K4+$L4+$M4+$N4+$O4+$P4+$Q4)</f>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.3">
@@ -5188,10 +5367,13 @@
       <c r="P5" s="1">
         <v>0</v>
       </c>
-      <c r="Q5" s="1"/>
+      <c r="Q5" s="1">
+        <v>0</v>
+      </c>
       <c r="R5" s="1"/>
       <c r="S5" s="1"/>
       <c r="T5" s="10">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -5244,11 +5426,14 @@
       <c r="P6" s="1">
         <v>1</v>
       </c>
-      <c r="Q6" s="1"/>
+      <c r="Q6" s="1">
+        <v>0</v>
+      </c>
       <c r="R6" s="1"/>
       <c r="S6" s="1"/>
       <c r="T6" s="10">
-        <v>28</v>
+        <f t="shared" si="0"/>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.3">
@@ -5300,11 +5485,14 @@
       <c r="P7" s="1">
         <v>3</v>
       </c>
-      <c r="Q7" s="1"/>
+      <c r="Q7" s="1">
+        <v>5</v>
+      </c>
       <c r="R7" s="1"/>
       <c r="S7" s="1"/>
       <c r="T7" s="10">
-        <v>33</v>
+        <f t="shared" si="0"/>
+        <v>47</v>
       </c>
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.3">
@@ -5356,11 +5544,14 @@
       <c r="P8" s="1">
         <v>2</v>
       </c>
-      <c r="Q8" s="1"/>
+      <c r="Q8" s="1">
+        <v>5</v>
+      </c>
       <c r="R8" s="1"/>
       <c r="S8" s="1"/>
       <c r="T8" s="10">
-        <v>5</v>
+        <f t="shared" si="0"/>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.3">
@@ -5412,11 +5603,14 @@
       <c r="P9" s="1">
         <v>2</v>
       </c>
-      <c r="Q9" s="1"/>
+      <c r="Q9" s="1">
+        <v>5</v>
+      </c>
       <c r="R9" s="1"/>
       <c r="S9" s="1"/>
       <c r="T9" s="10">
-        <v>33</v>
+        <f t="shared" si="0"/>
+        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.3">
@@ -5468,11 +5662,14 @@
       <c r="P10" s="1">
         <v>3</v>
       </c>
-      <c r="Q10" s="1"/>
+      <c r="Q10" s="1">
+        <v>5</v>
+      </c>
       <c r="R10" s="1"/>
       <c r="S10" s="1"/>
       <c r="T10" s="10">
-        <v>3</v>
+        <f t="shared" si="0"/>
+        <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.3">
@@ -5524,11 +5721,14 @@
       <c r="P11" s="1">
         <v>1</v>
       </c>
-      <c r="Q11" s="1"/>
+      <c r="Q11" s="1">
+        <v>0</v>
+      </c>
       <c r="R11" s="1"/>
       <c r="S11" s="1"/>
       <c r="T11" s="10">
-        <v>30</v>
+        <f t="shared" si="0"/>
+        <v>31</v>
       </c>
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.3">
@@ -5580,11 +5780,14 @@
       <c r="P12" s="1">
         <v>3</v>
       </c>
-      <c r="Q12" s="1"/>
+      <c r="Q12" s="1">
+        <v>5</v>
+      </c>
       <c r="R12" s="1"/>
       <c r="S12" s="1"/>
       <c r="T12" s="10">
-        <v>32</v>
+        <f t="shared" si="0"/>
+        <v>45</v>
       </c>
     </row>
     <row r="13" spans="1:20" x14ac:dyDescent="0.3">
@@ -5636,11 +5839,14 @@
       <c r="P13" s="1">
         <v>4</v>
       </c>
-      <c r="Q13" s="1"/>
+      <c r="Q13" s="1">
+        <v>5</v>
+      </c>
       <c r="R13" s="1"/>
       <c r="S13" s="1"/>
       <c r="T13" s="10">
-        <v>35</v>
+        <f t="shared" si="0"/>
+        <v>53</v>
       </c>
     </row>
     <row r="14" spans="1:20" x14ac:dyDescent="0.3">
@@ -5692,11 +5898,14 @@
       <c r="P14" s="1">
         <v>2</v>
       </c>
-      <c r="Q14" s="1"/>
+      <c r="Q14" s="1">
+        <v>0</v>
+      </c>
       <c r="R14" s="1"/>
       <c r="S14" s="1"/>
       <c r="T14" s="10">
-        <v>21</v>
+        <f t="shared" si="0"/>
+        <v>26</v>
       </c>
     </row>
     <row r="15" spans="1:20" x14ac:dyDescent="0.3">
@@ -5748,11 +5957,14 @@
       <c r="P15" s="1">
         <v>3</v>
       </c>
-      <c r="Q15" s="1"/>
+      <c r="Q15" s="1">
+        <v>5</v>
+      </c>
       <c r="R15" s="1"/>
       <c r="S15" s="1"/>
       <c r="T15" s="10">
-        <v>3</v>
+        <f t="shared" si="0"/>
+        <v>16</v>
       </c>
     </row>
     <row r="16" spans="1:20" x14ac:dyDescent="0.3">
@@ -5804,11 +6016,14 @@
       <c r="P16" s="1">
         <v>2</v>
       </c>
-      <c r="Q16" s="1"/>
+      <c r="Q16" s="1">
+        <v>5</v>
+      </c>
       <c r="R16" s="1"/>
       <c r="S16" s="1"/>
       <c r="T16" s="10">
-        <v>21</v>
+        <f t="shared" si="0"/>
+        <v>33</v>
       </c>
     </row>
     <row r="17" spans="1:20" x14ac:dyDescent="0.3">
@@ -5860,11 +6075,14 @@
       <c r="P17" s="1">
         <v>1</v>
       </c>
-      <c r="Q17" s="1"/>
+      <c r="Q17" s="1">
+        <v>5</v>
+      </c>
       <c r="R17" s="1"/>
       <c r="S17" s="1"/>
       <c r="T17" s="10">
-        <v>27</v>
+        <f t="shared" si="0"/>
+        <v>35</v>
       </c>
     </row>
     <row r="18" spans="1:20" x14ac:dyDescent="0.3">
@@ -5916,11 +6134,14 @@
       <c r="P18" s="1">
         <v>1</v>
       </c>
-      <c r="Q18" s="1"/>
+      <c r="Q18" s="1">
+        <v>5</v>
+      </c>
       <c r="R18" s="1"/>
       <c r="S18" s="1"/>
       <c r="T18" s="10">
-        <v>30</v>
+        <f t="shared" si="0"/>
+        <v>41</v>
       </c>
     </row>
     <row r="19" spans="1:20" x14ac:dyDescent="0.3">
@@ -5972,11 +6193,14 @@
       <c r="P19" s="1">
         <v>0</v>
       </c>
-      <c r="Q19" s="1"/>
+      <c r="Q19" s="1">
+        <v>5</v>
+      </c>
       <c r="R19" s="1"/>
       <c r="S19" s="1"/>
       <c r="T19" s="10">
-        <v>12</v>
+        <f t="shared" si="0"/>
+        <v>17</v>
       </c>
     </row>
     <row r="20" spans="1:20" x14ac:dyDescent="0.3">
@@ -6028,11 +6252,14 @@
       <c r="P20" s="1">
         <v>2</v>
       </c>
-      <c r="Q20" s="1"/>
+      <c r="Q20" s="1">
+        <v>5</v>
+      </c>
       <c r="R20" s="1"/>
       <c r="S20" s="1"/>
       <c r="T20" s="10">
-        <v>28</v>
+        <f t="shared" si="0"/>
+        <v>41</v>
       </c>
     </row>
     <row r="21" spans="1:20" x14ac:dyDescent="0.3">
@@ -6084,11 +6311,14 @@
       <c r="P21" s="1">
         <v>4</v>
       </c>
-      <c r="Q21" s="1"/>
+      <c r="Q21" s="1">
+        <v>5</v>
+      </c>
       <c r="R21" s="1"/>
       <c r="S21" s="1"/>
       <c r="T21" s="10">
-        <v>26</v>
+        <f t="shared" si="0"/>
+        <v>40</v>
       </c>
     </row>
     <row r="22" spans="1:20" x14ac:dyDescent="0.3">
@@ -6140,11 +6370,14 @@
       <c r="P22" s="1">
         <v>3</v>
       </c>
-      <c r="Q22" s="1"/>
+      <c r="Q22" s="1">
+        <v>5</v>
+      </c>
       <c r="R22" s="1"/>
       <c r="S22" s="1"/>
       <c r="T22" s="10">
-        <v>30</v>
+        <f t="shared" si="0"/>
+        <v>46</v>
       </c>
     </row>
     <row r="23" spans="1:20" x14ac:dyDescent="0.3">
@@ -6196,11 +6429,14 @@
       <c r="P23" s="1">
         <v>0</v>
       </c>
-      <c r="Q23" s="1"/>
+      <c r="Q23" s="1">
+        <v>5</v>
+      </c>
       <c r="R23" s="1"/>
       <c r="S23" s="1"/>
       <c r="T23" s="10">
-        <v>22</v>
+        <f t="shared" si="0"/>
+        <v>30</v>
       </c>
     </row>
     <row r="24" spans="1:20" x14ac:dyDescent="0.3">
@@ -6252,11 +6488,14 @@
       <c r="P24" s="1">
         <v>2</v>
       </c>
-      <c r="Q24" s="1"/>
+      <c r="Q24" s="1">
+        <v>5</v>
+      </c>
       <c r="R24" s="1"/>
       <c r="S24" s="1"/>
       <c r="T24" s="10">
-        <v>18</v>
+        <f t="shared" si="0"/>
+        <v>32</v>
       </c>
     </row>
     <row r="25" spans="1:20" x14ac:dyDescent="0.3">
@@ -6308,10 +6547,13 @@
       <c r="P25" s="1">
         <v>0</v>
       </c>
-      <c r="Q25" s="1"/>
+      <c r="Q25" s="1">
+        <v>0</v>
+      </c>
       <c r="R25" s="1"/>
       <c r="S25" s="1"/>
       <c r="T25" s="10">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -6364,11 +6606,14 @@
       <c r="P26" s="1">
         <v>0</v>
       </c>
-      <c r="Q26" s="1"/>
+      <c r="Q26" s="1">
+        <v>5</v>
+      </c>
       <c r="R26" s="1"/>
       <c r="S26" s="1"/>
       <c r="T26" s="10">
-        <v>32</v>
+        <f t="shared" si="0"/>
+        <v>37</v>
       </c>
     </row>
     <row r="27" spans="1:20" x14ac:dyDescent="0.3">
@@ -6420,11 +6665,14 @@
       <c r="P27" s="1">
         <v>3</v>
       </c>
-      <c r="Q27" s="1"/>
+      <c r="Q27" s="1">
+        <v>5</v>
+      </c>
       <c r="R27" s="1"/>
       <c r="S27" s="1"/>
       <c r="T27" s="10">
-        <v>34</v>
+        <f t="shared" si="0"/>
+        <v>47</v>
       </c>
     </row>
     <row r="28" spans="1:20" x14ac:dyDescent="0.3">
@@ -6476,11 +6724,14 @@
       <c r="P28" s="1">
         <v>3</v>
       </c>
-      <c r="Q28" s="1"/>
+      <c r="Q28" s="1">
+        <v>5</v>
+      </c>
       <c r="R28" s="1"/>
       <c r="S28" s="1"/>
       <c r="T28" s="10">
-        <v>34</v>
+        <f t="shared" si="0"/>
+        <v>49</v>
       </c>
     </row>
     <row r="29" spans="1:20" x14ac:dyDescent="0.3">
@@ -6532,10 +6783,13 @@
       <c r="P29" s="1">
         <v>0</v>
       </c>
-      <c r="Q29" s="1"/>
+      <c r="Q29" s="1">
+        <v>0</v>
+      </c>
       <c r="R29" s="1"/>
       <c r="S29" s="1"/>
       <c r="T29" s="10">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -6588,11 +6842,14 @@
       <c r="P30" s="1">
         <v>0</v>
       </c>
-      <c r="Q30" s="1"/>
+      <c r="Q30" s="1">
+        <v>5</v>
+      </c>
       <c r="R30" s="1"/>
       <c r="S30" s="1"/>
       <c r="T30" s="10">
-        <v>22</v>
+        <f t="shared" si="0"/>
+        <v>34</v>
       </c>
     </row>
     <row r="31" spans="1:20" x14ac:dyDescent="0.3">
@@ -6644,11 +6901,14 @@
       <c r="P31" s="1">
         <v>4</v>
       </c>
-      <c r="Q31" s="1"/>
+      <c r="Q31" s="1">
+        <v>5</v>
+      </c>
       <c r="R31" s="1"/>
       <c r="S31" s="1"/>
       <c r="T31" s="10">
-        <v>25</v>
+        <f t="shared" si="0"/>
+        <v>42</v>
       </c>
     </row>
     <row r="32" spans="1:20" x14ac:dyDescent="0.3">
@@ -6700,11 +6960,14 @@
       <c r="P32" s="1">
         <v>3</v>
       </c>
-      <c r="Q32" s="1"/>
+      <c r="Q32" s="1">
+        <v>4</v>
+      </c>
       <c r="R32" s="1"/>
       <c r="S32" s="1"/>
       <c r="T32" s="10">
-        <v>34</v>
+        <f t="shared" si="0"/>
+        <v>43</v>
       </c>
     </row>
     <row r="33" spans="1:20" x14ac:dyDescent="0.3">
@@ -6756,11 +7019,14 @@
       <c r="P33" s="1">
         <v>2</v>
       </c>
-      <c r="Q33" s="1"/>
+      <c r="Q33" s="1">
+        <v>0</v>
+      </c>
       <c r="R33" s="1"/>
       <c r="S33" s="1"/>
       <c r="T33" s="10">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>3</v>
       </c>
     </row>
     <row r="34" spans="1:20" x14ac:dyDescent="0.3">
@@ -6812,11 +7078,14 @@
       <c r="P34" s="1">
         <v>0</v>
       </c>
-      <c r="Q34" s="1"/>
+      <c r="Q34" s="1">
+        <v>5</v>
+      </c>
       <c r="R34" s="1"/>
       <c r="S34" s="1"/>
       <c r="T34" s="10">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>5</v>
       </c>
     </row>
     <row r="35" spans="1:20" x14ac:dyDescent="0.3">
@@ -6868,11 +7137,14 @@
       <c r="P35" s="1">
         <v>3</v>
       </c>
-      <c r="Q35" s="1"/>
+      <c r="Q35" s="1">
+        <v>4</v>
+      </c>
       <c r="R35" s="1"/>
       <c r="S35" s="1"/>
       <c r="T35" s="10">
-        <v>32</v>
+        <f t="shared" si="0"/>
+        <v>45</v>
       </c>
     </row>
     <row r="36" spans="1:20" x14ac:dyDescent="0.3">
@@ -6924,11 +7196,14 @@
       <c r="P36" s="1">
         <v>2</v>
       </c>
-      <c r="Q36" s="1"/>
+      <c r="Q36" s="1">
+        <v>0</v>
+      </c>
       <c r="R36" s="1"/>
       <c r="S36" s="1"/>
       <c r="T36" s="10">
-        <v>24</v>
+        <f t="shared" si="0"/>
+        <v>34</v>
       </c>
     </row>
     <row r="37" spans="1:20" x14ac:dyDescent="0.3">
@@ -6980,11 +7255,14 @@
       <c r="P37" s="1">
         <v>0</v>
       </c>
-      <c r="Q37" s="1"/>
+      <c r="Q37" s="1">
+        <v>5</v>
+      </c>
       <c r="R37" s="1"/>
       <c r="S37" s="1"/>
       <c r="T37" s="10">
-        <v>34</v>
+        <f t="shared" si="0"/>
+        <v>45</v>
       </c>
     </row>
     <row r="38" spans="1:20" x14ac:dyDescent="0.3">
@@ -7036,11 +7314,14 @@
       <c r="P38" s="1">
         <v>3</v>
       </c>
-      <c r="Q38" s="1"/>
+      <c r="Q38" s="1">
+        <v>5</v>
+      </c>
       <c r="R38" s="1"/>
       <c r="S38" s="1"/>
       <c r="T38" s="10">
-        <v>30</v>
+        <f t="shared" si="0"/>
+        <v>44</v>
       </c>
     </row>
     <row r="39" spans="1:20" x14ac:dyDescent="0.3">
@@ -7092,11 +7373,14 @@
       <c r="P39" s="1">
         <v>1</v>
       </c>
-      <c r="Q39" s="1"/>
+      <c r="Q39" s="1">
+        <v>5</v>
+      </c>
       <c r="R39" s="1"/>
       <c r="S39" s="1"/>
       <c r="T39" s="10">
-        <v>26</v>
+        <f t="shared" si="0"/>
+        <v>38</v>
       </c>
     </row>
     <row r="40" spans="1:20" x14ac:dyDescent="0.3">
@@ -7148,11 +7432,14 @@
       <c r="P40" s="1">
         <v>0</v>
       </c>
-      <c r="Q40" s="1"/>
+      <c r="Q40" s="1">
+        <v>5</v>
+      </c>
       <c r="R40" s="1"/>
       <c r="S40" s="1"/>
       <c r="T40" s="10">
-        <v>13</v>
+        <f t="shared" si="0"/>
+        <v>18</v>
       </c>
     </row>
     <row r="41" spans="1:20" x14ac:dyDescent="0.3">
@@ -7204,10 +7491,13 @@
       <c r="P41" s="1">
         <v>0</v>
       </c>
-      <c r="Q41" s="1"/>
+      <c r="Q41" s="1">
+        <v>0</v>
+      </c>
       <c r="R41" s="1"/>
       <c r="S41" s="1"/>
       <c r="T41" s="10">
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
     </row>
@@ -7260,11 +7550,14 @@
       <c r="P42" s="1">
         <v>2</v>
       </c>
-      <c r="Q42" s="1"/>
+      <c r="Q42" s="1">
+        <v>5</v>
+      </c>
       <c r="R42" s="1"/>
       <c r="S42" s="1"/>
       <c r="T42" s="10">
-        <v>27</v>
+        <f t="shared" si="0"/>
+        <v>38</v>
       </c>
     </row>
     <row r="43" spans="1:20" x14ac:dyDescent="0.3">
@@ -7316,11 +7609,14 @@
       <c r="P43" s="1">
         <v>3</v>
       </c>
-      <c r="Q43" s="1"/>
+      <c r="Q43" s="1">
+        <v>5</v>
+      </c>
       <c r="R43" s="1"/>
       <c r="S43" s="1"/>
       <c r="T43" s="10">
-        <v>30</v>
+        <f t="shared" si="0"/>
+        <v>47</v>
       </c>
     </row>
     <row r="44" spans="1:20" x14ac:dyDescent="0.3">
@@ -7372,11 +7668,14 @@
       <c r="P44" s="1">
         <v>0</v>
       </c>
-      <c r="Q44" s="1"/>
+      <c r="Q44" s="1">
+        <v>5</v>
+      </c>
       <c r="R44" s="1"/>
       <c r="S44" s="1"/>
       <c r="T44" s="10">
-        <v>3</v>
+        <f t="shared" si="0"/>
+        <v>8</v>
       </c>
     </row>
     <row r="45" spans="1:20" x14ac:dyDescent="0.3">
@@ -7428,11 +7727,14 @@
       <c r="P45" s="1">
         <v>1</v>
       </c>
-      <c r="Q45" s="1"/>
+      <c r="Q45" s="1">
+        <v>4</v>
+      </c>
       <c r="R45" s="1"/>
       <c r="S45" s="1"/>
       <c r="T45" s="10">
-        <v>28</v>
+        <f t="shared" si="0"/>
+        <v>36</v>
       </c>
     </row>
     <row r="46" spans="1:20" x14ac:dyDescent="0.3">
@@ -7484,11 +7786,14 @@
       <c r="P46" s="1">
         <v>2</v>
       </c>
-      <c r="Q46" s="1"/>
+      <c r="Q46" s="1">
+        <v>5</v>
+      </c>
       <c r="R46" s="1"/>
       <c r="S46" s="1"/>
       <c r="T46" s="10">
-        <v>29</v>
+        <f t="shared" si="0"/>
+        <v>41</v>
       </c>
     </row>
     <row r="47" spans="1:20" x14ac:dyDescent="0.3">
@@ -7540,11 +7845,14 @@
       <c r="P47" s="1">
         <v>2</v>
       </c>
-      <c r="Q47" s="1"/>
+      <c r="Q47" s="1">
+        <v>5</v>
+      </c>
       <c r="R47" s="1"/>
       <c r="S47" s="1"/>
       <c r="T47" s="10">
-        <v>29</v>
+        <f t="shared" si="0"/>
+        <v>43</v>
       </c>
     </row>
     <row r="48" spans="1:20" x14ac:dyDescent="0.3">
@@ -7596,11 +7904,14 @@
       <c r="P48" s="1">
         <v>4</v>
       </c>
-      <c r="Q48" s="1"/>
+      <c r="Q48" s="1">
+        <v>0</v>
+      </c>
       <c r="R48" s="1"/>
       <c r="S48" s="1"/>
       <c r="T48" s="10">
-        <v>29</v>
+        <f t="shared" si="0"/>
+        <v>38</v>
       </c>
     </row>
     <row r="49" spans="1:20" x14ac:dyDescent="0.3">
@@ -7652,11 +7963,14 @@
       <c r="P49" s="1">
         <v>3</v>
       </c>
-      <c r="Q49" s="1"/>
+      <c r="Q49" s="1">
+        <v>0</v>
+      </c>
       <c r="R49" s="1"/>
       <c r="S49" s="1"/>
       <c r="T49" s="10">
-        <v>2</v>
+        <f t="shared" si="0"/>
+        <v>8</v>
       </c>
     </row>
     <row r="50" spans="1:20" x14ac:dyDescent="0.3">
@@ -7708,11 +8022,14 @@
       <c r="P50" s="1">
         <v>3</v>
       </c>
-      <c r="Q50" s="1"/>
+      <c r="Q50" s="1">
+        <v>0</v>
+      </c>
       <c r="R50" s="1"/>
       <c r="S50" s="1"/>
       <c r="T50" s="10">
-        <v>28</v>
+        <f t="shared" si="0"/>
+        <v>39</v>
       </c>
     </row>
     <row r="51" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7764,12 +8081,18 @@
       <c r="P51" s="23">
         <v>3</v>
       </c>
-      <c r="Q51" s="23"/>
+      <c r="Q51" s="23">
+        <v>5</v>
+      </c>
       <c r="R51" s="23"/>
       <c r="S51" s="23"/>
       <c r="T51" s="10">
-        <v>34</v>
-      </c>
+        <f t="shared" si="0"/>
+        <v>47</v>
+      </c>
+    </row>
+    <row r="64" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R64" s="38"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -7779,13 +8102,4 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E8177AD-01C8-476C-943E-ED9E51CF18DE}">
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
📊 Update Excel with new controls
</commit_message>
<xml_diff>
--- a/data/reporte.xlsx
+++ b/data/reporte.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre\OneDrive\Escritorio\Universidad\2026-1\Modelos de Procesos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C6601AA-7D2D-4B12-9D5B-A3DBCA659876}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F53C1042-21C1-492A-9DFE-83ED05AE77EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EF01AC27-D1AA-450D-80FE-C50ADE1636E7}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="296">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="297">
   <si>
     <t>Puntajes Controles</t>
   </si>
@@ -925,13 +925,16 @@
   </si>
   <si>
     <t>MARTÍN SAMUEL</t>
+  </si>
+  <si>
+    <t>C15</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -974,6 +977,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -1001,7 +1010,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="26">
+  <borders count="27">
     <border>
       <left/>
       <right/>
@@ -1326,11 +1335,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1388,6 +1406,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1399,7 +1418,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1784,36 +1805,37 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FAFB6214-215B-45FB-8876-0D7E2F238F6A}">
-  <dimension ref="A1:T58"/>
+  <dimension ref="A1:U58"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A1" s="33"/>
-      <c r="B1" s="33"/>
+    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A1" s="34"/>
+      <c r="B1" s="34"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
-      <c r="F1" s="34" t="s">
-        <v>0</v>
-      </c>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
-      <c r="I1" s="35"/>
-      <c r="J1" s="35"/>
-      <c r="K1" s="35"/>
-      <c r="L1" s="35"/>
-      <c r="M1" s="35"/>
-      <c r="N1" s="35"/>
-      <c r="O1" s="35"/>
-      <c r="P1" s="35"/>
-      <c r="Q1" s="35"/>
-      <c r="R1" s="35"/>
-      <c r="S1" s="36"/>
-      <c r="T1" s="2"/>
-    </row>
-    <row r="2" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="37"/>
-      <c r="B2" s="37"/>
+      <c r="F1" s="35" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1" s="36"/>
+      <c r="H1" s="36"/>
+      <c r="I1" s="36"/>
+      <c r="J1" s="36"/>
+      <c r="K1" s="36"/>
+      <c r="L1" s="36"/>
+      <c r="M1" s="36"/>
+      <c r="N1" s="36"/>
+      <c r="O1" s="36"/>
+      <c r="P1" s="36"/>
+      <c r="Q1" s="36"/>
+      <c r="R1" s="36"/>
+      <c r="S1" s="37"/>
+      <c r="T1" s="39"/>
+      <c r="U1" s="2"/>
+    </row>
+    <row r="2" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="38"/>
+      <c r="B2" s="38"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -1859,11 +1881,14 @@
       <c r="S2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="T2" s="5" t="s">
+      <c r="T2" s="4" t="s">
+        <v>296</v>
+      </c>
+      <c r="U2" s="5" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A3" s="6">
         <v>1</v>
       </c>
@@ -1915,14 +1940,21 @@
       <c r="Q3" s="9">
         <v>5</v>
       </c>
-      <c r="R3" s="9"/>
-      <c r="S3" s="9"/>
-      <c r="T3" s="10">
-        <f>($F3+$G3+$H3+$I3+$J3+$K3+$L3+$M3+$N3+$O3+$P3+$Q3)</f>
-        <v>37</v>
-      </c>
-    </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R3" s="9">
+        <v>0</v>
+      </c>
+      <c r="S3" s="9">
+        <v>4</v>
+      </c>
+      <c r="T3" s="9">
+        <v>5</v>
+      </c>
+      <c r="U3" s="10">
+        <f>($F3+$G3+$H3+$I3+$J3+$K3+$L3+$M3+$N3+$O3+$P3+$Q3+$R3+$S3+$T3)</f>
+        <v>46</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A4" s="11">
         <v>2</v>
       </c>
@@ -1974,14 +2006,21 @@
       <c r="Q4" s="1">
         <v>5</v>
       </c>
-      <c r="R4" s="1"/>
-      <c r="S4" s="1"/>
-      <c r="T4" s="10">
-        <f t="shared" ref="T4:T57" si="0">($F4+$G4+$H4+$I4+$J4+$K4+$L4+$M4+$N4+$O4+$P4+$Q4)</f>
-        <v>26</v>
-      </c>
-    </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R4" s="1">
+        <v>4</v>
+      </c>
+      <c r="S4" s="1">
+        <v>4</v>
+      </c>
+      <c r="T4" s="1">
+        <v>4</v>
+      </c>
+      <c r="U4" s="10">
+        <f t="shared" ref="U4:U57" si="0">($F4+$G4+$H4+$I4+$J4+$K4+$L4+$M4+$N4+$O4+$P4+$Q4+$R4+$S4+$T4)</f>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A5" s="11">
         <v>3</v>
       </c>
@@ -2033,14 +2072,21 @@
       <c r="Q5" s="1">
         <v>4</v>
       </c>
-      <c r="R5" s="1"/>
-      <c r="S5" s="1"/>
-      <c r="T5" s="10">
-        <f t="shared" si="0"/>
-        <v>25</v>
-      </c>
-    </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R5" s="1">
+        <v>0</v>
+      </c>
+      <c r="S5" s="1">
+        <v>4</v>
+      </c>
+      <c r="T5" s="1">
+        <v>2</v>
+      </c>
+      <c r="U5" s="10">
+        <f t="shared" si="0"/>
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A6" s="11">
         <v>4</v>
       </c>
@@ -2092,14 +2138,21 @@
       <c r="Q6" s="1">
         <v>5</v>
       </c>
-      <c r="R6" s="1"/>
-      <c r="S6" s="1"/>
-      <c r="T6" s="10">
-        <f t="shared" si="0"/>
-        <v>38</v>
-      </c>
-    </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R6" s="1">
+        <v>3</v>
+      </c>
+      <c r="S6" s="1">
+        <v>4</v>
+      </c>
+      <c r="T6" s="1">
+        <v>4</v>
+      </c>
+      <c r="U6" s="10">
+        <f t="shared" si="0"/>
+        <v>49</v>
+      </c>
+    </row>
+    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A7" s="11">
         <v>5</v>
       </c>
@@ -2151,14 +2204,21 @@
       <c r="Q7" s="1">
         <v>0</v>
       </c>
-      <c r="R7" s="1"/>
-      <c r="S7" s="1"/>
-      <c r="T7" s="10">
-        <f t="shared" si="0"/>
-        <v>34</v>
-      </c>
-    </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R7" s="1">
+        <v>5</v>
+      </c>
+      <c r="S7" s="1">
+        <v>2</v>
+      </c>
+      <c r="T7" s="1">
+        <v>5</v>
+      </c>
+      <c r="U7" s="10">
+        <f t="shared" si="0"/>
+        <v>46</v>
+      </c>
+    </row>
+    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A8" s="11">
         <v>6</v>
       </c>
@@ -2210,14 +2270,21 @@
       <c r="Q8" s="1">
         <v>5</v>
       </c>
-      <c r="R8" s="1"/>
-      <c r="S8" s="1"/>
-      <c r="T8" s="10">
-        <f t="shared" si="0"/>
-        <v>55</v>
-      </c>
-    </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R8" s="1">
+        <v>5</v>
+      </c>
+      <c r="S8" s="1">
+        <v>5</v>
+      </c>
+      <c r="T8" s="1">
+        <v>3</v>
+      </c>
+      <c r="U8" s="10">
+        <f t="shared" si="0"/>
+        <v>68</v>
+      </c>
+    </row>
+    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A9" s="11">
         <v>7</v>
       </c>
@@ -2269,14 +2336,21 @@
       <c r="Q9" s="1">
         <v>0</v>
       </c>
-      <c r="R9" s="1"/>
-      <c r="S9" s="1"/>
-      <c r="T9" s="10">
-        <f t="shared" si="0"/>
-        <v>32</v>
-      </c>
-    </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R9" s="1">
+        <v>4</v>
+      </c>
+      <c r="S9" s="1">
+        <v>5</v>
+      </c>
+      <c r="T9" s="1">
+        <v>3</v>
+      </c>
+      <c r="U9" s="10">
+        <f t="shared" si="0"/>
+        <v>44</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A10" s="11">
         <v>8</v>
       </c>
@@ -2328,14 +2402,21 @@
       <c r="Q10" s="1">
         <v>5</v>
       </c>
-      <c r="R10" s="1"/>
-      <c r="S10" s="1"/>
-      <c r="T10" s="10">
-        <f t="shared" si="0"/>
-        <v>26</v>
-      </c>
-    </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R10" s="1">
+        <v>4</v>
+      </c>
+      <c r="S10" s="1">
+        <v>0</v>
+      </c>
+      <c r="T10" s="1">
+        <v>0</v>
+      </c>
+      <c r="U10" s="10">
+        <f t="shared" si="0"/>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A11" s="11">
         <v>9</v>
       </c>
@@ -2387,14 +2468,21 @@
       <c r="Q11" s="1">
         <v>4</v>
       </c>
-      <c r="R11" s="1"/>
-      <c r="S11" s="1"/>
-      <c r="T11" s="10">
-        <f t="shared" si="0"/>
-        <v>48</v>
-      </c>
-    </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R11" s="1">
+        <v>1</v>
+      </c>
+      <c r="S11" s="1">
+        <v>3</v>
+      </c>
+      <c r="T11" s="1">
+        <v>3</v>
+      </c>
+      <c r="U11" s="10">
+        <f t="shared" si="0"/>
+        <v>55</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A12" s="11">
         <v>10</v>
       </c>
@@ -2446,14 +2534,21 @@
       <c r="Q12" s="1">
         <v>5</v>
       </c>
-      <c r="R12" s="1"/>
-      <c r="S12" s="1"/>
-      <c r="T12" s="10">
-        <f t="shared" si="0"/>
-        <v>44</v>
-      </c>
-    </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R12" s="1">
+        <v>4</v>
+      </c>
+      <c r="S12" s="1">
+        <v>5</v>
+      </c>
+      <c r="T12" s="1">
+        <v>5</v>
+      </c>
+      <c r="U12" s="10">
+        <f t="shared" si="0"/>
+        <v>58</v>
+      </c>
+    </row>
+    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A13" s="11">
         <v>11</v>
       </c>
@@ -2505,14 +2600,21 @@
       <c r="Q13" s="1">
         <v>0</v>
       </c>
-      <c r="R13" s="1"/>
-      <c r="S13" s="1"/>
-      <c r="T13" s="10">
-        <f>($F13+$G13+$H13+$I13+$J13+$K13+$L13+$M13+$N13+$O13+$P13+$Q13)</f>
-        <v>23</v>
-      </c>
-    </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R13" s="1">
+        <v>4</v>
+      </c>
+      <c r="S13" s="1">
+        <v>4</v>
+      </c>
+      <c r="T13" s="1">
+        <v>4</v>
+      </c>
+      <c r="U13" s="10">
+        <f t="shared" si="0"/>
+        <v>35</v>
+      </c>
+    </row>
+    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A14" s="11">
         <v>12</v>
       </c>
@@ -2564,14 +2666,21 @@
       <c r="Q14" s="1">
         <v>5</v>
       </c>
-      <c r="R14" s="1"/>
-      <c r="S14" s="1"/>
-      <c r="T14" s="10">
-        <f t="shared" si="0"/>
-        <v>29</v>
-      </c>
-    </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R14" s="1">
+        <v>5</v>
+      </c>
+      <c r="S14" s="1">
+        <v>5</v>
+      </c>
+      <c r="T14" s="1">
+        <v>0</v>
+      </c>
+      <c r="U14" s="10">
+        <f t="shared" si="0"/>
+        <v>39</v>
+      </c>
+    </row>
+    <row r="15" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A15" s="11">
         <v>13</v>
       </c>
@@ -2623,14 +2732,21 @@
       <c r="Q15" s="1">
         <v>5</v>
       </c>
-      <c r="R15" s="1"/>
-      <c r="S15" s="1"/>
-      <c r="T15" s="10">
-        <f t="shared" si="0"/>
-        <v>37</v>
-      </c>
-    </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R15" s="1">
+        <v>0</v>
+      </c>
+      <c r="S15" s="1">
+        <v>3</v>
+      </c>
+      <c r="T15" s="1">
+        <v>3</v>
+      </c>
+      <c r="U15" s="10">
+        <f t="shared" si="0"/>
+        <v>43</v>
+      </c>
+    </row>
+    <row r="16" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A16" s="11">
         <v>14</v>
       </c>
@@ -2682,14 +2798,21 @@
       <c r="Q16" s="1">
         <v>5</v>
       </c>
-      <c r="R16" s="1"/>
-      <c r="S16" s="1"/>
-      <c r="T16" s="10">
-        <f t="shared" si="0"/>
-        <v>34</v>
-      </c>
-    </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R16" s="1">
+        <v>4</v>
+      </c>
+      <c r="S16" s="1">
+        <v>5</v>
+      </c>
+      <c r="T16" s="1">
+        <v>0</v>
+      </c>
+      <c r="U16" s="10">
+        <f t="shared" si="0"/>
+        <v>43</v>
+      </c>
+    </row>
+    <row r="17" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A17" s="11">
         <v>15</v>
       </c>
@@ -2741,14 +2864,21 @@
       <c r="Q17" s="1">
         <v>5</v>
       </c>
-      <c r="R17" s="1"/>
-      <c r="S17" s="1"/>
-      <c r="T17" s="10">
-        <f t="shared" si="0"/>
-        <v>32</v>
-      </c>
-    </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R17" s="1">
+        <v>3</v>
+      </c>
+      <c r="S17" s="1">
+        <v>5</v>
+      </c>
+      <c r="T17" s="1">
+        <v>0</v>
+      </c>
+      <c r="U17" s="10">
+        <f t="shared" si="0"/>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="18" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A18" s="11">
         <v>16</v>
       </c>
@@ -2800,14 +2930,21 @@
       <c r="Q18" s="1">
         <v>5</v>
       </c>
-      <c r="R18" s="1"/>
-      <c r="S18" s="1"/>
-      <c r="T18" s="10">
-        <f t="shared" si="0"/>
-        <v>44</v>
-      </c>
-    </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R18" s="1">
+        <v>1</v>
+      </c>
+      <c r="S18" s="1">
+        <v>1</v>
+      </c>
+      <c r="T18" s="1">
+        <v>0</v>
+      </c>
+      <c r="U18" s="10">
+        <f t="shared" si="0"/>
+        <v>46</v>
+      </c>
+    </row>
+    <row r="19" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A19" s="11">
         <v>17</v>
       </c>
@@ -2859,14 +2996,21 @@
       <c r="Q19" s="1">
         <v>5</v>
       </c>
-      <c r="R19" s="1"/>
-      <c r="S19" s="1"/>
-      <c r="T19" s="10">
-        <f t="shared" si="0"/>
-        <v>29</v>
-      </c>
-    </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R19" s="1">
+        <v>3</v>
+      </c>
+      <c r="S19" s="1">
+        <v>4</v>
+      </c>
+      <c r="T19" s="1">
+        <v>3</v>
+      </c>
+      <c r="U19" s="10">
+        <f t="shared" si="0"/>
+        <v>39</v>
+      </c>
+    </row>
+    <row r="20" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A20" s="11">
         <v>18</v>
       </c>
@@ -2918,14 +3062,21 @@
       <c r="Q20" s="1">
         <v>5</v>
       </c>
-      <c r="R20" s="1"/>
-      <c r="S20" s="1"/>
-      <c r="T20" s="10">
-        <f t="shared" si="0"/>
-        <v>41</v>
-      </c>
-    </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R20" s="1">
+        <v>4</v>
+      </c>
+      <c r="S20" s="1">
+        <v>4</v>
+      </c>
+      <c r="T20" s="1">
+        <v>3</v>
+      </c>
+      <c r="U20" s="10">
+        <f t="shared" si="0"/>
+        <v>52</v>
+      </c>
+    </row>
+    <row r="21" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A21" s="11">
         <v>19</v>
       </c>
@@ -2977,14 +3128,21 @@
       <c r="Q21" s="1">
         <v>3</v>
       </c>
-      <c r="R21" s="1"/>
-      <c r="S21" s="1"/>
-      <c r="T21" s="10">
-        <f t="shared" si="0"/>
-        <v>34</v>
-      </c>
-    </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R21" s="1">
+        <v>5</v>
+      </c>
+      <c r="S21" s="1">
+        <v>5</v>
+      </c>
+      <c r="T21" s="1">
+        <v>0</v>
+      </c>
+      <c r="U21" s="10">
+        <f t="shared" si="0"/>
+        <v>44</v>
+      </c>
+    </row>
+    <row r="22" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A22" s="11">
         <v>20</v>
       </c>
@@ -3036,14 +3194,21 @@
       <c r="Q22" s="1">
         <v>4</v>
       </c>
-      <c r="R22" s="1"/>
-      <c r="S22" s="1"/>
-      <c r="T22" s="10">
-        <f t="shared" si="0"/>
-        <v>46</v>
-      </c>
-    </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R22" s="1">
+        <v>1</v>
+      </c>
+      <c r="S22" s="1">
+        <v>0</v>
+      </c>
+      <c r="T22" s="1">
+        <v>0</v>
+      </c>
+      <c r="U22" s="10">
+        <f t="shared" si="0"/>
+        <v>47</v>
+      </c>
+    </row>
+    <row r="23" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A23" s="11">
         <v>21</v>
       </c>
@@ -3095,14 +3260,21 @@
       <c r="Q23" s="1">
         <v>5</v>
       </c>
-      <c r="R23" s="1"/>
-      <c r="S23" s="1"/>
-      <c r="T23" s="10">
-        <f t="shared" si="0"/>
-        <v>38</v>
-      </c>
-    </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R23" s="1">
+        <v>0</v>
+      </c>
+      <c r="S23" s="1">
+        <v>5</v>
+      </c>
+      <c r="T23" s="1">
+        <v>1</v>
+      </c>
+      <c r="U23" s="10">
+        <f t="shared" si="0"/>
+        <v>44</v>
+      </c>
+    </row>
+    <row r="24" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A24" s="11">
         <v>22</v>
       </c>
@@ -3154,14 +3326,21 @@
       <c r="Q24" s="1">
         <v>0</v>
       </c>
-      <c r="R24" s="1"/>
-      <c r="S24" s="1"/>
-      <c r="T24" s="10">
+      <c r="R24" s="1">
+        <v>0</v>
+      </c>
+      <c r="S24" s="1">
+        <v>0</v>
+      </c>
+      <c r="T24" s="1">
+        <v>0</v>
+      </c>
+      <c r="U24" s="10">
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A25" s="11">
         <v>23</v>
       </c>
@@ -3213,14 +3392,21 @@
       <c r="Q25" s="1">
         <v>5</v>
       </c>
-      <c r="R25" s="1"/>
-      <c r="S25" s="1"/>
-      <c r="T25" s="10">
-        <f t="shared" si="0"/>
-        <v>26</v>
-      </c>
-    </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R25" s="1">
+        <v>3</v>
+      </c>
+      <c r="S25" s="1">
+        <v>4</v>
+      </c>
+      <c r="T25" s="1">
+        <v>0</v>
+      </c>
+      <c r="U25" s="10">
+        <f t="shared" si="0"/>
+        <v>33</v>
+      </c>
+    </row>
+    <row r="26" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A26" s="11">
         <v>24</v>
       </c>
@@ -3272,14 +3458,21 @@
       <c r="Q26" s="1">
         <v>5</v>
       </c>
-      <c r="R26" s="1"/>
-      <c r="S26" s="1"/>
-      <c r="T26" s="10">
-        <f t="shared" si="0"/>
-        <v>20</v>
-      </c>
-    </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R26" s="1">
+        <v>3</v>
+      </c>
+      <c r="S26" s="1">
+        <v>5</v>
+      </c>
+      <c r="T26" s="1">
+        <v>0</v>
+      </c>
+      <c r="U26" s="10">
+        <f t="shared" si="0"/>
+        <v>28</v>
+      </c>
+    </row>
+    <row r="27" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A27" s="11">
         <v>25</v>
       </c>
@@ -3331,14 +3524,21 @@
       <c r="Q27" s="1">
         <v>5</v>
       </c>
-      <c r="R27" s="1"/>
-      <c r="S27" s="1"/>
-      <c r="T27" s="10">
-        <f t="shared" si="0"/>
-        <v>38</v>
-      </c>
-    </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R27" s="1">
+        <v>2</v>
+      </c>
+      <c r="S27" s="1">
+        <v>3</v>
+      </c>
+      <c r="T27" s="1">
+        <v>0</v>
+      </c>
+      <c r="U27" s="10">
+        <f t="shared" si="0"/>
+        <v>43</v>
+      </c>
+    </row>
+    <row r="28" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A28" s="11">
         <v>26</v>
       </c>
@@ -3390,14 +3590,21 @@
       <c r="Q28" s="1">
         <v>5</v>
       </c>
-      <c r="R28" s="1"/>
-      <c r="S28" s="1"/>
-      <c r="T28" s="10">
-        <f t="shared" si="0"/>
-        <v>36</v>
-      </c>
-    </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R28" s="1">
+        <v>3</v>
+      </c>
+      <c r="S28" s="1">
+        <v>5</v>
+      </c>
+      <c r="T28" s="1">
+        <v>3</v>
+      </c>
+      <c r="U28" s="10">
+        <f t="shared" si="0"/>
+        <v>47</v>
+      </c>
+    </row>
+    <row r="29" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A29" s="11">
         <v>27</v>
       </c>
@@ -3449,14 +3656,21 @@
       <c r="Q29" s="1">
         <v>5</v>
       </c>
-      <c r="R29" s="1"/>
-      <c r="S29" s="1"/>
-      <c r="T29" s="10">
-        <f t="shared" si="0"/>
-        <v>48</v>
-      </c>
-    </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R29" s="1">
+        <v>4</v>
+      </c>
+      <c r="S29" s="1">
+        <v>2</v>
+      </c>
+      <c r="T29" s="1">
+        <v>5</v>
+      </c>
+      <c r="U29" s="10">
+        <f t="shared" si="0"/>
+        <v>59</v>
+      </c>
+    </row>
+    <row r="30" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A30" s="11">
         <v>28</v>
       </c>
@@ -3508,14 +3722,21 @@
       <c r="Q30" s="1">
         <v>0</v>
       </c>
-      <c r="R30" s="1"/>
-      <c r="S30" s="1"/>
-      <c r="T30" s="10">
-        <f t="shared" si="0"/>
-        <v>14</v>
-      </c>
-    </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R30" s="1">
+        <v>0</v>
+      </c>
+      <c r="S30" s="1">
+        <v>2</v>
+      </c>
+      <c r="T30" s="1">
+        <v>0</v>
+      </c>
+      <c r="U30" s="10">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="31" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A31" s="11">
         <v>29</v>
       </c>
@@ -3567,14 +3788,21 @@
       <c r="Q31" s="1">
         <v>5</v>
       </c>
-      <c r="R31" s="1"/>
-      <c r="S31" s="1"/>
-      <c r="T31" s="10">
-        <f t="shared" si="0"/>
-        <v>38</v>
-      </c>
-    </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R31" s="1">
+        <v>5</v>
+      </c>
+      <c r="S31" s="1">
+        <v>5</v>
+      </c>
+      <c r="T31" s="1">
+        <v>5</v>
+      </c>
+      <c r="U31" s="10">
+        <f t="shared" si="0"/>
+        <v>53</v>
+      </c>
+    </row>
+    <row r="32" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A32" s="11">
         <v>30</v>
       </c>
@@ -3626,14 +3854,21 @@
       <c r="Q32" s="1">
         <v>0</v>
       </c>
-      <c r="R32" s="1"/>
-      <c r="S32" s="1"/>
-      <c r="T32" s="10">
-        <f t="shared" si="0"/>
-        <v>34</v>
-      </c>
-    </row>
-    <row r="33" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R32" s="1">
+        <v>4</v>
+      </c>
+      <c r="S32" s="1">
+        <v>0</v>
+      </c>
+      <c r="T32" s="1">
+        <v>5</v>
+      </c>
+      <c r="U32" s="10">
+        <f t="shared" si="0"/>
+        <v>43</v>
+      </c>
+    </row>
+    <row r="33" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A33" s="11">
         <v>31</v>
       </c>
@@ -3685,14 +3920,21 @@
       <c r="Q33" s="1">
         <v>5</v>
       </c>
-      <c r="R33" s="1"/>
-      <c r="S33" s="1"/>
-      <c r="T33" s="10">
-        <f t="shared" si="0"/>
-        <v>50</v>
-      </c>
-    </row>
-    <row r="34" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R33" s="1">
+        <v>5</v>
+      </c>
+      <c r="S33" s="1">
+        <v>5</v>
+      </c>
+      <c r="T33" s="1">
+        <v>4</v>
+      </c>
+      <c r="U33" s="10">
+        <f t="shared" si="0"/>
+        <v>64</v>
+      </c>
+    </row>
+    <row r="34" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A34" s="11">
         <v>32</v>
       </c>
@@ -3744,14 +3986,21 @@
       <c r="Q34" s="1">
         <v>5</v>
       </c>
-      <c r="R34" s="1"/>
-      <c r="S34" s="1"/>
-      <c r="T34" s="10">
-        <f t="shared" si="0"/>
-        <v>45</v>
-      </c>
-    </row>
-    <row r="35" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R34" s="1">
+        <v>4</v>
+      </c>
+      <c r="S34" s="1">
+        <v>5</v>
+      </c>
+      <c r="T34" s="1">
+        <v>5</v>
+      </c>
+      <c r="U34" s="10">
+        <f t="shared" si="0"/>
+        <v>59</v>
+      </c>
+    </row>
+    <row r="35" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A35" s="11">
         <v>33</v>
       </c>
@@ -3803,14 +4052,21 @@
       <c r="Q35" s="1">
         <v>5</v>
       </c>
-      <c r="R35" s="1"/>
-      <c r="S35" s="1"/>
-      <c r="T35" s="10">
-        <f t="shared" si="0"/>
-        <v>39</v>
-      </c>
-    </row>
-    <row r="36" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R35" s="1">
+        <v>3</v>
+      </c>
+      <c r="S35" s="1">
+        <v>4</v>
+      </c>
+      <c r="T35" s="1">
+        <v>5</v>
+      </c>
+      <c r="U35" s="10">
+        <f t="shared" si="0"/>
+        <v>51</v>
+      </c>
+    </row>
+    <row r="36" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A36" s="11">
         <v>34</v>
       </c>
@@ -3862,14 +4118,21 @@
       <c r="Q36" s="1">
         <v>5</v>
       </c>
-      <c r="R36" s="1"/>
-      <c r="S36" s="1"/>
-      <c r="T36" s="10">
-        <f t="shared" si="0"/>
-        <v>36</v>
-      </c>
-    </row>
-    <row r="37" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R36" s="1">
+        <v>4</v>
+      </c>
+      <c r="S36" s="1">
+        <v>5</v>
+      </c>
+      <c r="T36" s="1">
+        <v>3</v>
+      </c>
+      <c r="U36" s="10">
+        <f t="shared" si="0"/>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="37" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A37" s="11">
         <v>35</v>
       </c>
@@ -3921,14 +4184,21 @@
       <c r="Q37" s="1">
         <v>5</v>
       </c>
-      <c r="R37" s="1"/>
-      <c r="S37" s="1"/>
-      <c r="T37" s="10">
-        <f t="shared" si="0"/>
-        <v>32</v>
-      </c>
-    </row>
-    <row r="38" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R37" s="1">
+        <v>5</v>
+      </c>
+      <c r="S37" s="1">
+        <v>5</v>
+      </c>
+      <c r="T37" s="1">
+        <v>5</v>
+      </c>
+      <c r="U37" s="10">
+        <f t="shared" si="0"/>
+        <v>47</v>
+      </c>
+    </row>
+    <row r="38" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A38" s="11">
         <v>36</v>
       </c>
@@ -3980,14 +4250,21 @@
       <c r="Q38" s="1">
         <v>0</v>
       </c>
-      <c r="R38" s="1"/>
-      <c r="S38" s="1"/>
-      <c r="T38" s="10">
-        <f t="shared" si="0"/>
-        <v>12</v>
-      </c>
-    </row>
-    <row r="39" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R38" s="1">
+        <v>4</v>
+      </c>
+      <c r="S38" s="1">
+        <v>5</v>
+      </c>
+      <c r="T38" s="1">
+        <v>0</v>
+      </c>
+      <c r="U38" s="10">
+        <f t="shared" si="0"/>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="39" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A39" s="11">
         <v>37</v>
       </c>
@@ -4039,14 +4316,21 @@
       <c r="Q39" s="1">
         <v>5</v>
       </c>
-      <c r="R39" s="1"/>
-      <c r="S39" s="1"/>
-      <c r="T39" s="10">
-        <f t="shared" si="0"/>
-        <v>50</v>
-      </c>
-    </row>
-    <row r="40" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R39" s="1">
+        <v>3</v>
+      </c>
+      <c r="S39" s="1">
+        <v>3</v>
+      </c>
+      <c r="T39" s="1">
+        <v>4</v>
+      </c>
+      <c r="U39" s="10">
+        <f t="shared" si="0"/>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="40" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A40" s="11">
         <v>38</v>
       </c>
@@ -4098,14 +4382,21 @@
       <c r="Q40" s="1">
         <v>0</v>
       </c>
-      <c r="R40" s="1"/>
-      <c r="S40" s="1"/>
-      <c r="T40" s="10">
-        <f t="shared" si="0"/>
-        <v>23</v>
-      </c>
-    </row>
-    <row r="41" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R40" s="1">
+        <v>3</v>
+      </c>
+      <c r="S40" s="1">
+        <v>4</v>
+      </c>
+      <c r="T40" s="1">
+        <v>5</v>
+      </c>
+      <c r="U40" s="10">
+        <f t="shared" si="0"/>
+        <v>35</v>
+      </c>
+    </row>
+    <row r="41" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A41" s="11">
         <v>39</v>
       </c>
@@ -4157,14 +4448,21 @@
       <c r="Q41" s="1">
         <v>3</v>
       </c>
-      <c r="R41" s="1"/>
-      <c r="S41" s="1"/>
-      <c r="T41" s="10">
-        <f t="shared" si="0"/>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="42" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R41" s="1">
+        <v>4</v>
+      </c>
+      <c r="S41" s="1">
+        <v>2</v>
+      </c>
+      <c r="T41" s="1">
+        <v>3</v>
+      </c>
+      <c r="U41" s="10">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="42" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A42" s="11">
         <v>40</v>
       </c>
@@ -4216,14 +4514,21 @@
       <c r="Q42" s="1">
         <v>5</v>
       </c>
-      <c r="R42" s="1"/>
-      <c r="S42" s="1"/>
-      <c r="T42" s="10">
-        <f t="shared" si="0"/>
-        <v>17</v>
-      </c>
-    </row>
-    <row r="43" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R42" s="1">
+        <v>5</v>
+      </c>
+      <c r="S42" s="1">
+        <v>5</v>
+      </c>
+      <c r="T42" s="1">
+        <v>0</v>
+      </c>
+      <c r="U42" s="10">
+        <f t="shared" si="0"/>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="43" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A43" s="11">
         <v>41</v>
       </c>
@@ -4275,14 +4580,21 @@
       <c r="Q43" s="1">
         <v>5</v>
       </c>
-      <c r="R43" s="1"/>
-      <c r="S43" s="1"/>
-      <c r="T43" s="10">
-        <f t="shared" si="0"/>
-        <v>39</v>
-      </c>
-    </row>
-    <row r="44" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R43" s="1">
+        <v>5</v>
+      </c>
+      <c r="S43" s="1">
+        <v>4</v>
+      </c>
+      <c r="T43" s="1">
+        <v>0</v>
+      </c>
+      <c r="U43" s="10">
+        <f t="shared" si="0"/>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="44" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A44" s="11">
         <v>42</v>
       </c>
@@ -4334,14 +4646,21 @@
       <c r="Q44" s="1">
         <v>5</v>
       </c>
-      <c r="R44" s="1"/>
-      <c r="S44" s="1"/>
-      <c r="T44" s="10">
-        <f t="shared" si="0"/>
-        <v>27</v>
-      </c>
-    </row>
-    <row r="45" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R44" s="1">
+        <v>4</v>
+      </c>
+      <c r="S44" s="1">
+        <v>4</v>
+      </c>
+      <c r="T44" s="1">
+        <v>0</v>
+      </c>
+      <c r="U44" s="10">
+        <f t="shared" si="0"/>
+        <v>35</v>
+      </c>
+    </row>
+    <row r="45" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A45" s="11">
         <v>43</v>
       </c>
@@ -4393,14 +4712,21 @@
       <c r="Q45" s="1">
         <v>5</v>
       </c>
-      <c r="R45" s="1"/>
-      <c r="S45" s="1"/>
-      <c r="T45" s="10">
-        <f t="shared" si="0"/>
-        <v>33</v>
-      </c>
-    </row>
-    <row r="46" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R45" s="1">
+        <v>3</v>
+      </c>
+      <c r="S45" s="1">
+        <v>5</v>
+      </c>
+      <c r="T45" s="1">
+        <v>3</v>
+      </c>
+      <c r="U45" s="10">
+        <f t="shared" si="0"/>
+        <v>44</v>
+      </c>
+    </row>
+    <row r="46" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A46" s="11">
         <v>44</v>
       </c>
@@ -4452,14 +4778,21 @@
       <c r="Q46" s="1">
         <v>5</v>
       </c>
-      <c r="R46" s="1"/>
-      <c r="S46" s="1"/>
-      <c r="T46" s="10">
-        <f t="shared" si="0"/>
-        <v>42</v>
-      </c>
-    </row>
-    <row r="47" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R46" s="1">
+        <v>3</v>
+      </c>
+      <c r="S46" s="1">
+        <v>5</v>
+      </c>
+      <c r="T46" s="1">
+        <v>0</v>
+      </c>
+      <c r="U46" s="10">
+        <f t="shared" si="0"/>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="47" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A47" s="11">
         <v>45</v>
       </c>
@@ -4511,14 +4844,21 @@
       <c r="Q47" s="1">
         <v>5</v>
       </c>
-      <c r="R47" s="1"/>
-      <c r="S47" s="1"/>
-      <c r="T47" s="10">
-        <f t="shared" si="0"/>
-        <v>43</v>
-      </c>
-    </row>
-    <row r="48" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R47" s="1">
+        <v>5</v>
+      </c>
+      <c r="S47" s="1">
+        <v>5</v>
+      </c>
+      <c r="T47" s="1">
+        <v>5</v>
+      </c>
+      <c r="U47" s="10">
+        <f t="shared" si="0"/>
+        <v>58</v>
+      </c>
+    </row>
+    <row r="48" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A48" s="11">
         <v>46</v>
       </c>
@@ -4570,14 +4910,21 @@
       <c r="Q48" s="1">
         <v>5</v>
       </c>
-      <c r="R48" s="1"/>
-      <c r="S48" s="1"/>
-      <c r="T48" s="10">
-        <f t="shared" si="0"/>
-        <v>49</v>
-      </c>
-    </row>
-    <row r="49" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R48" s="1">
+        <v>3</v>
+      </c>
+      <c r="S48" s="1">
+        <v>5</v>
+      </c>
+      <c r="T48" s="1">
+        <v>0</v>
+      </c>
+      <c r="U48" s="10">
+        <f t="shared" si="0"/>
+        <v>57</v>
+      </c>
+    </row>
+    <row r="49" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A49" s="11">
         <v>47</v>
       </c>
@@ -4629,14 +4976,21 @@
       <c r="Q49" s="1">
         <v>5</v>
       </c>
-      <c r="R49" s="1"/>
-      <c r="S49" s="1"/>
-      <c r="T49" s="10">
-        <f t="shared" si="0"/>
-        <v>41</v>
-      </c>
-    </row>
-    <row r="50" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R49" s="1">
+        <v>4</v>
+      </c>
+      <c r="S49" s="1">
+        <v>0</v>
+      </c>
+      <c r="T49" s="1">
+        <v>0</v>
+      </c>
+      <c r="U49" s="10">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="50" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A50" s="11">
         <v>48</v>
       </c>
@@ -4688,14 +5042,21 @@
       <c r="Q50" s="1">
         <v>5</v>
       </c>
-      <c r="R50" s="1"/>
-      <c r="S50" s="1"/>
-      <c r="T50" s="10">
-        <f t="shared" si="0"/>
-        <v>46</v>
-      </c>
-    </row>
-    <row r="51" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R50" s="1">
+        <v>4</v>
+      </c>
+      <c r="S50" s="1">
+        <v>0</v>
+      </c>
+      <c r="T50" s="1">
+        <v>4</v>
+      </c>
+      <c r="U50" s="10">
+        <f t="shared" si="0"/>
+        <v>54</v>
+      </c>
+    </row>
+    <row r="51" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A51" s="11">
         <v>49</v>
       </c>
@@ -4747,14 +5108,21 @@
       <c r="Q51" s="1">
         <v>3</v>
       </c>
-      <c r="R51" s="1"/>
-      <c r="S51" s="1"/>
-      <c r="T51" s="10">
-        <f t="shared" si="0"/>
-        <v>26</v>
-      </c>
-    </row>
-    <row r="52" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R51" s="1">
+        <v>0</v>
+      </c>
+      <c r="S51" s="1">
+        <v>4</v>
+      </c>
+      <c r="T51" s="1">
+        <v>2</v>
+      </c>
+      <c r="U51" s="10">
+        <f t="shared" si="0"/>
+        <v>32</v>
+      </c>
+    </row>
+    <row r="52" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A52" s="11">
         <v>50</v>
       </c>
@@ -4806,14 +5174,21 @@
       <c r="Q52" s="1">
         <v>5</v>
       </c>
-      <c r="R52" s="1"/>
-      <c r="S52" s="1"/>
-      <c r="T52" s="10">
-        <f t="shared" si="0"/>
-        <v>34</v>
-      </c>
-    </row>
-    <row r="53" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R52" s="1">
+        <v>3</v>
+      </c>
+      <c r="S52" s="1">
+        <v>4</v>
+      </c>
+      <c r="T52" s="1">
+        <v>5</v>
+      </c>
+      <c r="U52" s="10">
+        <f t="shared" si="0"/>
+        <v>46</v>
+      </c>
+    </row>
+    <row r="53" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A53" s="11">
         <v>51</v>
       </c>
@@ -4865,14 +5240,21 @@
       <c r="Q53" s="1">
         <v>5</v>
       </c>
-      <c r="R53" s="1"/>
-      <c r="S53" s="1"/>
-      <c r="T53" s="10">
-        <f t="shared" si="0"/>
-        <v>47</v>
-      </c>
-    </row>
-    <row r="54" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R53" s="1">
+        <v>3</v>
+      </c>
+      <c r="S53" s="1">
+        <v>4</v>
+      </c>
+      <c r="T53" s="1">
+        <v>0</v>
+      </c>
+      <c r="U53" s="10">
+        <f t="shared" si="0"/>
+        <v>54</v>
+      </c>
+    </row>
+    <row r="54" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A54" s="11">
         <v>52</v>
       </c>
@@ -4924,14 +5306,21 @@
       <c r="Q54" s="1">
         <v>5</v>
       </c>
-      <c r="R54" s="1"/>
-      <c r="S54" s="1"/>
-      <c r="T54" s="10">
-        <f t="shared" si="0"/>
-        <v>51</v>
-      </c>
-    </row>
-    <row r="55" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R54" s="1">
+        <v>3</v>
+      </c>
+      <c r="S54" s="1">
+        <v>5</v>
+      </c>
+      <c r="T54" s="1">
+        <v>5</v>
+      </c>
+      <c r="U54" s="10">
+        <f t="shared" si="0"/>
+        <v>64</v>
+      </c>
+    </row>
+    <row r="55" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A55" s="11">
         <v>53</v>
       </c>
@@ -4983,14 +5372,21 @@
       <c r="Q55" s="1">
         <v>4</v>
       </c>
-      <c r="R55" s="1"/>
-      <c r="S55" s="1"/>
-      <c r="T55" s="10">
-        <f t="shared" si="0"/>
-        <v>53</v>
-      </c>
-    </row>
-    <row r="56" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R55" s="1">
+        <v>5</v>
+      </c>
+      <c r="S55" s="1">
+        <v>5</v>
+      </c>
+      <c r="T55" s="1">
+        <v>5</v>
+      </c>
+      <c r="U55" s="10">
+        <f t="shared" si="0"/>
+        <v>68</v>
+      </c>
+    </row>
+    <row r="56" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A56" s="11">
         <v>54</v>
       </c>
@@ -5042,14 +5438,21 @@
       <c r="Q56" s="1">
         <v>5</v>
       </c>
-      <c r="R56" s="1"/>
-      <c r="S56" s="1"/>
-      <c r="T56" s="10">
-        <f t="shared" si="0"/>
-        <v>48</v>
-      </c>
-    </row>
-    <row r="57" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="R56" s="1">
+        <v>4</v>
+      </c>
+      <c r="S56" s="1">
+        <v>5</v>
+      </c>
+      <c r="T56" s="1">
+        <v>4</v>
+      </c>
+      <c r="U56" s="10">
+        <f t="shared" si="0"/>
+        <v>61</v>
+      </c>
+    </row>
+    <row r="57" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A57" s="19">
         <v>55</v>
       </c>
@@ -5101,56 +5504,65 @@
       <c r="Q57" s="22">
         <v>5</v>
       </c>
-      <c r="R57" s="22"/>
-      <c r="S57" s="22"/>
-      <c r="T57" s="10">
-        <f t="shared" si="0"/>
-        <v>49</v>
-      </c>
-    </row>
-    <row r="58" spans="1:20" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+      <c r="R57" s="22">
+        <v>4</v>
+      </c>
+      <c r="S57" s="22">
+        <v>0</v>
+      </c>
+      <c r="T57" s="22">
+        <v>2</v>
+      </c>
+      <c r="U57" s="10">
+        <f>($F57+$G57+$H57+$I57+$J57+$K57+$L57+$M57+$N57+$O57+$P57+$Q57+$R57+$S57+$T57)</f>
+        <v>55</v>
+      </c>
+    </row>
+    <row r="58" spans="1:21" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="F1:S1"/>
     <mergeCell ref="A2:B2"/>
   </mergeCells>
+  <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7CD6AE0E-6B38-4517-9EE7-74576DF1F95D}">
-  <dimension ref="A1:T64"/>
+  <dimension ref="A1:U64"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A1" s="33"/>
-      <c r="B1" s="33"/>
+    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A1" s="34"/>
+      <c r="B1" s="34"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
-      <c r="F1" s="34" t="s">
-        <v>0</v>
-      </c>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
-      <c r="I1" s="35"/>
-      <c r="J1" s="35"/>
-      <c r="K1" s="35"/>
-      <c r="L1" s="35"/>
-      <c r="M1" s="35"/>
-      <c r="N1" s="35"/>
-      <c r="O1" s="35"/>
-      <c r="P1" s="35"/>
-      <c r="Q1" s="35"/>
-      <c r="R1" s="35"/>
-      <c r="S1" s="36"/>
-      <c r="T1" s="2"/>
-    </row>
-    <row r="2" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="33"/>
-      <c r="B2" s="33"/>
+      <c r="F1" s="35" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1" s="36"/>
+      <c r="H1" s="36"/>
+      <c r="I1" s="36"/>
+      <c r="J1" s="36"/>
+      <c r="K1" s="36"/>
+      <c r="L1" s="36"/>
+      <c r="M1" s="36"/>
+      <c r="N1" s="36"/>
+      <c r="O1" s="36"/>
+      <c r="P1" s="36"/>
+      <c r="Q1" s="36"/>
+      <c r="R1" s="36"/>
+      <c r="S1" s="37"/>
+      <c r="T1" s="39"/>
+      <c r="U1" s="2"/>
+    </row>
+    <row r="2" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="34"/>
+      <c r="B2" s="34"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -5196,11 +5608,14 @@
       <c r="S2" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="T2" s="5" t="s">
+      <c r="T2" s="32" t="s">
+        <v>296</v>
+      </c>
+      <c r="U2" s="5" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A3" s="11">
         <v>1</v>
       </c>
@@ -5252,14 +5667,21 @@
       <c r="Q3" s="1">
         <v>0</v>
       </c>
-      <c r="R3" s="1"/>
-      <c r="S3" s="1"/>
-      <c r="T3" s="10">
-        <f>($F3+$G3+$H3+$I3+$J3+$K3+$L3+$M3+$N3+$O3+$P3+$Q3)</f>
-        <v>35</v>
-      </c>
-    </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R3" s="1">
+        <v>5</v>
+      </c>
+      <c r="S3" s="1">
+        <v>0</v>
+      </c>
+      <c r="T3" s="1">
+        <v>0</v>
+      </c>
+      <c r="U3" s="10">
+        <f>($F3+$G3+$H3+$I3+$J3+$K3+$L3+$M3+$N3+$O3+$P3+$Q3+$R3+$S3+$T3)</f>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A4" s="11">
         <v>2</v>
       </c>
@@ -5311,14 +5733,21 @@
       <c r="Q4" s="1">
         <v>5</v>
       </c>
-      <c r="R4" s="1"/>
-      <c r="S4" s="1"/>
-      <c r="T4" s="10">
-        <f t="shared" ref="T4:T51" si="0">($F4+$G4+$H4+$I4+$J4+$K4+$L4+$M4+$N4+$O4+$P4+$Q4)</f>
-        <v>29</v>
-      </c>
-    </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R4" s="1">
+        <v>4</v>
+      </c>
+      <c r="S4" s="1">
+        <v>4</v>
+      </c>
+      <c r="T4" s="1">
+        <v>4</v>
+      </c>
+      <c r="U4" s="10">
+        <f t="shared" ref="U4:U51" si="0">($F4+$G4+$H4+$I4+$J4+$K4+$L4+$M4+$N4+$O4+$P4+$Q4+$R4+$S4+$T4)</f>
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A5" s="11">
         <v>3</v>
       </c>
@@ -5370,14 +5799,21 @@
       <c r="Q5" s="1">
         <v>0</v>
       </c>
-      <c r="R5" s="1"/>
-      <c r="S5" s="1"/>
-      <c r="T5" s="10">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R5" s="1">
+        <v>0</v>
+      </c>
+      <c r="S5" s="1">
+        <v>0</v>
+      </c>
+      <c r="T5" s="1">
+        <v>0</v>
+      </c>
+      <c r="U5" s="10">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A6" s="11">
         <v>4</v>
       </c>
@@ -5429,14 +5865,21 @@
       <c r="Q6" s="1">
         <v>0</v>
       </c>
-      <c r="R6" s="1"/>
-      <c r="S6" s="1"/>
-      <c r="T6" s="10">
-        <f t="shared" si="0"/>
-        <v>30</v>
-      </c>
-    </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R6" s="1">
+        <v>2</v>
+      </c>
+      <c r="S6" s="1">
+        <v>0</v>
+      </c>
+      <c r="T6" s="1">
+        <v>0</v>
+      </c>
+      <c r="U6" s="10">
+        <f t="shared" si="0"/>
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A7" s="11">
         <v>5</v>
       </c>
@@ -5488,14 +5931,21 @@
       <c r="Q7" s="1">
         <v>5</v>
       </c>
-      <c r="R7" s="1"/>
-      <c r="S7" s="1"/>
-      <c r="T7" s="10">
-        <f t="shared" si="0"/>
-        <v>47</v>
-      </c>
-    </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R7" s="1">
+        <v>4</v>
+      </c>
+      <c r="S7" s="1">
+        <v>4</v>
+      </c>
+      <c r="T7" s="1">
+        <v>4</v>
+      </c>
+      <c r="U7" s="10">
+        <f t="shared" si="0"/>
+        <v>59</v>
+      </c>
+    </row>
+    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A8" s="11">
         <v>6</v>
       </c>
@@ -5547,14 +5997,21 @@
       <c r="Q8" s="1">
         <v>5</v>
       </c>
-      <c r="R8" s="1"/>
-      <c r="S8" s="1"/>
-      <c r="T8" s="10">
-        <f t="shared" si="0"/>
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R8" s="1">
+        <v>5</v>
+      </c>
+      <c r="S8" s="1">
+        <v>5</v>
+      </c>
+      <c r="T8" s="1">
+        <v>4</v>
+      </c>
+      <c r="U8" s="10">
+        <f t="shared" si="0"/>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A9" s="11">
         <v>7</v>
       </c>
@@ -5606,14 +6063,21 @@
       <c r="Q9" s="1">
         <v>5</v>
       </c>
-      <c r="R9" s="1"/>
-      <c r="S9" s="1"/>
-      <c r="T9" s="10">
-        <f t="shared" si="0"/>
-        <v>48</v>
-      </c>
-    </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R9" s="1">
+        <v>4</v>
+      </c>
+      <c r="S9" s="1">
+        <v>5</v>
+      </c>
+      <c r="T9" s="1">
+        <v>5</v>
+      </c>
+      <c r="U9" s="10">
+        <f t="shared" si="0"/>
+        <v>62</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A10" s="11">
         <v>8</v>
       </c>
@@ -5665,14 +6129,21 @@
       <c r="Q10" s="1">
         <v>5</v>
       </c>
-      <c r="R10" s="1"/>
-      <c r="S10" s="1"/>
-      <c r="T10" s="10">
-        <f t="shared" si="0"/>
-        <v>17</v>
-      </c>
-    </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R10" s="1">
+        <v>0</v>
+      </c>
+      <c r="S10" s="1">
+        <v>5</v>
+      </c>
+      <c r="T10" s="1">
+        <v>1</v>
+      </c>
+      <c r="U10" s="10">
+        <f t="shared" si="0"/>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A11" s="11">
         <v>9</v>
       </c>
@@ -5724,14 +6195,21 @@
       <c r="Q11" s="1">
         <v>0</v>
       </c>
-      <c r="R11" s="1"/>
-      <c r="S11" s="1"/>
-      <c r="T11" s="10">
-        <f t="shared" si="0"/>
-        <v>31</v>
-      </c>
-    </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R11" s="1">
+        <v>0</v>
+      </c>
+      <c r="S11" s="1">
+        <v>5</v>
+      </c>
+      <c r="T11" s="1">
+        <v>5</v>
+      </c>
+      <c r="U11" s="10">
+        <f t="shared" si="0"/>
+        <v>41</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A12" s="11">
         <v>10</v>
       </c>
@@ -5783,14 +6261,21 @@
       <c r="Q12" s="1">
         <v>5</v>
       </c>
-      <c r="R12" s="1"/>
-      <c r="S12" s="1"/>
-      <c r="T12" s="10">
-        <f t="shared" si="0"/>
-        <v>45</v>
-      </c>
-    </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R12" s="1">
+        <v>4</v>
+      </c>
+      <c r="S12" s="1">
+        <v>5</v>
+      </c>
+      <c r="T12" s="1">
+        <v>4</v>
+      </c>
+      <c r="U12" s="10">
+        <f t="shared" si="0"/>
+        <v>58</v>
+      </c>
+    </row>
+    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A13" s="11">
         <v>11</v>
       </c>
@@ -5842,14 +6327,21 @@
       <c r="Q13" s="1">
         <v>5</v>
       </c>
-      <c r="R13" s="1"/>
-      <c r="S13" s="1"/>
-      <c r="T13" s="10">
-        <f t="shared" si="0"/>
-        <v>53</v>
-      </c>
-    </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R13" s="1">
+        <v>4</v>
+      </c>
+      <c r="S13" s="1">
+        <v>5</v>
+      </c>
+      <c r="T13" s="1">
+        <v>5</v>
+      </c>
+      <c r="U13" s="10">
+        <f t="shared" si="0"/>
+        <v>67</v>
+      </c>
+    </row>
+    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A14" s="11">
         <v>12</v>
       </c>
@@ -5901,14 +6393,21 @@
       <c r="Q14" s="1">
         <v>0</v>
       </c>
-      <c r="R14" s="1"/>
-      <c r="S14" s="1"/>
-      <c r="T14" s="10">
-        <f t="shared" si="0"/>
-        <v>26</v>
-      </c>
-    </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R14" s="1">
+        <v>4</v>
+      </c>
+      <c r="S14" s="1">
+        <v>5</v>
+      </c>
+      <c r="T14" s="1">
+        <v>2</v>
+      </c>
+      <c r="U14" s="10">
+        <f t="shared" si="0"/>
+        <v>37</v>
+      </c>
+    </row>
+    <row r="15" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A15" s="11">
         <v>13</v>
       </c>
@@ -5960,14 +6459,21 @@
       <c r="Q15" s="1">
         <v>5</v>
       </c>
-      <c r="R15" s="1"/>
-      <c r="S15" s="1"/>
-      <c r="T15" s="10">
-        <f t="shared" si="0"/>
-        <v>16</v>
-      </c>
-    </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R15" s="1">
+        <v>5</v>
+      </c>
+      <c r="S15" s="1">
+        <v>4</v>
+      </c>
+      <c r="T15" s="1">
+        <v>3</v>
+      </c>
+      <c r="U15" s="10">
+        <f t="shared" si="0"/>
+        <v>28</v>
+      </c>
+    </row>
+    <row r="16" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A16" s="11">
         <v>14</v>
       </c>
@@ -6019,14 +6525,21 @@
       <c r="Q16" s="1">
         <v>5</v>
       </c>
-      <c r="R16" s="1"/>
-      <c r="S16" s="1"/>
-      <c r="T16" s="10">
-        <f t="shared" si="0"/>
-        <v>33</v>
-      </c>
-    </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R16" s="1">
+        <v>4</v>
+      </c>
+      <c r="S16" s="1">
+        <v>0</v>
+      </c>
+      <c r="T16" s="1">
+        <v>0</v>
+      </c>
+      <c r="U16" s="10">
+        <f t="shared" si="0"/>
+        <v>37</v>
+      </c>
+    </row>
+    <row r="17" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A17" s="11">
         <v>15</v>
       </c>
@@ -6078,14 +6591,21 @@
       <c r="Q17" s="1">
         <v>5</v>
       </c>
-      <c r="R17" s="1"/>
-      <c r="S17" s="1"/>
-      <c r="T17" s="10">
-        <f t="shared" si="0"/>
-        <v>35</v>
-      </c>
-    </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R17" s="1">
+        <v>3</v>
+      </c>
+      <c r="S17" s="1">
+        <v>5</v>
+      </c>
+      <c r="T17" s="1">
+        <v>1</v>
+      </c>
+      <c r="U17" s="10">
+        <f t="shared" si="0"/>
+        <v>44</v>
+      </c>
+    </row>
+    <row r="18" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A18" s="11">
         <v>16</v>
       </c>
@@ -6137,14 +6657,21 @@
       <c r="Q18" s="1">
         <v>5</v>
       </c>
-      <c r="R18" s="1"/>
-      <c r="S18" s="1"/>
-      <c r="T18" s="10">
-        <f t="shared" si="0"/>
-        <v>41</v>
-      </c>
-    </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R18" s="1">
+        <v>4</v>
+      </c>
+      <c r="S18" s="1">
+        <v>4</v>
+      </c>
+      <c r="T18" s="1">
+        <v>2</v>
+      </c>
+      <c r="U18" s="10">
+        <f t="shared" si="0"/>
+        <v>51</v>
+      </c>
+    </row>
+    <row r="19" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A19" s="11">
         <v>17</v>
       </c>
@@ -6196,14 +6723,21 @@
       <c r="Q19" s="1">
         <v>5</v>
       </c>
-      <c r="R19" s="1"/>
-      <c r="S19" s="1"/>
-      <c r="T19" s="10">
-        <f t="shared" si="0"/>
-        <v>17</v>
-      </c>
-    </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R19" s="1">
+        <v>2</v>
+      </c>
+      <c r="S19" s="1">
+        <v>4</v>
+      </c>
+      <c r="T19" s="1">
+        <v>4</v>
+      </c>
+      <c r="U19" s="10">
+        <f t="shared" si="0"/>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="20" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A20" s="11">
         <v>18</v>
       </c>
@@ -6255,14 +6789,21 @@
       <c r="Q20" s="1">
         <v>5</v>
       </c>
-      <c r="R20" s="1"/>
-      <c r="S20" s="1"/>
-      <c r="T20" s="10">
-        <f t="shared" si="0"/>
-        <v>41</v>
-      </c>
-    </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R20" s="1">
+        <v>4</v>
+      </c>
+      <c r="S20" s="1">
+        <v>4</v>
+      </c>
+      <c r="T20" s="1">
+        <v>4</v>
+      </c>
+      <c r="U20" s="10">
+        <f t="shared" si="0"/>
+        <v>53</v>
+      </c>
+    </row>
+    <row r="21" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A21" s="11">
         <v>19</v>
       </c>
@@ -6314,14 +6855,21 @@
       <c r="Q21" s="1">
         <v>5</v>
       </c>
-      <c r="R21" s="1"/>
-      <c r="S21" s="1"/>
-      <c r="T21" s="10">
-        <f t="shared" si="0"/>
-        <v>40</v>
-      </c>
-    </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R21" s="1">
+        <v>2</v>
+      </c>
+      <c r="S21" s="1">
+        <v>2</v>
+      </c>
+      <c r="T21" s="1">
+        <v>4</v>
+      </c>
+      <c r="U21" s="10">
+        <f t="shared" si="0"/>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="22" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A22" s="11">
         <v>20</v>
       </c>
@@ -6373,14 +6921,21 @@
       <c r="Q22" s="1">
         <v>5</v>
       </c>
-      <c r="R22" s="1"/>
-      <c r="S22" s="1"/>
-      <c r="T22" s="10">
-        <f t="shared" si="0"/>
-        <v>46</v>
-      </c>
-    </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R22" s="1">
+        <v>4</v>
+      </c>
+      <c r="S22" s="1">
+        <v>5</v>
+      </c>
+      <c r="T22" s="1">
+        <v>4</v>
+      </c>
+      <c r="U22" s="10">
+        <f t="shared" si="0"/>
+        <v>59</v>
+      </c>
+    </row>
+    <row r="23" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A23" s="11">
         <v>21</v>
       </c>
@@ -6432,14 +6987,21 @@
       <c r="Q23" s="1">
         <v>5</v>
       </c>
-      <c r="R23" s="1"/>
-      <c r="S23" s="1"/>
-      <c r="T23" s="10">
-        <f t="shared" si="0"/>
-        <v>30</v>
-      </c>
-    </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R23" s="1">
+        <v>2</v>
+      </c>
+      <c r="S23" s="1">
+        <v>0</v>
+      </c>
+      <c r="T23" s="1">
+        <v>0</v>
+      </c>
+      <c r="U23" s="10">
+        <f t="shared" si="0"/>
+        <v>32</v>
+      </c>
+    </row>
+    <row r="24" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A24" s="11">
         <v>22</v>
       </c>
@@ -6491,14 +7053,21 @@
       <c r="Q24" s="1">
         <v>5</v>
       </c>
-      <c r="R24" s="1"/>
-      <c r="S24" s="1"/>
-      <c r="T24" s="10">
-        <f t="shared" si="0"/>
-        <v>32</v>
-      </c>
-    </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R24" s="1">
+        <v>4</v>
+      </c>
+      <c r="S24" s="1">
+        <v>5</v>
+      </c>
+      <c r="T24" s="1">
+        <v>0</v>
+      </c>
+      <c r="U24" s="10">
+        <f t="shared" si="0"/>
+        <v>41</v>
+      </c>
+    </row>
+    <row r="25" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A25" s="11">
         <v>23</v>
       </c>
@@ -6550,14 +7119,21 @@
       <c r="Q25" s="1">
         <v>0</v>
       </c>
-      <c r="R25" s="1"/>
-      <c r="S25" s="1"/>
-      <c r="T25" s="10">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R25" s="1">
+        <v>0</v>
+      </c>
+      <c r="S25" s="1">
+        <v>0</v>
+      </c>
+      <c r="T25" s="1">
+        <v>0</v>
+      </c>
+      <c r="U25" s="10">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A26" s="11">
         <v>24</v>
       </c>
@@ -6609,14 +7185,21 @@
       <c r="Q26" s="1">
         <v>5</v>
       </c>
-      <c r="R26" s="1"/>
-      <c r="S26" s="1"/>
-      <c r="T26" s="10">
-        <f t="shared" si="0"/>
-        <v>37</v>
-      </c>
-    </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R26" s="1">
+        <v>4</v>
+      </c>
+      <c r="S26" s="1">
+        <v>3</v>
+      </c>
+      <c r="T26" s="1">
+        <v>4</v>
+      </c>
+      <c r="U26" s="10">
+        <f t="shared" si="0"/>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="27" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A27" s="11">
         <v>25</v>
       </c>
@@ -6668,14 +7251,21 @@
       <c r="Q27" s="1">
         <v>5</v>
       </c>
-      <c r="R27" s="1"/>
-      <c r="S27" s="1"/>
-      <c r="T27" s="10">
+      <c r="R27" s="1">
+        <v>0</v>
+      </c>
+      <c r="S27" s="1">
+        <v>0</v>
+      </c>
+      <c r="T27" s="1">
+        <v>0</v>
+      </c>
+      <c r="U27" s="10">
         <f t="shared" si="0"/>
         <v>47</v>
       </c>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A28" s="11">
         <v>26</v>
       </c>
@@ -6727,14 +7317,21 @@
       <c r="Q28" s="1">
         <v>5</v>
       </c>
-      <c r="R28" s="1"/>
-      <c r="S28" s="1"/>
-      <c r="T28" s="10">
-        <f t="shared" si="0"/>
-        <v>49</v>
-      </c>
-    </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R28" s="1">
+        <v>3</v>
+      </c>
+      <c r="S28" s="1">
+        <v>5</v>
+      </c>
+      <c r="T28" s="1">
+        <v>5</v>
+      </c>
+      <c r="U28" s="10">
+        <f t="shared" si="0"/>
+        <v>62</v>
+      </c>
+    </row>
+    <row r="29" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A29" s="11">
         <v>27</v>
       </c>
@@ -6786,14 +7383,21 @@
       <c r="Q29" s="1">
         <v>0</v>
       </c>
-      <c r="R29" s="1"/>
-      <c r="S29" s="1"/>
-      <c r="T29" s="10">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R29" s="1">
+        <v>3</v>
+      </c>
+      <c r="S29" s="1">
+        <v>0</v>
+      </c>
+      <c r="T29" s="1">
+        <v>0</v>
+      </c>
+      <c r="U29" s="10">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A30" s="11">
         <v>28</v>
       </c>
@@ -6845,14 +7449,21 @@
       <c r="Q30" s="1">
         <v>5</v>
       </c>
-      <c r="R30" s="1"/>
-      <c r="S30" s="1"/>
-      <c r="T30" s="10">
-        <f t="shared" si="0"/>
-        <v>34</v>
-      </c>
-    </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R30" s="1">
+        <v>0</v>
+      </c>
+      <c r="S30" s="1">
+        <v>4</v>
+      </c>
+      <c r="T30" s="1">
+        <v>3</v>
+      </c>
+      <c r="U30" s="10">
+        <f t="shared" si="0"/>
+        <v>41</v>
+      </c>
+    </row>
+    <row r="31" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A31" s="11">
         <v>29</v>
       </c>
@@ -6904,14 +7515,21 @@
       <c r="Q31" s="1">
         <v>5</v>
       </c>
-      <c r="R31" s="1"/>
-      <c r="S31" s="1"/>
-      <c r="T31" s="10">
-        <f t="shared" si="0"/>
-        <v>42</v>
-      </c>
-    </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R31" s="1">
+        <v>0</v>
+      </c>
+      <c r="S31" s="1">
+        <v>3</v>
+      </c>
+      <c r="T31" s="1">
+        <v>3</v>
+      </c>
+      <c r="U31" s="10">
+        <f t="shared" si="0"/>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="32" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A32" s="11">
         <v>30</v>
       </c>
@@ -6963,14 +7581,21 @@
       <c r="Q32" s="1">
         <v>4</v>
       </c>
-      <c r="R32" s="1"/>
-      <c r="S32" s="1"/>
-      <c r="T32" s="10">
-        <f t="shared" si="0"/>
-        <v>43</v>
-      </c>
-    </row>
-    <row r="33" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R32" s="1">
+        <v>3</v>
+      </c>
+      <c r="S32" s="1">
+        <v>2</v>
+      </c>
+      <c r="T32" s="1">
+        <v>4</v>
+      </c>
+      <c r="U32" s="10">
+        <f t="shared" si="0"/>
+        <v>52</v>
+      </c>
+    </row>
+    <row r="33" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A33" s="11">
         <v>31</v>
       </c>
@@ -7022,14 +7647,21 @@
       <c r="Q33" s="1">
         <v>0</v>
       </c>
-      <c r="R33" s="1"/>
-      <c r="S33" s="1"/>
-      <c r="T33" s="10">
-        <f t="shared" si="0"/>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="34" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R33" s="1">
+        <v>4</v>
+      </c>
+      <c r="S33" s="1">
+        <v>0</v>
+      </c>
+      <c r="T33" s="1">
+        <v>0</v>
+      </c>
+      <c r="U33" s="10">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="34" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A34" s="11">
         <v>32</v>
       </c>
@@ -7081,14 +7713,21 @@
       <c r="Q34" s="1">
         <v>5</v>
       </c>
-      <c r="R34" s="1"/>
-      <c r="S34" s="1"/>
-      <c r="T34" s="10">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="35" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R34" s="1">
+        <v>4</v>
+      </c>
+      <c r="S34" s="1">
+        <v>5</v>
+      </c>
+      <c r="T34" s="1">
+        <v>0</v>
+      </c>
+      <c r="U34" s="10">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="35" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A35" s="11">
         <v>33</v>
       </c>
@@ -7140,14 +7779,21 @@
       <c r="Q35" s="1">
         <v>4</v>
       </c>
-      <c r="R35" s="1"/>
-      <c r="S35" s="1"/>
-      <c r="T35" s="10">
-        <f t="shared" si="0"/>
-        <v>45</v>
-      </c>
-    </row>
-    <row r="36" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R35" s="1">
+        <v>2</v>
+      </c>
+      <c r="S35" s="1">
+        <v>4</v>
+      </c>
+      <c r="T35" s="1">
+        <v>5</v>
+      </c>
+      <c r="U35" s="10">
+        <f t="shared" si="0"/>
+        <v>56</v>
+      </c>
+    </row>
+    <row r="36" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A36" s="11">
         <v>34</v>
       </c>
@@ -7199,14 +7845,21 @@
       <c r="Q36" s="1">
         <v>0</v>
       </c>
-      <c r="R36" s="1"/>
-      <c r="S36" s="1"/>
-      <c r="T36" s="10">
-        <f t="shared" si="0"/>
-        <v>34</v>
-      </c>
-    </row>
-    <row r="37" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R36" s="1">
+        <v>0</v>
+      </c>
+      <c r="S36" s="1">
+        <v>5</v>
+      </c>
+      <c r="T36" s="1">
+        <v>4</v>
+      </c>
+      <c r="U36" s="10">
+        <f t="shared" si="0"/>
+        <v>43</v>
+      </c>
+    </row>
+    <row r="37" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A37" s="11">
         <v>35</v>
       </c>
@@ -7258,14 +7911,21 @@
       <c r="Q37" s="1">
         <v>5</v>
       </c>
-      <c r="R37" s="1"/>
-      <c r="S37" s="1"/>
-      <c r="T37" s="10">
-        <f t="shared" si="0"/>
-        <v>45</v>
-      </c>
-    </row>
-    <row r="38" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R37" s="1">
+        <v>4</v>
+      </c>
+      <c r="S37" s="1">
+        <v>4</v>
+      </c>
+      <c r="T37" s="1">
+        <v>4</v>
+      </c>
+      <c r="U37" s="10">
+        <f t="shared" si="0"/>
+        <v>57</v>
+      </c>
+    </row>
+    <row r="38" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A38" s="11">
         <v>36</v>
       </c>
@@ -7317,14 +7977,21 @@
       <c r="Q38" s="1">
         <v>5</v>
       </c>
-      <c r="R38" s="1"/>
-      <c r="S38" s="1"/>
-      <c r="T38" s="10">
-        <f t="shared" si="0"/>
-        <v>44</v>
-      </c>
-    </row>
-    <row r="39" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R38" s="1">
+        <v>3</v>
+      </c>
+      <c r="S38" s="1">
+        <v>5</v>
+      </c>
+      <c r="T38" s="1">
+        <v>2</v>
+      </c>
+      <c r="U38" s="10">
+        <f t="shared" si="0"/>
+        <v>54</v>
+      </c>
+    </row>
+    <row r="39" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A39" s="11">
         <v>37</v>
       </c>
@@ -7376,14 +8043,21 @@
       <c r="Q39" s="1">
         <v>5</v>
       </c>
-      <c r="R39" s="1"/>
-      <c r="S39" s="1"/>
-      <c r="T39" s="10">
+      <c r="R39" s="1">
+        <v>0</v>
+      </c>
+      <c r="S39" s="1">
+        <v>0</v>
+      </c>
+      <c r="T39" s="1">
+        <v>0</v>
+      </c>
+      <c r="U39" s="10">
         <f t="shared" si="0"/>
         <v>38</v>
       </c>
     </row>
-    <row r="40" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A40" s="11">
         <v>38</v>
       </c>
@@ -7435,14 +8109,21 @@
       <c r="Q40" s="1">
         <v>5</v>
       </c>
-      <c r="R40" s="1"/>
-      <c r="S40" s="1"/>
-      <c r="T40" s="10">
-        <f t="shared" si="0"/>
-        <v>18</v>
-      </c>
-    </row>
-    <row r="41" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R40" s="1">
+        <v>2</v>
+      </c>
+      <c r="S40" s="1">
+        <v>5</v>
+      </c>
+      <c r="T40" s="1">
+        <v>5</v>
+      </c>
+      <c r="U40" s="10">
+        <f t="shared" si="0"/>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="41" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A41" s="11">
         <v>39</v>
       </c>
@@ -7494,14 +8175,21 @@
       <c r="Q41" s="1">
         <v>0</v>
       </c>
-      <c r="R41" s="1"/>
-      <c r="S41" s="1"/>
-      <c r="T41" s="10">
+      <c r="R41" s="1">
+        <v>0</v>
+      </c>
+      <c r="S41" s="1">
+        <v>0</v>
+      </c>
+      <c r="T41" s="1">
+        <v>0</v>
+      </c>
+      <c r="U41" s="10">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
     </row>
-    <row r="42" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A42" s="11">
         <v>40</v>
       </c>
@@ -7553,14 +8241,21 @@
       <c r="Q42" s="1">
         <v>5</v>
       </c>
-      <c r="R42" s="1"/>
-      <c r="S42" s="1"/>
-      <c r="T42" s="10">
-        <f t="shared" si="0"/>
-        <v>38</v>
-      </c>
-    </row>
-    <row r="43" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R42" s="1">
+        <v>5</v>
+      </c>
+      <c r="S42" s="1">
+        <v>5</v>
+      </c>
+      <c r="T42" s="1">
+        <v>3</v>
+      </c>
+      <c r="U42" s="10">
+        <f t="shared" si="0"/>
+        <v>51</v>
+      </c>
+    </row>
+    <row r="43" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A43" s="11">
         <v>41</v>
       </c>
@@ -7612,14 +8307,21 @@
       <c r="Q43" s="1">
         <v>5</v>
       </c>
-      <c r="R43" s="1"/>
-      <c r="S43" s="1"/>
-      <c r="T43" s="10">
-        <f t="shared" si="0"/>
-        <v>47</v>
-      </c>
-    </row>
-    <row r="44" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R43" s="1">
+        <v>5</v>
+      </c>
+      <c r="S43" s="1">
+        <v>5</v>
+      </c>
+      <c r="T43" s="1">
+        <v>4</v>
+      </c>
+      <c r="U43" s="10">
+        <f t="shared" si="0"/>
+        <v>61</v>
+      </c>
+    </row>
+    <row r="44" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A44" s="11">
         <v>42</v>
       </c>
@@ -7671,14 +8373,21 @@
       <c r="Q44" s="1">
         <v>5</v>
       </c>
-      <c r="R44" s="1"/>
-      <c r="S44" s="1"/>
-      <c r="T44" s="10">
+      <c r="R44" s="1">
+        <v>0</v>
+      </c>
+      <c r="S44" s="1">
+        <v>0</v>
+      </c>
+      <c r="T44" s="1">
+        <v>0</v>
+      </c>
+      <c r="U44" s="10">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
     </row>
-    <row r="45" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A45" s="11">
         <v>43</v>
       </c>
@@ -7730,14 +8439,21 @@
       <c r="Q45" s="1">
         <v>4</v>
       </c>
-      <c r="R45" s="1"/>
-      <c r="S45" s="1"/>
-      <c r="T45" s="10">
-        <f t="shared" si="0"/>
-        <v>36</v>
-      </c>
-    </row>
-    <row r="46" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R45" s="1">
+        <v>3</v>
+      </c>
+      <c r="S45" s="1">
+        <v>5</v>
+      </c>
+      <c r="T45" s="1">
+        <v>5</v>
+      </c>
+      <c r="U45" s="10">
+        <f t="shared" si="0"/>
+        <v>49</v>
+      </c>
+    </row>
+    <row r="46" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A46" s="11">
         <v>44</v>
       </c>
@@ -7789,14 +8505,21 @@
       <c r="Q46" s="1">
         <v>5</v>
       </c>
-      <c r="R46" s="1"/>
-      <c r="S46" s="1"/>
-      <c r="T46" s="10">
-        <f t="shared" si="0"/>
-        <v>41</v>
-      </c>
-    </row>
-    <row r="47" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R46" s="1">
+        <v>5</v>
+      </c>
+      <c r="S46" s="1">
+        <v>4</v>
+      </c>
+      <c r="T46" s="1">
+        <v>4</v>
+      </c>
+      <c r="U46" s="10">
+        <f t="shared" si="0"/>
+        <v>54</v>
+      </c>
+    </row>
+    <row r="47" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A47" s="11">
         <v>45</v>
       </c>
@@ -7848,14 +8571,21 @@
       <c r="Q47" s="1">
         <v>5</v>
       </c>
-      <c r="R47" s="1"/>
-      <c r="S47" s="1"/>
-      <c r="T47" s="10">
-        <f t="shared" si="0"/>
-        <v>43</v>
-      </c>
-    </row>
-    <row r="48" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R47" s="1">
+        <v>4</v>
+      </c>
+      <c r="S47" s="1">
+        <v>5</v>
+      </c>
+      <c r="T47" s="1">
+        <v>5</v>
+      </c>
+      <c r="U47" s="10">
+        <f t="shared" si="0"/>
+        <v>57</v>
+      </c>
+    </row>
+    <row r="48" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A48" s="11">
         <v>46</v>
       </c>
@@ -7907,14 +8637,21 @@
       <c r="Q48" s="1">
         <v>0</v>
       </c>
-      <c r="R48" s="1"/>
-      <c r="S48" s="1"/>
-      <c r="T48" s="10">
-        <f t="shared" si="0"/>
-        <v>38</v>
-      </c>
-    </row>
-    <row r="49" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R48" s="1">
+        <v>4</v>
+      </c>
+      <c r="S48" s="1">
+        <v>5</v>
+      </c>
+      <c r="T48" s="1">
+        <v>5</v>
+      </c>
+      <c r="U48" s="10">
+        <f t="shared" si="0"/>
+        <v>52</v>
+      </c>
+    </row>
+    <row r="49" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A49" s="11">
         <v>47</v>
       </c>
@@ -7966,14 +8703,21 @@
       <c r="Q49" s="1">
         <v>0</v>
       </c>
-      <c r="R49" s="1"/>
-      <c r="S49" s="1"/>
-      <c r="T49" s="10">
-        <f t="shared" si="0"/>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="50" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R49" s="1">
+        <v>4</v>
+      </c>
+      <c r="S49" s="1">
+        <v>4</v>
+      </c>
+      <c r="T49" s="1">
+        <v>2</v>
+      </c>
+      <c r="U49" s="10">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="50" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A50" s="11">
         <v>48</v>
       </c>
@@ -8025,14 +8769,21 @@
       <c r="Q50" s="1">
         <v>0</v>
       </c>
-      <c r="R50" s="1"/>
-      <c r="S50" s="1"/>
-      <c r="T50" s="10">
-        <f t="shared" si="0"/>
-        <v>39</v>
-      </c>
-    </row>
-    <row r="51" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="R50" s="1">
+        <v>4</v>
+      </c>
+      <c r="S50" s="1">
+        <v>5</v>
+      </c>
+      <c r="T50" s="1">
+        <v>4</v>
+      </c>
+      <c r="U50" s="10">
+        <f t="shared" si="0"/>
+        <v>52</v>
+      </c>
+    </row>
+    <row r="51" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A51" s="27">
         <v>49</v>
       </c>
@@ -8084,15 +8835,22 @@
       <c r="Q51" s="23">
         <v>5</v>
       </c>
-      <c r="R51" s="23"/>
-      <c r="S51" s="23"/>
-      <c r="T51" s="10">
-        <f t="shared" si="0"/>
-        <v>47</v>
-      </c>
-    </row>
-    <row r="64" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="R64" s="38"/>
+      <c r="R51" s="23">
+        <v>3</v>
+      </c>
+      <c r="S51" s="23">
+        <v>4</v>
+      </c>
+      <c r="T51" s="23">
+        <v>4</v>
+      </c>
+      <c r="U51" s="10">
+        <f t="shared" si="0"/>
+        <v>58</v>
+      </c>
+    </row>
+    <row r="64" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="R64" s="33"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -8100,6 +8858,7 @@
     <mergeCell ref="F1:S1"/>
     <mergeCell ref="A2:B2"/>
   </mergeCells>
+  <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
📊 Update Excel with controls C16, C17, C18
</commit_message>
<xml_diff>
--- a/data/reporte.xlsx
+++ b/data/reporte.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre\OneDrive\Escritorio\Universidad\2026-1\Modelos de Procesos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F53C1042-21C1-492A-9DFE-83ED05AE77EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{491B2D62-519E-4085-84B7-6B1C2E9D242E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EF01AC27-D1AA-450D-80FE-C50ADE1636E7}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="297">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="300">
   <si>
     <t>Puntajes Controles</t>
   </si>
@@ -928,6 +928,15 @@
   </si>
   <si>
     <t>C15</t>
+  </si>
+  <si>
+    <t>C16</t>
+  </si>
+  <si>
+    <t>C17</t>
+  </si>
+  <si>
+    <t>C18</t>
   </si>
 </sst>
 </file>
@@ -1407,6 +1416,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1418,9 +1430,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1805,37 +1814,40 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FAFB6214-215B-45FB-8876-0D7E2F238F6A}">
-  <dimension ref="A1:U58"/>
+  <dimension ref="A1:Z58"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A1" s="34"/>
-      <c r="B1" s="34"/>
+    <row r="1" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="A1" s="35"/>
+      <c r="B1" s="35"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
-      <c r="F1" s="35" t="s">
-        <v>0</v>
-      </c>
-      <c r="G1" s="36"/>
-      <c r="H1" s="36"/>
-      <c r="I1" s="36"/>
-      <c r="J1" s="36"/>
-      <c r="K1" s="36"/>
-      <c r="L1" s="36"/>
-      <c r="M1" s="36"/>
-      <c r="N1" s="36"/>
-      <c r="O1" s="36"/>
-      <c r="P1" s="36"/>
-      <c r="Q1" s="36"/>
-      <c r="R1" s="36"/>
-      <c r="S1" s="37"/>
-      <c r="T1" s="39"/>
-      <c r="U1" s="2"/>
-    </row>
-    <row r="2" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="38"/>
-      <c r="B2" s="38"/>
+      <c r="F1" s="36" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1" s="37"/>
+      <c r="H1" s="37"/>
+      <c r="I1" s="37"/>
+      <c r="J1" s="37"/>
+      <c r="K1" s="37"/>
+      <c r="L1" s="37"/>
+      <c r="M1" s="37"/>
+      <c r="N1" s="37"/>
+      <c r="O1" s="37"/>
+      <c r="P1" s="37"/>
+      <c r="Q1" s="37"/>
+      <c r="R1" s="37"/>
+      <c r="S1" s="38"/>
+      <c r="T1" s="34"/>
+      <c r="U1" s="34"/>
+      <c r="V1" s="34"/>
+      <c r="W1" s="34"/>
+      <c r="X1" s="2"/>
+    </row>
+    <row r="2" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="39"/>
+      <c r="B2" s="39"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -1884,11 +1896,20 @@
       <c r="T2" s="4" t="s">
         <v>296</v>
       </c>
-      <c r="U2" s="5" t="s">
+      <c r="U2" s="4" t="s">
+        <v>297</v>
+      </c>
+      <c r="V2" s="4" t="s">
+        <v>298</v>
+      </c>
+      <c r="W2" s="4" t="s">
+        <v>299</v>
+      </c>
+      <c r="X2" s="5" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A3" s="6">
         <v>1</v>
       </c>
@@ -1949,12 +1970,21 @@
       <c r="T3" s="9">
         <v>5</v>
       </c>
-      <c r="U3" s="10">
-        <f>($F3+$G3+$H3+$I3+$J3+$K3+$L3+$M3+$N3+$O3+$P3+$Q3+$R3+$S3+$T3)</f>
-        <v>46</v>
-      </c>
-    </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U3" s="9">
+        <v>5</v>
+      </c>
+      <c r="V3" s="9">
+        <v>0</v>
+      </c>
+      <c r="W3" s="9">
+        <v>5</v>
+      </c>
+      <c r="X3" s="10">
+        <f>($F3+$G3+$H3+$I3+$J3+$K3+$L3+$M3+$N3+$O3+$P3+$Q3+$R3+$S3+$T3+$U3+$V3+$W3)</f>
+        <v>56</v>
+      </c>
+    </row>
+    <row r="4" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A4" s="11">
         <v>2</v>
       </c>
@@ -2015,12 +2045,21 @@
       <c r="T4" s="1">
         <v>4</v>
       </c>
-      <c r="U4" s="10">
-        <f t="shared" ref="U4:U57" si="0">($F4+$G4+$H4+$I4+$J4+$K4+$L4+$M4+$N4+$O4+$P4+$Q4+$R4+$S4+$T4)</f>
-        <v>38</v>
-      </c>
-    </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U4" s="1">
+        <v>5</v>
+      </c>
+      <c r="V4" s="1">
+        <v>5</v>
+      </c>
+      <c r="W4" s="1">
+        <v>5</v>
+      </c>
+      <c r="X4" s="10">
+        <f t="shared" ref="X4:X57" si="0">($F4+$G4+$H4+$I4+$J4+$K4+$L4+$M4+$N4+$O4+$P4+$Q4+$R4+$S4+$T4+$U4+$V4+$W4)</f>
+        <v>53</v>
+      </c>
+    </row>
+    <row r="5" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A5" s="11">
         <v>3</v>
       </c>
@@ -2081,12 +2120,21 @@
       <c r="T5" s="1">
         <v>2</v>
       </c>
-      <c r="U5" s="10">
-        <f t="shared" si="0"/>
-        <v>31</v>
-      </c>
-    </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U5" s="1">
+        <v>3</v>
+      </c>
+      <c r="V5" s="1">
+        <v>5</v>
+      </c>
+      <c r="W5" s="1">
+        <v>5</v>
+      </c>
+      <c r="X5" s="10">
+        <f t="shared" si="0"/>
+        <v>44</v>
+      </c>
+    </row>
+    <row r="6" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A6" s="11">
         <v>4</v>
       </c>
@@ -2147,12 +2195,21 @@
       <c r="T6" s="1">
         <v>4</v>
       </c>
-      <c r="U6" s="10">
-        <f t="shared" si="0"/>
-        <v>49</v>
-      </c>
-    </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U6" s="1">
+        <v>4</v>
+      </c>
+      <c r="V6" s="1">
+        <v>5</v>
+      </c>
+      <c r="W6" s="1">
+        <v>4</v>
+      </c>
+      <c r="X6" s="10">
+        <f t="shared" si="0"/>
+        <v>62</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A7" s="11">
         <v>5</v>
       </c>
@@ -2213,12 +2270,21 @@
       <c r="T7" s="1">
         <v>5</v>
       </c>
-      <c r="U7" s="10">
-        <f t="shared" si="0"/>
-        <v>46</v>
-      </c>
-    </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U7" s="1">
+        <v>5</v>
+      </c>
+      <c r="V7" s="1">
+        <v>5</v>
+      </c>
+      <c r="W7" s="1">
+        <v>4</v>
+      </c>
+      <c r="X7" s="10">
+        <f t="shared" si="0"/>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="8" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A8" s="11">
         <v>6</v>
       </c>
@@ -2279,12 +2345,21 @@
       <c r="T8" s="1">
         <v>3</v>
       </c>
-      <c r="U8" s="10">
-        <f t="shared" si="0"/>
-        <v>68</v>
-      </c>
-    </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U8" s="1">
+        <v>4</v>
+      </c>
+      <c r="V8" s="1">
+        <v>0</v>
+      </c>
+      <c r="W8" s="1">
+        <v>4</v>
+      </c>
+      <c r="X8" s="10">
+        <f t="shared" si="0"/>
+        <v>76</v>
+      </c>
+    </row>
+    <row r="9" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A9" s="11">
         <v>7</v>
       </c>
@@ -2345,12 +2420,21 @@
       <c r="T9" s="1">
         <v>3</v>
       </c>
-      <c r="U9" s="10">
-        <f t="shared" si="0"/>
-        <v>44</v>
-      </c>
-    </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U9" s="1">
+        <v>0</v>
+      </c>
+      <c r="V9" s="1">
+        <v>5</v>
+      </c>
+      <c r="W9" s="1">
+        <v>5</v>
+      </c>
+      <c r="X9" s="10">
+        <f t="shared" si="0"/>
+        <v>54</v>
+      </c>
+    </row>
+    <row r="10" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A10" s="11">
         <v>8</v>
       </c>
@@ -2411,12 +2495,21 @@
       <c r="T10" s="1">
         <v>0</v>
       </c>
-      <c r="U10" s="10">
-        <f t="shared" si="0"/>
-        <v>30</v>
-      </c>
-    </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U10" s="1">
+        <v>5</v>
+      </c>
+      <c r="V10" s="1">
+        <v>0</v>
+      </c>
+      <c r="W10" s="1">
+        <v>0</v>
+      </c>
+      <c r="X10" s="10">
+        <f t="shared" si="0"/>
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A11" s="11">
         <v>9</v>
       </c>
@@ -2477,12 +2570,22 @@
       <c r="T11" s="1">
         <v>3</v>
       </c>
-      <c r="U11" s="10">
-        <f t="shared" si="0"/>
-        <v>55</v>
-      </c>
-    </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U11" s="1">
+        <v>5</v>
+      </c>
+      <c r="V11" s="1">
+        <v>5</v>
+      </c>
+      <c r="W11" s="1">
+        <v>5</v>
+      </c>
+      <c r="X11" s="10">
+        <f t="shared" si="0"/>
+        <v>70</v>
+      </c>
+      <c r="Z11" s="33"/>
+    </row>
+    <row r="12" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A12" s="11">
         <v>10</v>
       </c>
@@ -2543,12 +2646,21 @@
       <c r="T12" s="1">
         <v>5</v>
       </c>
-      <c r="U12" s="10">
-        <f t="shared" si="0"/>
-        <v>58</v>
-      </c>
-    </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U12" s="1">
+        <v>4</v>
+      </c>
+      <c r="V12" s="1">
+        <v>4</v>
+      </c>
+      <c r="W12" s="1">
+        <v>5</v>
+      </c>
+      <c r="X12" s="10">
+        <f t="shared" si="0"/>
+        <v>71</v>
+      </c>
+    </row>
+    <row r="13" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A13" s="11">
         <v>11</v>
       </c>
@@ -2609,12 +2721,21 @@
       <c r="T13" s="1">
         <v>4</v>
       </c>
-      <c r="U13" s="10">
-        <f t="shared" si="0"/>
-        <v>35</v>
-      </c>
-    </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U13" s="1">
+        <v>5</v>
+      </c>
+      <c r="V13" s="1">
+        <v>0</v>
+      </c>
+      <c r="W13" s="1">
+        <v>5</v>
+      </c>
+      <c r="X13" s="10">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="14" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A14" s="11">
         <v>12</v>
       </c>
@@ -2675,12 +2796,21 @@
       <c r="T14" s="1">
         <v>0</v>
       </c>
-      <c r="U14" s="10">
-        <f t="shared" si="0"/>
-        <v>39</v>
-      </c>
-    </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U14" s="1">
+        <v>5</v>
+      </c>
+      <c r="V14" s="1">
+        <v>5</v>
+      </c>
+      <c r="W14" s="1">
+        <v>5</v>
+      </c>
+      <c r="X14" s="10">
+        <f t="shared" si="0"/>
+        <v>54</v>
+      </c>
+    </row>
+    <row r="15" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A15" s="11">
         <v>13</v>
       </c>
@@ -2741,12 +2871,21 @@
       <c r="T15" s="1">
         <v>3</v>
       </c>
-      <c r="U15" s="10">
-        <f t="shared" si="0"/>
-        <v>43</v>
-      </c>
-    </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U15" s="1">
+        <v>4</v>
+      </c>
+      <c r="V15" s="1">
+        <v>5</v>
+      </c>
+      <c r="W15" s="1">
+        <v>3</v>
+      </c>
+      <c r="X15" s="10">
+        <f t="shared" si="0"/>
+        <v>55</v>
+      </c>
+    </row>
+    <row r="16" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A16" s="11">
         <v>14</v>
       </c>
@@ -2807,12 +2946,21 @@
       <c r="T16" s="1">
         <v>0</v>
       </c>
-      <c r="U16" s="10">
-        <f t="shared" si="0"/>
-        <v>43</v>
-      </c>
-    </row>
-    <row r="17" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U16" s="1">
+        <v>5</v>
+      </c>
+      <c r="V16" s="1">
+        <v>5</v>
+      </c>
+      <c r="W16" s="1">
+        <v>5</v>
+      </c>
+      <c r="X16" s="10">
+        <f t="shared" si="0"/>
+        <v>58</v>
+      </c>
+    </row>
+    <row r="17" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A17" s="11">
         <v>15</v>
       </c>
@@ -2873,12 +3021,21 @@
       <c r="T17" s="1">
         <v>0</v>
       </c>
-      <c r="U17" s="10">
-        <f t="shared" si="0"/>
-        <v>40</v>
-      </c>
-    </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U17" s="1">
+        <v>3</v>
+      </c>
+      <c r="V17" s="1">
+        <v>0</v>
+      </c>
+      <c r="W17" s="1">
+        <v>4</v>
+      </c>
+      <c r="X17" s="10">
+        <f t="shared" si="0"/>
+        <v>47</v>
+      </c>
+    </row>
+    <row r="18" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A18" s="11">
         <v>16</v>
       </c>
@@ -2939,12 +3096,21 @@
       <c r="T18" s="1">
         <v>0</v>
       </c>
-      <c r="U18" s="10">
-        <f t="shared" si="0"/>
-        <v>46</v>
-      </c>
-    </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U18" s="1">
+        <v>5</v>
+      </c>
+      <c r="V18" s="1">
+        <v>0</v>
+      </c>
+      <c r="W18" s="1">
+        <v>3</v>
+      </c>
+      <c r="X18" s="10">
+        <f t="shared" si="0"/>
+        <v>54</v>
+      </c>
+    </row>
+    <row r="19" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A19" s="11">
         <v>17</v>
       </c>
@@ -3005,12 +3171,21 @@
       <c r="T19" s="1">
         <v>3</v>
       </c>
-      <c r="U19" s="10">
-        <f t="shared" si="0"/>
-        <v>39</v>
-      </c>
-    </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U19" s="1">
+        <v>3</v>
+      </c>
+      <c r="V19" s="1">
+        <v>3</v>
+      </c>
+      <c r="W19" s="1">
+        <v>5</v>
+      </c>
+      <c r="X19" s="10">
+        <f t="shared" si="0"/>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="20" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A20" s="11">
         <v>18</v>
       </c>
@@ -3071,12 +3246,21 @@
       <c r="T20" s="1">
         <v>3</v>
       </c>
-      <c r="U20" s="10">
-        <f t="shared" si="0"/>
-        <v>52</v>
-      </c>
-    </row>
-    <row r="21" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U20" s="1">
+        <v>3</v>
+      </c>
+      <c r="V20" s="1">
+        <v>5</v>
+      </c>
+      <c r="W20" s="1">
+        <v>4</v>
+      </c>
+      <c r="X20" s="10">
+        <f t="shared" si="0"/>
+        <v>64</v>
+      </c>
+    </row>
+    <row r="21" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A21" s="11">
         <v>19</v>
       </c>
@@ -3137,12 +3321,21 @@
       <c r="T21" s="1">
         <v>0</v>
       </c>
-      <c r="U21" s="10">
-        <f t="shared" si="0"/>
-        <v>44</v>
-      </c>
-    </row>
-    <row r="22" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U21" s="1">
+        <v>5</v>
+      </c>
+      <c r="V21" s="1">
+        <v>0</v>
+      </c>
+      <c r="W21" s="1">
+        <v>0</v>
+      </c>
+      <c r="X21" s="10">
+        <f t="shared" si="0"/>
+        <v>49</v>
+      </c>
+    </row>
+    <row r="22" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A22" s="11">
         <v>20</v>
       </c>
@@ -3203,12 +3396,21 @@
       <c r="T22" s="1">
         <v>0</v>
       </c>
-      <c r="U22" s="10">
-        <f t="shared" si="0"/>
-        <v>47</v>
-      </c>
-    </row>
-    <row r="23" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U22" s="1">
+        <v>3</v>
+      </c>
+      <c r="V22" s="1">
+        <v>0</v>
+      </c>
+      <c r="W22" s="1">
+        <v>4</v>
+      </c>
+      <c r="X22" s="10">
+        <f t="shared" si="0"/>
+        <v>54</v>
+      </c>
+    </row>
+    <row r="23" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A23" s="11">
         <v>21</v>
       </c>
@@ -3269,12 +3471,21 @@
       <c r="T23" s="1">
         <v>1</v>
       </c>
-      <c r="U23" s="10">
-        <f t="shared" si="0"/>
-        <v>44</v>
-      </c>
-    </row>
-    <row r="24" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U23" s="1">
+        <v>4</v>
+      </c>
+      <c r="V23" s="1">
+        <v>5</v>
+      </c>
+      <c r="W23" s="1">
+        <v>1</v>
+      </c>
+      <c r="X23" s="10">
+        <f t="shared" si="0"/>
+        <v>54</v>
+      </c>
+    </row>
+    <row r="24" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A24" s="11">
         <v>22</v>
       </c>
@@ -3335,12 +3546,21 @@
       <c r="T24" s="1">
         <v>0</v>
       </c>
-      <c r="U24" s="10">
+      <c r="U24" s="1">
+        <v>0</v>
+      </c>
+      <c r="V24" s="1">
+        <v>0</v>
+      </c>
+      <c r="W24" s="1">
+        <v>0</v>
+      </c>
+      <c r="X24" s="10">
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
     </row>
-    <row r="25" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A25" s="11">
         <v>23</v>
       </c>
@@ -3401,12 +3621,21 @@
       <c r="T25" s="1">
         <v>0</v>
       </c>
-      <c r="U25" s="10">
-        <f t="shared" si="0"/>
-        <v>33</v>
-      </c>
-    </row>
-    <row r="26" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U25" s="1">
+        <v>5</v>
+      </c>
+      <c r="V25" s="1">
+        <v>3</v>
+      </c>
+      <c r="W25" s="1">
+        <v>0</v>
+      </c>
+      <c r="X25" s="10">
+        <f t="shared" si="0"/>
+        <v>41</v>
+      </c>
+    </row>
+    <row r="26" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A26" s="11">
         <v>24</v>
       </c>
@@ -3467,12 +3696,21 @@
       <c r="T26" s="1">
         <v>0</v>
       </c>
-      <c r="U26" s="10">
-        <f t="shared" si="0"/>
-        <v>28</v>
-      </c>
-    </row>
-    <row r="27" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U26" s="1">
+        <v>5</v>
+      </c>
+      <c r="V26" s="1">
+        <v>5</v>
+      </c>
+      <c r="W26" s="1">
+        <v>5</v>
+      </c>
+      <c r="X26" s="10">
+        <f t="shared" si="0"/>
+        <v>43</v>
+      </c>
+    </row>
+    <row r="27" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A27" s="11">
         <v>25</v>
       </c>
@@ -3533,12 +3771,21 @@
       <c r="T27" s="1">
         <v>0</v>
       </c>
-      <c r="U27" s="10">
-        <f t="shared" si="0"/>
-        <v>43</v>
-      </c>
-    </row>
-    <row r="28" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U27" s="1">
+        <v>5</v>
+      </c>
+      <c r="V27" s="1">
+        <v>5</v>
+      </c>
+      <c r="W27" s="1">
+        <v>5</v>
+      </c>
+      <c r="X27" s="10">
+        <f t="shared" si="0"/>
+        <v>58</v>
+      </c>
+    </row>
+    <row r="28" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A28" s="11">
         <v>26</v>
       </c>
@@ -3599,12 +3846,21 @@
       <c r="T28" s="1">
         <v>3</v>
       </c>
-      <c r="U28" s="10">
-        <f t="shared" si="0"/>
-        <v>47</v>
-      </c>
-    </row>
-    <row r="29" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U28" s="1">
+        <v>3</v>
+      </c>
+      <c r="V28" s="1">
+        <v>5</v>
+      </c>
+      <c r="W28" s="1">
+        <v>4</v>
+      </c>
+      <c r="X28" s="10">
+        <f t="shared" si="0"/>
+        <v>59</v>
+      </c>
+    </row>
+    <row r="29" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A29" s="11">
         <v>27</v>
       </c>
@@ -3665,12 +3921,21 @@
       <c r="T29" s="1">
         <v>5</v>
       </c>
-      <c r="U29" s="10">
-        <f t="shared" si="0"/>
-        <v>59</v>
-      </c>
-    </row>
-    <row r="30" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U29" s="1">
+        <v>5</v>
+      </c>
+      <c r="V29" s="1">
+        <v>5</v>
+      </c>
+      <c r="W29" s="1">
+        <v>0</v>
+      </c>
+      <c r="X29" s="10">
+        <f t="shared" si="0"/>
+        <v>69</v>
+      </c>
+    </row>
+    <row r="30" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A30" s="11">
         <v>28</v>
       </c>
@@ -3731,12 +3996,21 @@
       <c r="T30" s="1">
         <v>0</v>
       </c>
-      <c r="U30" s="10">
+      <c r="U30" s="1">
+        <v>0</v>
+      </c>
+      <c r="V30" s="1">
+        <v>0</v>
+      </c>
+      <c r="W30" s="1">
+        <v>0</v>
+      </c>
+      <c r="X30" s="10">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
     </row>
-    <row r="31" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A31" s="11">
         <v>29</v>
       </c>
@@ -3797,12 +4071,21 @@
       <c r="T31" s="1">
         <v>5</v>
       </c>
-      <c r="U31" s="10">
-        <f t="shared" si="0"/>
-        <v>53</v>
-      </c>
-    </row>
-    <row r="32" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U31" s="1">
+        <v>5</v>
+      </c>
+      <c r="V31" s="1">
+        <v>5</v>
+      </c>
+      <c r="W31" s="1">
+        <v>5</v>
+      </c>
+      <c r="X31" s="10">
+        <f t="shared" si="0"/>
+        <v>68</v>
+      </c>
+    </row>
+    <row r="32" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A32" s="11">
         <v>30</v>
       </c>
@@ -3863,12 +4146,21 @@
       <c r="T32" s="1">
         <v>5</v>
       </c>
-      <c r="U32" s="10">
-        <f t="shared" si="0"/>
-        <v>43</v>
-      </c>
-    </row>
-    <row r="33" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U32" s="1">
+        <v>3</v>
+      </c>
+      <c r="V32" s="1">
+        <v>0</v>
+      </c>
+      <c r="W32" s="1">
+        <v>0</v>
+      </c>
+      <c r="X32" s="10">
+        <f t="shared" si="0"/>
+        <v>46</v>
+      </c>
+    </row>
+    <row r="33" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A33" s="11">
         <v>31</v>
       </c>
@@ -3929,12 +4221,21 @@
       <c r="T33" s="1">
         <v>4</v>
       </c>
-      <c r="U33" s="10">
-        <f t="shared" si="0"/>
-        <v>64</v>
-      </c>
-    </row>
-    <row r="34" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U33" s="1">
+        <v>5</v>
+      </c>
+      <c r="V33" s="1">
+        <v>0</v>
+      </c>
+      <c r="W33" s="1">
+        <v>0</v>
+      </c>
+      <c r="X33" s="10">
+        <f t="shared" si="0"/>
+        <v>69</v>
+      </c>
+    </row>
+    <row r="34" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A34" s="11">
         <v>32</v>
       </c>
@@ -3995,12 +4296,21 @@
       <c r="T34" s="1">
         <v>5</v>
       </c>
-      <c r="U34" s="10">
-        <f t="shared" si="0"/>
-        <v>59</v>
-      </c>
-    </row>
-    <row r="35" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U34" s="1">
+        <v>5</v>
+      </c>
+      <c r="V34" s="1">
+        <v>0</v>
+      </c>
+      <c r="W34" s="1">
+        <v>0</v>
+      </c>
+      <c r="X34" s="10">
+        <f t="shared" si="0"/>
+        <v>64</v>
+      </c>
+    </row>
+    <row r="35" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A35" s="11">
         <v>33</v>
       </c>
@@ -4061,12 +4371,21 @@
       <c r="T35" s="1">
         <v>5</v>
       </c>
-      <c r="U35" s="10">
-        <f t="shared" si="0"/>
-        <v>51</v>
-      </c>
-    </row>
-    <row r="36" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U35" s="1">
+        <v>5</v>
+      </c>
+      <c r="V35" s="1">
+        <v>5</v>
+      </c>
+      <c r="W35" s="1">
+        <v>4</v>
+      </c>
+      <c r="X35" s="10">
+        <f t="shared" si="0"/>
+        <v>65</v>
+      </c>
+    </row>
+    <row r="36" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A36" s="11">
         <v>34</v>
       </c>
@@ -4127,12 +4446,21 @@
       <c r="T36" s="1">
         <v>3</v>
       </c>
-      <c r="U36" s="10">
-        <f t="shared" si="0"/>
-        <v>48</v>
-      </c>
-    </row>
-    <row r="37" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U36" s="1">
+        <v>3</v>
+      </c>
+      <c r="V36" s="1">
+        <v>0</v>
+      </c>
+      <c r="W36" s="1">
+        <v>5</v>
+      </c>
+      <c r="X36" s="10">
+        <f t="shared" si="0"/>
+        <v>56</v>
+      </c>
+    </row>
+    <row r="37" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A37" s="11">
         <v>35</v>
       </c>
@@ -4193,12 +4521,21 @@
       <c r="T37" s="1">
         <v>5</v>
       </c>
-      <c r="U37" s="10">
-        <f t="shared" si="0"/>
-        <v>47</v>
-      </c>
-    </row>
-    <row r="38" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U37" s="1">
+        <v>5</v>
+      </c>
+      <c r="V37" s="1">
+        <v>5</v>
+      </c>
+      <c r="W37" s="1">
+        <v>0</v>
+      </c>
+      <c r="X37" s="10">
+        <f t="shared" si="0"/>
+        <v>57</v>
+      </c>
+    </row>
+    <row r="38" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A38" s="11">
         <v>36</v>
       </c>
@@ -4259,12 +4596,21 @@
       <c r="T38" s="1">
         <v>0</v>
       </c>
-      <c r="U38" s="10">
-        <f t="shared" si="0"/>
-        <v>21</v>
-      </c>
-    </row>
-    <row r="39" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U38" s="1">
+        <v>4</v>
+      </c>
+      <c r="V38" s="1">
+        <v>5</v>
+      </c>
+      <c r="W38" s="1">
+        <v>5</v>
+      </c>
+      <c r="X38" s="10">
+        <f t="shared" si="0"/>
+        <v>35</v>
+      </c>
+    </row>
+    <row r="39" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A39" s="11">
         <v>37</v>
       </c>
@@ -4325,12 +4671,21 @@
       <c r="T39" s="1">
         <v>4</v>
       </c>
-      <c r="U39" s="10">
-        <f t="shared" si="0"/>
-        <v>60</v>
-      </c>
-    </row>
-    <row r="40" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U39" s="1">
+        <v>4</v>
+      </c>
+      <c r="V39" s="1">
+        <v>0</v>
+      </c>
+      <c r="W39" s="1">
+        <v>4</v>
+      </c>
+      <c r="X39" s="10">
+        <f t="shared" si="0"/>
+        <v>68</v>
+      </c>
+    </row>
+    <row r="40" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A40" s="11">
         <v>38</v>
       </c>
@@ -4391,12 +4746,21 @@
       <c r="T40" s="1">
         <v>5</v>
       </c>
-      <c r="U40" s="10">
-        <f t="shared" si="0"/>
-        <v>35</v>
-      </c>
-    </row>
-    <row r="41" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U40" s="1">
+        <v>3</v>
+      </c>
+      <c r="V40" s="1">
+        <v>5</v>
+      </c>
+      <c r="W40" s="1">
+        <v>0</v>
+      </c>
+      <c r="X40" s="10">
+        <f t="shared" si="0"/>
+        <v>43</v>
+      </c>
+    </row>
+    <row r="41" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A41" s="11">
         <v>39</v>
       </c>
@@ -4457,12 +4821,21 @@
       <c r="T41" s="1">
         <v>3</v>
       </c>
-      <c r="U41" s="10">
-        <f t="shared" si="0"/>
-        <v>13</v>
-      </c>
-    </row>
-    <row r="42" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U41" s="1">
+        <v>4</v>
+      </c>
+      <c r="V41" s="1">
+        <v>4</v>
+      </c>
+      <c r="W41" s="1">
+        <v>2</v>
+      </c>
+      <c r="X41" s="10">
+        <f t="shared" si="0"/>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="42" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A42" s="11">
         <v>40</v>
       </c>
@@ -4523,12 +4896,21 @@
       <c r="T42" s="1">
         <v>0</v>
       </c>
-      <c r="U42" s="10">
-        <f t="shared" si="0"/>
-        <v>27</v>
-      </c>
-    </row>
-    <row r="43" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U42" s="1">
+        <v>4</v>
+      </c>
+      <c r="V42" s="1">
+        <v>0</v>
+      </c>
+      <c r="W42" s="1">
+        <v>0</v>
+      </c>
+      <c r="X42" s="10">
+        <f t="shared" si="0"/>
+        <v>31</v>
+      </c>
+    </row>
+    <row r="43" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A43" s="11">
         <v>41</v>
       </c>
@@ -4589,12 +4971,21 @@
       <c r="T43" s="1">
         <v>0</v>
       </c>
-      <c r="U43" s="10">
-        <f t="shared" si="0"/>
-        <v>48</v>
-      </c>
-    </row>
-    <row r="44" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U43" s="1">
+        <v>5</v>
+      </c>
+      <c r="V43" s="1">
+        <v>0</v>
+      </c>
+      <c r="W43" s="1">
+        <v>4</v>
+      </c>
+      <c r="X43" s="10">
+        <f t="shared" si="0"/>
+        <v>57</v>
+      </c>
+    </row>
+    <row r="44" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A44" s="11">
         <v>42</v>
       </c>
@@ -4655,12 +5046,21 @@
       <c r="T44" s="1">
         <v>0</v>
       </c>
-      <c r="U44" s="10">
-        <f t="shared" si="0"/>
-        <v>35</v>
-      </c>
-    </row>
-    <row r="45" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U44" s="1">
+        <v>5</v>
+      </c>
+      <c r="V44" s="1">
+        <v>5</v>
+      </c>
+      <c r="W44" s="1">
+        <v>5</v>
+      </c>
+      <c r="X44" s="10">
+        <f t="shared" si="0"/>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="45" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A45" s="11">
         <v>43</v>
       </c>
@@ -4721,12 +5121,21 @@
       <c r="T45" s="1">
         <v>3</v>
       </c>
-      <c r="U45" s="10">
-        <f t="shared" si="0"/>
-        <v>44</v>
-      </c>
-    </row>
-    <row r="46" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U45" s="1">
+        <v>4</v>
+      </c>
+      <c r="V45" s="1">
+        <v>5</v>
+      </c>
+      <c r="W45" s="1">
+        <v>5</v>
+      </c>
+      <c r="X45" s="10">
+        <f t="shared" si="0"/>
+        <v>58</v>
+      </c>
+    </row>
+    <row r="46" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A46" s="11">
         <v>44</v>
       </c>
@@ -4787,12 +5196,21 @@
       <c r="T46" s="1">
         <v>0</v>
       </c>
-      <c r="U46" s="10">
-        <f t="shared" si="0"/>
-        <v>50</v>
-      </c>
-    </row>
-    <row r="47" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U46" s="1">
+        <v>4</v>
+      </c>
+      <c r="V46" s="1">
+        <v>5</v>
+      </c>
+      <c r="W46" s="1">
+        <v>4</v>
+      </c>
+      <c r="X46" s="10">
+        <f t="shared" si="0"/>
+        <v>63</v>
+      </c>
+    </row>
+    <row r="47" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A47" s="11">
         <v>45</v>
       </c>
@@ -4853,12 +5271,21 @@
       <c r="T47" s="1">
         <v>5</v>
       </c>
-      <c r="U47" s="10">
-        <f t="shared" si="0"/>
-        <v>58</v>
-      </c>
-    </row>
-    <row r="48" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U47" s="1">
+        <v>5</v>
+      </c>
+      <c r="V47" s="1">
+        <v>5</v>
+      </c>
+      <c r="W47" s="1">
+        <v>5</v>
+      </c>
+      <c r="X47" s="10">
+        <f t="shared" si="0"/>
+        <v>73</v>
+      </c>
+    </row>
+    <row r="48" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A48" s="11">
         <v>46</v>
       </c>
@@ -4919,12 +5346,21 @@
       <c r="T48" s="1">
         <v>0</v>
       </c>
-      <c r="U48" s="10">
-        <f t="shared" si="0"/>
-        <v>57</v>
-      </c>
-    </row>
-    <row r="49" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U48" s="1">
+        <v>5</v>
+      </c>
+      <c r="V48" s="1">
+        <v>5</v>
+      </c>
+      <c r="W48" s="1">
+        <v>5</v>
+      </c>
+      <c r="X48" s="10">
+        <f t="shared" si="0"/>
+        <v>72</v>
+      </c>
+    </row>
+    <row r="49" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A49" s="11">
         <v>47</v>
       </c>
@@ -4985,12 +5421,21 @@
       <c r="T49" s="1">
         <v>0</v>
       </c>
-      <c r="U49" s="10">
-        <f t="shared" si="0"/>
-        <v>45</v>
-      </c>
-    </row>
-    <row r="50" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U49" s="1">
+        <v>5</v>
+      </c>
+      <c r="V49" s="1">
+        <v>5</v>
+      </c>
+      <c r="W49" s="1">
+        <v>5</v>
+      </c>
+      <c r="X49" s="10">
+        <f t="shared" si="0"/>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="50" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A50" s="11">
         <v>48</v>
       </c>
@@ -5051,12 +5496,21 @@
       <c r="T50" s="1">
         <v>4</v>
       </c>
-      <c r="U50" s="10">
-        <f t="shared" si="0"/>
-        <v>54</v>
-      </c>
-    </row>
-    <row r="51" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U50" s="1">
+        <v>5</v>
+      </c>
+      <c r="V50" s="1">
+        <v>0</v>
+      </c>
+      <c r="W50" s="1">
+        <v>0</v>
+      </c>
+      <c r="X50" s="10">
+        <f t="shared" si="0"/>
+        <v>59</v>
+      </c>
+    </row>
+    <row r="51" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A51" s="11">
         <v>49</v>
       </c>
@@ -5117,12 +5571,21 @@
       <c r="T51" s="1">
         <v>2</v>
       </c>
-      <c r="U51" s="10">
-        <f t="shared" si="0"/>
-        <v>32</v>
-      </c>
-    </row>
-    <row r="52" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U51" s="1">
+        <v>3</v>
+      </c>
+      <c r="V51" s="1">
+        <v>3</v>
+      </c>
+      <c r="W51" s="1">
+        <v>4</v>
+      </c>
+      <c r="X51" s="10">
+        <f t="shared" si="0"/>
+        <v>42</v>
+      </c>
+    </row>
+    <row r="52" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A52" s="11">
         <v>50</v>
       </c>
@@ -5183,12 +5646,21 @@
       <c r="T52" s="1">
         <v>5</v>
       </c>
-      <c r="U52" s="10">
-        <f t="shared" si="0"/>
-        <v>46</v>
-      </c>
-    </row>
-    <row r="53" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U52" s="1">
+        <v>5</v>
+      </c>
+      <c r="V52" s="1">
+        <v>3</v>
+      </c>
+      <c r="W52" s="1">
+        <v>0</v>
+      </c>
+      <c r="X52" s="10">
+        <f t="shared" si="0"/>
+        <v>54</v>
+      </c>
+    </row>
+    <row r="53" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A53" s="11">
         <v>51</v>
       </c>
@@ -5249,12 +5721,21 @@
       <c r="T53" s="1">
         <v>0</v>
       </c>
-      <c r="U53" s="10">
-        <f t="shared" si="0"/>
-        <v>54</v>
-      </c>
-    </row>
-    <row r="54" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U53" s="1">
+        <v>4</v>
+      </c>
+      <c r="V53" s="1">
+        <v>5</v>
+      </c>
+      <c r="W53" s="1">
+        <v>3</v>
+      </c>
+      <c r="X53" s="10">
+        <f t="shared" si="0"/>
+        <v>66</v>
+      </c>
+    </row>
+    <row r="54" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A54" s="11">
         <v>52</v>
       </c>
@@ -5315,12 +5796,21 @@
       <c r="T54" s="1">
         <v>5</v>
       </c>
-      <c r="U54" s="10">
-        <f t="shared" si="0"/>
-        <v>64</v>
-      </c>
-    </row>
-    <row r="55" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U54" s="1">
+        <v>3</v>
+      </c>
+      <c r="V54" s="1">
+        <v>5</v>
+      </c>
+      <c r="W54" s="1">
+        <v>4</v>
+      </c>
+      <c r="X54" s="10">
+        <f t="shared" si="0"/>
+        <v>76</v>
+      </c>
+    </row>
+    <row r="55" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A55" s="11">
         <v>53</v>
       </c>
@@ -5381,12 +5871,21 @@
       <c r="T55" s="1">
         <v>5</v>
       </c>
-      <c r="U55" s="10">
-        <f t="shared" si="0"/>
-        <v>68</v>
-      </c>
-    </row>
-    <row r="56" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U55" s="1">
+        <v>5</v>
+      </c>
+      <c r="V55" s="1">
+        <v>5</v>
+      </c>
+      <c r="W55" s="1">
+        <v>5</v>
+      </c>
+      <c r="X55" s="10">
+        <f t="shared" si="0"/>
+        <v>83</v>
+      </c>
+    </row>
+    <row r="56" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A56" s="11">
         <v>54</v>
       </c>
@@ -5447,12 +5946,21 @@
       <c r="T56" s="1">
         <v>4</v>
       </c>
-      <c r="U56" s="10">
-        <f t="shared" si="0"/>
-        <v>61</v>
-      </c>
-    </row>
-    <row r="57" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="U56" s="1">
+        <v>5</v>
+      </c>
+      <c r="V56" s="1">
+        <v>5</v>
+      </c>
+      <c r="W56" s="1">
+        <v>5</v>
+      </c>
+      <c r="X56" s="10">
+        <f t="shared" si="0"/>
+        <v>76</v>
+      </c>
+    </row>
+    <row r="57" spans="1:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A57" s="19">
         <v>55</v>
       </c>
@@ -5513,12 +6021,21 @@
       <c r="T57" s="22">
         <v>2</v>
       </c>
-      <c r="U57" s="10">
-        <f>($F57+$G57+$H57+$I57+$J57+$K57+$L57+$M57+$N57+$O57+$P57+$Q57+$R57+$S57+$T57)</f>
-        <v>55</v>
-      </c>
-    </row>
-    <row r="58" spans="1:21" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+      <c r="U57" s="22">
+        <v>5</v>
+      </c>
+      <c r="V57" s="22">
+        <v>4</v>
+      </c>
+      <c r="W57" s="22">
+        <v>0</v>
+      </c>
+      <c r="X57" s="10">
+        <f t="shared" si="0"/>
+        <v>64</v>
+      </c>
+    </row>
+    <row r="58" spans="1:24" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:B1"/>
@@ -5532,37 +6049,40 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7CD6AE0E-6B38-4517-9EE7-74576DF1F95D}">
-  <dimension ref="A1:U64"/>
+  <dimension ref="A1:AB64"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A1" s="34"/>
-      <c r="B1" s="34"/>
+    <row r="1" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A1" s="35"/>
+      <c r="B1" s="35"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
-      <c r="F1" s="35" t="s">
-        <v>0</v>
-      </c>
-      <c r="G1" s="36"/>
-      <c r="H1" s="36"/>
-      <c r="I1" s="36"/>
-      <c r="J1" s="36"/>
-      <c r="K1" s="36"/>
-      <c r="L1" s="36"/>
-      <c r="M1" s="36"/>
-      <c r="N1" s="36"/>
-      <c r="O1" s="36"/>
-      <c r="P1" s="36"/>
-      <c r="Q1" s="36"/>
-      <c r="R1" s="36"/>
-      <c r="S1" s="37"/>
-      <c r="T1" s="39"/>
-      <c r="U1" s="2"/>
-    </row>
-    <row r="2" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="34"/>
-      <c r="B2" s="34"/>
+      <c r="F1" s="36" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1" s="37"/>
+      <c r="H1" s="37"/>
+      <c r="I1" s="37"/>
+      <c r="J1" s="37"/>
+      <c r="K1" s="37"/>
+      <c r="L1" s="37"/>
+      <c r="M1" s="37"/>
+      <c r="N1" s="37"/>
+      <c r="O1" s="37"/>
+      <c r="P1" s="37"/>
+      <c r="Q1" s="37"/>
+      <c r="R1" s="37"/>
+      <c r="S1" s="38"/>
+      <c r="T1" s="34"/>
+      <c r="U1" s="34"/>
+      <c r="V1" s="34"/>
+      <c r="W1" s="34"/>
+      <c r="X1" s="2"/>
+    </row>
+    <row r="2" spans="1:28" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="35"/>
+      <c r="B2" s="35"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -5611,11 +6131,20 @@
       <c r="T2" s="32" t="s">
         <v>296</v>
       </c>
-      <c r="U2" s="5" t="s">
+      <c r="U2" s="32" t="s">
+        <v>297</v>
+      </c>
+      <c r="V2" s="32" t="s">
+        <v>298</v>
+      </c>
+      <c r="W2" s="32" t="s">
+        <v>299</v>
+      </c>
+      <c r="X2" s="5" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A3" s="11">
         <v>1</v>
       </c>
@@ -5676,12 +6205,21 @@
       <c r="T3" s="1">
         <v>0</v>
       </c>
-      <c r="U3" s="10">
-        <f>($F3+$G3+$H3+$I3+$J3+$K3+$L3+$M3+$N3+$O3+$P3+$Q3+$R3+$S3+$T3)</f>
-        <v>40</v>
-      </c>
-    </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U3" s="1">
+        <v>0</v>
+      </c>
+      <c r="V3" s="1">
+        <v>5</v>
+      </c>
+      <c r="W3" s="1">
+        <v>4</v>
+      </c>
+      <c r="X3" s="10">
+        <f>($F3+$G3+$H3+$I3+$J3+$K3+$L3+$M3+$N3+$O3+$P3+$Q3+$R3+$S3+$T3+$U3+$V3+$W3)</f>
+        <v>49</v>
+      </c>
+    </row>
+    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A4" s="11">
         <v>2</v>
       </c>
@@ -5742,12 +6280,21 @@
       <c r="T4" s="1">
         <v>4</v>
       </c>
-      <c r="U4" s="10">
-        <f t="shared" ref="U4:U51" si="0">($F4+$G4+$H4+$I4+$J4+$K4+$L4+$M4+$N4+$O4+$P4+$Q4+$R4+$S4+$T4)</f>
-        <v>41</v>
-      </c>
-    </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U4" s="1">
+        <v>2</v>
+      </c>
+      <c r="V4" s="1">
+        <v>4</v>
+      </c>
+      <c r="W4" s="1">
+        <v>0</v>
+      </c>
+      <c r="X4" s="10">
+        <f t="shared" ref="X4:X51" si="0">($F4+$G4+$H4+$I4+$J4+$K4+$L4+$M4+$N4+$O4+$P4+$Q4+$R4+$S4+$T4+$U4+$V4+$W4)</f>
+        <v>47</v>
+      </c>
+    </row>
+    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A5" s="11">
         <v>3</v>
       </c>
@@ -5808,12 +6355,21 @@
       <c r="T5" s="1">
         <v>0</v>
       </c>
-      <c r="U5" s="10">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U5" s="1">
+        <v>0</v>
+      </c>
+      <c r="V5" s="1">
+        <v>0</v>
+      </c>
+      <c r="W5" s="1">
+        <v>0</v>
+      </c>
+      <c r="X5" s="10">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A6" s="11">
         <v>4</v>
       </c>
@@ -5874,12 +6430,21 @@
       <c r="T6" s="1">
         <v>0</v>
       </c>
-      <c r="U6" s="10">
+      <c r="U6" s="1">
+        <v>0</v>
+      </c>
+      <c r="V6" s="1">
+        <v>0</v>
+      </c>
+      <c r="W6" s="1">
+        <v>0</v>
+      </c>
+      <c r="X6" s="10">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A7" s="11">
         <v>5</v>
       </c>
@@ -5940,12 +6505,21 @@
       <c r="T7" s="1">
         <v>4</v>
       </c>
-      <c r="U7" s="10">
-        <f t="shared" si="0"/>
-        <v>59</v>
-      </c>
-    </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U7" s="1">
+        <v>5</v>
+      </c>
+      <c r="V7" s="1">
+        <v>5</v>
+      </c>
+      <c r="W7" s="1">
+        <v>0</v>
+      </c>
+      <c r="X7" s="10">
+        <f t="shared" si="0"/>
+        <v>69</v>
+      </c>
+    </row>
+    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A8" s="11">
         <v>6</v>
       </c>
@@ -6006,12 +6580,22 @@
       <c r="T8" s="1">
         <v>4</v>
       </c>
-      <c r="U8" s="10">
-        <f t="shared" si="0"/>
-        <v>30</v>
-      </c>
-    </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U8" s="1">
+        <v>4</v>
+      </c>
+      <c r="V8" s="1">
+        <v>5</v>
+      </c>
+      <c r="W8" s="1">
+        <v>0</v>
+      </c>
+      <c r="X8" s="10">
+        <f t="shared" si="0"/>
+        <v>39</v>
+      </c>
+      <c r="AA8" s="33"/>
+    </row>
+    <row r="9" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A9" s="11">
         <v>7</v>
       </c>
@@ -6072,12 +6656,22 @@
       <c r="T9" s="1">
         <v>5</v>
       </c>
-      <c r="U9" s="10">
-        <f t="shared" si="0"/>
-        <v>62</v>
-      </c>
-    </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U9" s="1">
+        <v>5</v>
+      </c>
+      <c r="V9" s="1">
+        <v>5</v>
+      </c>
+      <c r="W9" s="1">
+        <v>5</v>
+      </c>
+      <c r="X9" s="10">
+        <f t="shared" si="0"/>
+        <v>77</v>
+      </c>
+      <c r="AB9" s="33"/>
+    </row>
+    <row r="10" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A10" s="11">
         <v>8</v>
       </c>
@@ -6138,12 +6732,21 @@
       <c r="T10" s="1">
         <v>1</v>
       </c>
-      <c r="U10" s="10">
-        <f t="shared" si="0"/>
-        <v>23</v>
-      </c>
-    </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U10" s="1">
+        <v>0</v>
+      </c>
+      <c r="V10" s="1">
+        <v>5</v>
+      </c>
+      <c r="W10" s="1">
+        <v>0</v>
+      </c>
+      <c r="X10" s="10">
+        <f t="shared" si="0"/>
+        <v>28</v>
+      </c>
+    </row>
+    <row r="11" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A11" s="11">
         <v>9</v>
       </c>
@@ -6204,12 +6807,22 @@
       <c r="T11" s="1">
         <v>5</v>
       </c>
-      <c r="U11" s="10">
-        <f t="shared" si="0"/>
-        <v>41</v>
-      </c>
-    </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U11" s="1">
+        <v>5</v>
+      </c>
+      <c r="V11" s="1">
+        <v>5</v>
+      </c>
+      <c r="W11" s="1">
+        <v>5</v>
+      </c>
+      <c r="X11" s="10">
+        <f t="shared" si="0"/>
+        <v>56</v>
+      </c>
+      <c r="AA11" s="33"/>
+    </row>
+    <row r="12" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A12" s="11">
         <v>10</v>
       </c>
@@ -6270,12 +6883,21 @@
       <c r="T12" s="1">
         <v>4</v>
       </c>
-      <c r="U12" s="10">
-        <f t="shared" si="0"/>
-        <v>58</v>
-      </c>
-    </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U12" s="1">
+        <v>3</v>
+      </c>
+      <c r="V12" s="1">
+        <v>4</v>
+      </c>
+      <c r="W12" s="1">
+        <v>1</v>
+      </c>
+      <c r="X12" s="10">
+        <f t="shared" si="0"/>
+        <v>66</v>
+      </c>
+    </row>
+    <row r="13" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A13" s="11">
         <v>11</v>
       </c>
@@ -6336,12 +6958,21 @@
       <c r="T13" s="1">
         <v>5</v>
       </c>
-      <c r="U13" s="10">
-        <f t="shared" si="0"/>
-        <v>67</v>
-      </c>
-    </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U13" s="1">
+        <v>5</v>
+      </c>
+      <c r="V13" s="1">
+        <v>4</v>
+      </c>
+      <c r="W13" s="1">
+        <v>4</v>
+      </c>
+      <c r="X13" s="10">
+        <f t="shared" si="0"/>
+        <v>80</v>
+      </c>
+    </row>
+    <row r="14" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A14" s="11">
         <v>12</v>
       </c>
@@ -6402,12 +7033,22 @@
       <c r="T14" s="1">
         <v>2</v>
       </c>
-      <c r="U14" s="10">
-        <f t="shared" si="0"/>
-        <v>37</v>
-      </c>
-    </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U14" s="1">
+        <v>5</v>
+      </c>
+      <c r="V14" s="1">
+        <v>5</v>
+      </c>
+      <c r="W14" s="1">
+        <v>0</v>
+      </c>
+      <c r="X14" s="10">
+        <f t="shared" si="0"/>
+        <v>47</v>
+      </c>
+      <c r="AA14" s="33"/>
+    </row>
+    <row r="15" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A15" s="11">
         <v>13</v>
       </c>
@@ -6468,12 +7109,21 @@
       <c r="T15" s="1">
         <v>3</v>
       </c>
-      <c r="U15" s="10">
-        <f t="shared" si="0"/>
-        <v>28</v>
-      </c>
-    </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U15" s="1">
+        <v>5</v>
+      </c>
+      <c r="V15" s="1">
+        <v>5</v>
+      </c>
+      <c r="W15" s="1">
+        <v>4</v>
+      </c>
+      <c r="X15" s="10">
+        <f t="shared" si="0"/>
+        <v>42</v>
+      </c>
+    </row>
+    <row r="16" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A16" s="11">
         <v>14</v>
       </c>
@@ -6534,12 +7184,21 @@
       <c r="T16" s="1">
         <v>0</v>
       </c>
-      <c r="U16" s="10">
-        <f t="shared" si="0"/>
-        <v>37</v>
-      </c>
-    </row>
-    <row r="17" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U16" s="1">
+        <v>5</v>
+      </c>
+      <c r="V16" s="1">
+        <v>5</v>
+      </c>
+      <c r="W16" s="1">
+        <v>5</v>
+      </c>
+      <c r="X16" s="10">
+        <f t="shared" si="0"/>
+        <v>52</v>
+      </c>
+    </row>
+    <row r="17" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A17" s="11">
         <v>15</v>
       </c>
@@ -6600,12 +7259,21 @@
       <c r="T17" s="1">
         <v>1</v>
       </c>
-      <c r="U17" s="10">
-        <f t="shared" si="0"/>
-        <v>44</v>
-      </c>
-    </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U17" s="1">
+        <v>3</v>
+      </c>
+      <c r="V17" s="1">
+        <v>5</v>
+      </c>
+      <c r="W17" s="1">
+        <v>4</v>
+      </c>
+      <c r="X17" s="10">
+        <f t="shared" si="0"/>
+        <v>56</v>
+      </c>
+    </row>
+    <row r="18" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A18" s="11">
         <v>16</v>
       </c>
@@ -6666,12 +7334,22 @@
       <c r="T18" s="1">
         <v>2</v>
       </c>
-      <c r="U18" s="10">
-        <f t="shared" si="0"/>
-        <v>51</v>
-      </c>
-    </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U18" s="1">
+        <v>3</v>
+      </c>
+      <c r="V18" s="1">
+        <v>5</v>
+      </c>
+      <c r="W18" s="1">
+        <v>5</v>
+      </c>
+      <c r="X18" s="10">
+        <f t="shared" si="0"/>
+        <v>64</v>
+      </c>
+      <c r="AA18" s="33"/>
+    </row>
+    <row r="19" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A19" s="11">
         <v>17</v>
       </c>
@@ -6732,12 +7410,21 @@
       <c r="T19" s="1">
         <v>4</v>
       </c>
-      <c r="U19" s="10">
-        <f t="shared" si="0"/>
-        <v>27</v>
-      </c>
-    </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U19" s="1">
+        <v>2</v>
+      </c>
+      <c r="V19" s="1">
+        <v>5</v>
+      </c>
+      <c r="W19" s="1">
+        <v>0</v>
+      </c>
+      <c r="X19" s="10">
+        <f t="shared" si="0"/>
+        <v>34</v>
+      </c>
+    </row>
+    <row r="20" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A20" s="11">
         <v>18</v>
       </c>
@@ -6798,12 +7485,21 @@
       <c r="T20" s="1">
         <v>4</v>
       </c>
-      <c r="U20" s="10">
-        <f t="shared" si="0"/>
-        <v>53</v>
-      </c>
-    </row>
-    <row r="21" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U20" s="1">
+        <v>4</v>
+      </c>
+      <c r="V20" s="1">
+        <v>5</v>
+      </c>
+      <c r="W20" s="1">
+        <v>5</v>
+      </c>
+      <c r="X20" s="10">
+        <f t="shared" si="0"/>
+        <v>67</v>
+      </c>
+    </row>
+    <row r="21" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A21" s="11">
         <v>19</v>
       </c>
@@ -6864,12 +7560,21 @@
       <c r="T21" s="1">
         <v>4</v>
       </c>
-      <c r="U21" s="10">
-        <f t="shared" si="0"/>
-        <v>48</v>
-      </c>
-    </row>
-    <row r="22" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U21" s="1">
+        <v>0</v>
+      </c>
+      <c r="V21" s="1">
+        <v>0</v>
+      </c>
+      <c r="W21" s="1">
+        <v>5</v>
+      </c>
+      <c r="X21" s="10">
+        <f t="shared" si="0"/>
+        <v>53</v>
+      </c>
+    </row>
+    <row r="22" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A22" s="11">
         <v>20</v>
       </c>
@@ -6930,12 +7635,21 @@
       <c r="T22" s="1">
         <v>4</v>
       </c>
-      <c r="U22" s="10">
-        <f t="shared" si="0"/>
-        <v>59</v>
-      </c>
-    </row>
-    <row r="23" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U22" s="1">
+        <v>4</v>
+      </c>
+      <c r="V22" s="1">
+        <v>0</v>
+      </c>
+      <c r="W22" s="1">
+        <v>4</v>
+      </c>
+      <c r="X22" s="10">
+        <f t="shared" si="0"/>
+        <v>67</v>
+      </c>
+    </row>
+    <row r="23" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A23" s="11">
         <v>21</v>
       </c>
@@ -6996,12 +7710,21 @@
       <c r="T23" s="1">
         <v>0</v>
       </c>
-      <c r="U23" s="10">
-        <f t="shared" si="0"/>
-        <v>32</v>
-      </c>
-    </row>
-    <row r="24" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U23" s="1">
+        <v>5</v>
+      </c>
+      <c r="V23" s="1">
+        <v>5</v>
+      </c>
+      <c r="W23" s="1">
+        <v>4</v>
+      </c>
+      <c r="X23" s="10">
+        <f t="shared" si="0"/>
+        <v>46</v>
+      </c>
+    </row>
+    <row r="24" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A24" s="11">
         <v>22</v>
       </c>
@@ -7062,12 +7785,21 @@
       <c r="T24" s="1">
         <v>0</v>
       </c>
-      <c r="U24" s="10">
-        <f t="shared" si="0"/>
-        <v>41</v>
-      </c>
-    </row>
-    <row r="25" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U24" s="1">
+        <v>0</v>
+      </c>
+      <c r="V24" s="1">
+        <v>0</v>
+      </c>
+      <c r="W24" s="1">
+        <v>5</v>
+      </c>
+      <c r="X24" s="10">
+        <f t="shared" si="0"/>
+        <v>46</v>
+      </c>
+    </row>
+    <row r="25" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A25" s="11">
         <v>23</v>
       </c>
@@ -7128,12 +7860,21 @@
       <c r="T25" s="1">
         <v>0</v>
       </c>
-      <c r="U25" s="10">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U25" s="1">
+        <v>0</v>
+      </c>
+      <c r="V25" s="1">
+        <v>0</v>
+      </c>
+      <c r="W25" s="1">
+        <v>0</v>
+      </c>
+      <c r="X25" s="10">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A26" s="11">
         <v>24</v>
       </c>
@@ -7194,12 +7935,21 @@
       <c r="T26" s="1">
         <v>4</v>
       </c>
-      <c r="U26" s="10">
-        <f t="shared" si="0"/>
-        <v>48</v>
-      </c>
-    </row>
-    <row r="27" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U26" s="1">
+        <v>0</v>
+      </c>
+      <c r="V26" s="1">
+        <v>5</v>
+      </c>
+      <c r="W26" s="1">
+        <v>0</v>
+      </c>
+      <c r="X26" s="10">
+        <f t="shared" si="0"/>
+        <v>53</v>
+      </c>
+    </row>
+    <row r="27" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A27" s="11">
         <v>25</v>
       </c>
@@ -7260,12 +8010,21 @@
       <c r="T27" s="1">
         <v>0</v>
       </c>
-      <c r="U27" s="10">
-        <f t="shared" si="0"/>
-        <v>47</v>
-      </c>
-    </row>
-    <row r="28" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U27" s="1">
+        <v>0</v>
+      </c>
+      <c r="V27" s="1">
+        <v>0</v>
+      </c>
+      <c r="W27" s="1">
+        <v>3</v>
+      </c>
+      <c r="X27" s="10">
+        <f t="shared" si="0"/>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="28" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A28" s="11">
         <v>26</v>
       </c>
@@ -7326,12 +8085,21 @@
       <c r="T28" s="1">
         <v>5</v>
       </c>
-      <c r="U28" s="10">
-        <f t="shared" si="0"/>
-        <v>62</v>
-      </c>
-    </row>
-    <row r="29" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U28" s="1">
+        <v>0</v>
+      </c>
+      <c r="V28" s="1">
+        <v>5</v>
+      </c>
+      <c r="W28" s="1">
+        <v>5</v>
+      </c>
+      <c r="X28" s="10">
+        <f t="shared" si="0"/>
+        <v>72</v>
+      </c>
+    </row>
+    <row r="29" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A29" s="11">
         <v>27</v>
       </c>
@@ -7392,12 +8160,21 @@
       <c r="T29" s="1">
         <v>0</v>
       </c>
-      <c r="U29" s="10">
-        <f t="shared" si="0"/>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="30" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U29" s="1">
+        <v>0</v>
+      </c>
+      <c r="V29" s="1">
+        <v>0</v>
+      </c>
+      <c r="W29" s="1">
+        <v>5</v>
+      </c>
+      <c r="X29" s="10">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="30" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A30" s="11">
         <v>28</v>
       </c>
@@ -7458,12 +8235,21 @@
       <c r="T30" s="1">
         <v>3</v>
       </c>
-      <c r="U30" s="10">
-        <f t="shared" si="0"/>
-        <v>41</v>
-      </c>
-    </row>
-    <row r="31" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U30" s="1">
+        <v>2</v>
+      </c>
+      <c r="V30" s="1">
+        <v>4</v>
+      </c>
+      <c r="W30" s="1">
+        <v>0</v>
+      </c>
+      <c r="X30" s="10">
+        <f t="shared" si="0"/>
+        <v>47</v>
+      </c>
+    </row>
+    <row r="31" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A31" s="11">
         <v>29</v>
       </c>
@@ -7524,12 +8310,21 @@
       <c r="T31" s="1">
         <v>3</v>
       </c>
-      <c r="U31" s="10">
-        <f t="shared" si="0"/>
-        <v>48</v>
-      </c>
-    </row>
-    <row r="32" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U31" s="1">
+        <v>3</v>
+      </c>
+      <c r="V31" s="1">
+        <v>5</v>
+      </c>
+      <c r="W31" s="1">
+        <v>5</v>
+      </c>
+      <c r="X31" s="10">
+        <f t="shared" si="0"/>
+        <v>61</v>
+      </c>
+    </row>
+    <row r="32" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A32" s="11">
         <v>30</v>
       </c>
@@ -7590,12 +8385,21 @@
       <c r="T32" s="1">
         <v>4</v>
       </c>
-      <c r="U32" s="10">
-        <f t="shared" si="0"/>
-        <v>52</v>
-      </c>
-    </row>
-    <row r="33" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U32" s="1">
+        <v>3</v>
+      </c>
+      <c r="V32" s="1">
+        <v>5</v>
+      </c>
+      <c r="W32" s="1">
+        <v>0</v>
+      </c>
+      <c r="X32" s="10">
+        <f t="shared" si="0"/>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="33" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A33" s="11">
         <v>31</v>
       </c>
@@ -7656,12 +8460,21 @@
       <c r="T33" s="1">
         <v>0</v>
       </c>
-      <c r="U33" s="10">
-        <f t="shared" si="0"/>
-        <v>7</v>
-      </c>
-    </row>
-    <row r="34" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U33" s="1">
+        <v>0</v>
+      </c>
+      <c r="V33" s="1">
+        <v>5</v>
+      </c>
+      <c r="W33" s="1">
+        <v>0</v>
+      </c>
+      <c r="X33" s="10">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="34" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A34" s="11">
         <v>32</v>
       </c>
@@ -7722,12 +8535,21 @@
       <c r="T34" s="1">
         <v>0</v>
       </c>
-      <c r="U34" s="10">
-        <f t="shared" si="0"/>
-        <v>14</v>
-      </c>
-    </row>
-    <row r="35" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U34" s="1">
+        <v>0</v>
+      </c>
+      <c r="V34" s="1">
+        <v>5</v>
+      </c>
+      <c r="W34" s="1">
+        <v>5</v>
+      </c>
+      <c r="X34" s="10">
+        <f t="shared" si="0"/>
+        <v>24</v>
+      </c>
+    </row>
+    <row r="35" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A35" s="11">
         <v>33</v>
       </c>
@@ -7788,12 +8610,21 @@
       <c r="T35" s="1">
         <v>5</v>
       </c>
-      <c r="U35" s="10">
-        <f t="shared" si="0"/>
-        <v>56</v>
-      </c>
-    </row>
-    <row r="36" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U35" s="1">
+        <v>4</v>
+      </c>
+      <c r="V35" s="1">
+        <v>5</v>
+      </c>
+      <c r="W35" s="1">
+        <v>5</v>
+      </c>
+      <c r="X35" s="10">
+        <f t="shared" si="0"/>
+        <v>70</v>
+      </c>
+    </row>
+    <row r="36" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A36" s="11">
         <v>34</v>
       </c>
@@ -7854,12 +8685,21 @@
       <c r="T36" s="1">
         <v>4</v>
       </c>
-      <c r="U36" s="10">
-        <f t="shared" si="0"/>
-        <v>43</v>
-      </c>
-    </row>
-    <row r="37" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U36" s="1">
+        <v>5</v>
+      </c>
+      <c r="V36" s="1">
+        <v>0</v>
+      </c>
+      <c r="W36" s="1">
+        <v>5</v>
+      </c>
+      <c r="X36" s="10">
+        <f t="shared" si="0"/>
+        <v>53</v>
+      </c>
+    </row>
+    <row r="37" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A37" s="11">
         <v>35</v>
       </c>
@@ -7920,12 +8760,21 @@
       <c r="T37" s="1">
         <v>4</v>
       </c>
-      <c r="U37" s="10">
-        <f t="shared" si="0"/>
-        <v>57</v>
-      </c>
-    </row>
-    <row r="38" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U37" s="1">
+        <v>3</v>
+      </c>
+      <c r="V37" s="1">
+        <v>5</v>
+      </c>
+      <c r="W37" s="1">
+        <v>0</v>
+      </c>
+      <c r="X37" s="10">
+        <f t="shared" si="0"/>
+        <v>65</v>
+      </c>
+    </row>
+    <row r="38" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A38" s="11">
         <v>36</v>
       </c>
@@ -7986,12 +8835,21 @@
       <c r="T38" s="1">
         <v>2</v>
       </c>
-      <c r="U38" s="10">
-        <f t="shared" si="0"/>
-        <v>54</v>
-      </c>
-    </row>
-    <row r="39" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U38" s="1">
+        <v>1</v>
+      </c>
+      <c r="V38" s="1">
+        <v>0</v>
+      </c>
+      <c r="W38" s="1">
+        <v>4</v>
+      </c>
+      <c r="X38" s="10">
+        <f t="shared" si="0"/>
+        <v>59</v>
+      </c>
+    </row>
+    <row r="39" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A39" s="11">
         <v>37</v>
       </c>
@@ -8052,12 +8910,21 @@
       <c r="T39" s="1">
         <v>0</v>
       </c>
-      <c r="U39" s="10">
-        <f t="shared" si="0"/>
-        <v>38</v>
-      </c>
-    </row>
-    <row r="40" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U39" s="1">
+        <v>0</v>
+      </c>
+      <c r="V39" s="1">
+        <v>4</v>
+      </c>
+      <c r="W39" s="1">
+        <v>4</v>
+      </c>
+      <c r="X39" s="10">
+        <f t="shared" si="0"/>
+        <v>46</v>
+      </c>
+    </row>
+    <row r="40" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A40" s="11">
         <v>38</v>
       </c>
@@ -8118,12 +8985,21 @@
       <c r="T40" s="1">
         <v>5</v>
       </c>
-      <c r="U40" s="10">
-        <f t="shared" si="0"/>
-        <v>30</v>
-      </c>
-    </row>
-    <row r="41" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U40" s="1">
+        <v>4</v>
+      </c>
+      <c r="V40" s="1">
+        <v>4</v>
+      </c>
+      <c r="W40" s="1">
+        <v>5</v>
+      </c>
+      <c r="X40" s="10">
+        <f t="shared" si="0"/>
+        <v>43</v>
+      </c>
+    </row>
+    <row r="41" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A41" s="11">
         <v>39</v>
       </c>
@@ -8184,12 +9060,21 @@
       <c r="T41" s="1">
         <v>0</v>
       </c>
-      <c r="U41" s="10">
-        <f t="shared" si="0"/>
-        <v>11</v>
-      </c>
-    </row>
-    <row r="42" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U41" s="1">
+        <v>0</v>
+      </c>
+      <c r="V41" s="1">
+        <v>4</v>
+      </c>
+      <c r="W41" s="1">
+        <v>0</v>
+      </c>
+      <c r="X41" s="10">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="42" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A42" s="11">
         <v>40</v>
       </c>
@@ -8250,12 +9135,21 @@
       <c r="T42" s="1">
         <v>3</v>
       </c>
-      <c r="U42" s="10">
-        <f t="shared" si="0"/>
-        <v>51</v>
-      </c>
-    </row>
-    <row r="43" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U42" s="1">
+        <v>4</v>
+      </c>
+      <c r="V42" s="1">
+        <v>5</v>
+      </c>
+      <c r="W42" s="1">
+        <v>5</v>
+      </c>
+      <c r="X42" s="10">
+        <f t="shared" si="0"/>
+        <v>65</v>
+      </c>
+    </row>
+    <row r="43" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A43" s="11">
         <v>41</v>
       </c>
@@ -8316,12 +9210,21 @@
       <c r="T43" s="1">
         <v>4</v>
       </c>
-      <c r="U43" s="10">
-        <f t="shared" si="0"/>
-        <v>61</v>
-      </c>
-    </row>
-    <row r="44" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U43" s="1">
+        <v>5</v>
+      </c>
+      <c r="V43" s="1">
+        <v>0</v>
+      </c>
+      <c r="W43" s="1">
+        <v>5</v>
+      </c>
+      <c r="X43" s="10">
+        <f t="shared" si="0"/>
+        <v>71</v>
+      </c>
+    </row>
+    <row r="44" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A44" s="11">
         <v>42</v>
       </c>
@@ -8382,12 +9285,21 @@
       <c r="T44" s="1">
         <v>0</v>
       </c>
-      <c r="U44" s="10">
-        <f t="shared" si="0"/>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="45" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U44" s="1">
+        <v>5</v>
+      </c>
+      <c r="V44" s="1">
+        <v>5</v>
+      </c>
+      <c r="W44" s="1">
+        <v>0</v>
+      </c>
+      <c r="X44" s="10">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="45" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A45" s="11">
         <v>43</v>
       </c>
@@ -8448,12 +9360,21 @@
       <c r="T45" s="1">
         <v>5</v>
       </c>
-      <c r="U45" s="10">
-        <f t="shared" si="0"/>
-        <v>49</v>
-      </c>
-    </row>
-    <row r="46" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U45" s="1">
+        <v>5</v>
+      </c>
+      <c r="V45" s="1">
+        <v>5</v>
+      </c>
+      <c r="W45" s="1">
+        <v>5</v>
+      </c>
+      <c r="X45" s="10">
+        <f t="shared" si="0"/>
+        <v>64</v>
+      </c>
+    </row>
+    <row r="46" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A46" s="11">
         <v>44</v>
       </c>
@@ -8514,12 +9435,21 @@
       <c r="T46" s="1">
         <v>4</v>
       </c>
-      <c r="U46" s="10">
-        <f t="shared" si="0"/>
-        <v>54</v>
-      </c>
-    </row>
-    <row r="47" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U46" s="1">
+        <v>5</v>
+      </c>
+      <c r="V46" s="1">
+        <v>5</v>
+      </c>
+      <c r="W46" s="1">
+        <v>4</v>
+      </c>
+      <c r="X46" s="10">
+        <f t="shared" si="0"/>
+        <v>68</v>
+      </c>
+    </row>
+    <row r="47" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A47" s="11">
         <v>45</v>
       </c>
@@ -8580,12 +9510,21 @@
       <c r="T47" s="1">
         <v>5</v>
       </c>
-      <c r="U47" s="10">
-        <f t="shared" si="0"/>
-        <v>57</v>
-      </c>
-    </row>
-    <row r="48" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U47" s="1">
+        <v>4</v>
+      </c>
+      <c r="V47" s="1">
+        <v>5</v>
+      </c>
+      <c r="W47" s="1">
+        <v>0</v>
+      </c>
+      <c r="X47" s="10">
+        <f t="shared" si="0"/>
+        <v>66</v>
+      </c>
+    </row>
+    <row r="48" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A48" s="11">
         <v>46</v>
       </c>
@@ -8646,12 +9585,21 @@
       <c r="T48" s="1">
         <v>5</v>
       </c>
-      <c r="U48" s="10">
-        <f t="shared" si="0"/>
-        <v>52</v>
-      </c>
-    </row>
-    <row r="49" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U48" s="1">
+        <v>5</v>
+      </c>
+      <c r="V48" s="1">
+        <v>5</v>
+      </c>
+      <c r="W48" s="1">
+        <v>5</v>
+      </c>
+      <c r="X48" s="10">
+        <f t="shared" si="0"/>
+        <v>67</v>
+      </c>
+    </row>
+    <row r="49" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A49" s="11">
         <v>47</v>
       </c>
@@ -8712,12 +9660,21 @@
       <c r="T49" s="1">
         <v>2</v>
       </c>
-      <c r="U49" s="10">
-        <f t="shared" si="0"/>
-        <v>18</v>
-      </c>
-    </row>
-    <row r="50" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U49" s="1">
+        <v>5</v>
+      </c>
+      <c r="V49" s="1">
+        <v>5</v>
+      </c>
+      <c r="W49" s="1">
+        <v>5</v>
+      </c>
+      <c r="X49" s="10">
+        <f t="shared" si="0"/>
+        <v>33</v>
+      </c>
+    </row>
+    <row r="50" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A50" s="11">
         <v>48</v>
       </c>
@@ -8778,12 +9735,21 @@
       <c r="T50" s="1">
         <v>4</v>
       </c>
-      <c r="U50" s="10">
-        <f t="shared" si="0"/>
-        <v>52</v>
-      </c>
-    </row>
-    <row r="51" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="U50" s="1">
+        <v>3</v>
+      </c>
+      <c r="V50" s="1">
+        <v>0</v>
+      </c>
+      <c r="W50" s="1">
+        <v>0</v>
+      </c>
+      <c r="X50" s="10">
+        <f t="shared" si="0"/>
+        <v>55</v>
+      </c>
+    </row>
+    <row r="51" spans="1:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A51" s="27">
         <v>49</v>
       </c>
@@ -8844,12 +9810,21 @@
       <c r="T51" s="23">
         <v>4</v>
       </c>
-      <c r="U51" s="10">
-        <f t="shared" si="0"/>
-        <v>58</v>
-      </c>
-    </row>
-    <row r="64" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U51" s="23">
+        <v>4</v>
+      </c>
+      <c r="V51" s="23">
+        <v>5</v>
+      </c>
+      <c r="W51" s="23">
+        <v>5</v>
+      </c>
+      <c r="X51" s="10">
+        <f t="shared" si="0"/>
+        <v>72</v>
+      </c>
+    </row>
+    <row r="64" spans="1:24" x14ac:dyDescent="0.3">
       <c r="R64" s="33"/>
     </row>
   </sheetData>

</xml_diff>